<commit_message>
Address workbook architecture review findings
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -2488,19 +2488,18 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22" customHeight="1">
+    <row r="1" spans="1:6" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>EquipmentID</t>
@@ -2523,22 +2522,17 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Configuration</t>
+          <t>SourceID</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>SourceID</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
           <t>Confidence</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3156,7 +3150,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3168,10 +3162,9 @@
     <col min="7" max="7" width="72" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
     <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="22" customHeight="1">
+    <row r="1" spans="1:9" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ReviewID</t>
@@ -3209,22 +3202,17 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>SourceID</t>
+          <t>EvidenceID</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>EvidenceID</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
           <t>FrameworkVersion</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Implement workbook enumeration contract
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -20,6 +20,20 @@
     <sheet name="10_Scoring" sheetId="11" r:id="rId11"/>
     <sheet name="11_DecisionLog" sheetId="12" r:id="rId12"/>
   </sheets>
+  <definedNames>
+    <definedName name="Enum_Availability">'README'!$X$2:$X$6</definedName>
+    <definedName name="Enum_Confidence">'README'!$Y$2:$Y$5</definedName>
+    <definedName name="Enum_VehicleStatus">'README'!$Z$2:$Z$7</definedName>
+    <definedName name="Enum_ConfigurationStatus">'README'!$AA$2:$AA$5</definedName>
+    <definedName name="Enum_RequirementType">'README'!$AB$2:$AB$5</definedName>
+    <definedName name="Enum_SourceType">'README'!$AC$2:$AC$10</definedName>
+    <definedName name="Enum_EvidenceType">'README'!$AD$2:$AD$7</definedName>
+    <definedName name="Enum_Market">'README'!$AE$2:$AE$8</definedName>
+    <definedName name="Enum_Unit">'README'!$AF$2:$AF$13</definedName>
+    <definedName name="Enum_FrameworkStatus">'README'!$AG$2:$AG$5</definedName>
+    <definedName name="Enum_DecisionStatus">'README'!$AH$2:$AH$5</definedName>
+    <definedName name="Validation_Boolean">'README'!$AI$2:$AI$3</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -171,12 +185,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:AI13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="90" customWidth="1"/>
+    <col min="24" max="24" width="12" customWidth="1" hidden="1"/>
+    <col min="25" max="25" width="12" customWidth="1" hidden="1"/>
+    <col min="26" max="26" width="12" customWidth="1" hidden="1"/>
+    <col min="27" max="27" width="12" customWidth="1" hidden="1"/>
+    <col min="28" max="28" width="12" customWidth="1" hidden="1"/>
+    <col min="29" max="29" width="12" customWidth="1" hidden="1"/>
+    <col min="30" max="30" width="12" customWidth="1" hidden="1"/>
+    <col min="31" max="31" width="12" customWidth="1" hidden="1"/>
+    <col min="32" max="32" width="12" customWidth="1" hidden="1"/>
+    <col min="33" max="33" width="12" customWidth="1" hidden="1"/>
+    <col min="34" max="34" width="12" customWidth="1" hidden="1"/>
+    <col min="35" max="35" width="12" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="22" customHeight="1">
@@ -190,6 +216,66 @@
           <t>Value</t>
         </is>
       </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Enum_Availability</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Enum_Confidence</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Enum_VehicleStatus</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Enum_ConfigurationStatus</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Enum_RequirementType</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Enum_SourceType</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Enum_EvidenceType</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Enum_Market</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Enum_Unit</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Enum_FrameworkStatus</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Enum_DecisionStatus</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Validation_Boolean</t>
+        </is>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="inlineStr">
@@ -202,6 +288,66 @@
           <t>1.0</t>
         </is>
       </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>ANNOUNCED</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>SPECIFICATION</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="inlineStr">
@@ -214,6 +360,66 @@
           <t>1.0</t>
         </is>
       </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>PREORDER</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>UPCOMING</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>WEIGHTED</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>GOVERNMENT</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>MEASUREMENT</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="inlineStr">
@@ -226,6 +432,61 @@
           <t>2026-07-06</t>
         </is>
       </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>PACKAGE</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>DISCONTINUED</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>INFORMATIONAL</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>CERTIFICATION</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>LOCKED</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="inlineStr">
@@ -238,6 +499,61 @@
           <t>Battery electric vehicle decision framework</t>
         </is>
       </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>DISCONTINUED</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>TEST_RESULT</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>FI</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>DEPRECATED</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>SUPERSEDED</t>
+        </is>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="inlineStr">
@@ -250,6 +566,36 @@
           <t>Reference implementation of the documented EV Decision Framework schema.</t>
         </is>
       </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>CANCELLED</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>OWNER_REPORT</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>REVIEW_SUMMARY</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>KMH</t>
+        </is>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="inlineStr">
@@ -262,15 +608,117 @@
           <t>Structure synchronized to Framework Version 1.0. Production data is not introduced by this workbook sync.</t>
         </is>
       </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>COMMUNITY</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>OWNER_EXPERIENCE</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>KWH</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LOCKED</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>DATABASE</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>KWH_100KM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>VIDEO</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B8"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B8:B8">
+      <formula1>Enum_FrameworkStatus</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -328,12 +776,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B1048576">
+      <formula1>Enum_SourceType</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -396,7 +849,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -515,7 +968,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:J30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -606,7 +1059,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>HARD</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -616,12 +1069,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I2"/>
@@ -654,7 +1107,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>HARD</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -664,12 +1117,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I3"/>
@@ -702,7 +1155,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>HARD</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -712,12 +1165,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I4"/>
@@ -750,7 +1203,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>HARD</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -760,12 +1213,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I5"/>
@@ -798,7 +1251,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>HARD</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -808,12 +1261,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I6"/>
@@ -846,7 +1299,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -856,12 +1309,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I7"/>
@@ -894,7 +1347,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -904,12 +1357,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I8"/>
@@ -942,7 +1395,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -952,12 +1405,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I9"/>
@@ -990,7 +1443,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1000,12 +1453,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I10"/>
@@ -1038,7 +1491,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1048,12 +1501,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I11"/>
@@ -1086,7 +1539,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1096,12 +1549,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I12"/>
@@ -1134,7 +1587,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1144,12 +1597,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I13"/>
@@ -1182,7 +1635,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1192,12 +1645,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I14"/>
@@ -1230,7 +1683,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1240,12 +1693,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I15"/>
@@ -1278,7 +1731,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1288,12 +1741,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I16"/>
@@ -1326,7 +1779,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1336,12 +1789,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I17"/>
@@ -1374,7 +1827,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1384,12 +1837,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I18"/>
@@ -1422,7 +1875,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1432,12 +1885,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I19"/>
@@ -1470,7 +1923,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1480,12 +1933,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I20"/>
@@ -1518,7 +1971,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1528,12 +1981,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I21"/>
@@ -1566,7 +2019,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1576,12 +2029,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I22"/>
@@ -1614,7 +2067,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1624,12 +2077,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I23"/>
@@ -1662,7 +2115,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1672,12 +2125,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I24"/>
@@ -1710,7 +2163,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1720,12 +2173,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I25"/>
@@ -1758,7 +2211,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Weighted</t>
+          <t>WEIGHTED</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1768,12 +2221,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I26"/>
@@ -1806,7 +2259,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>INFORMATIONAL</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1816,12 +2269,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I27"/>
@@ -1854,7 +2307,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>INFORMATIONAL</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1864,12 +2317,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I28"/>
@@ -1902,7 +2355,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>INFORMATIONAL</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1912,12 +2365,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I29"/>
@@ -1950,7 +2403,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>INFORMATIONAL</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1960,12 +2413,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I30"/>
@@ -1977,12 +2430,23 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J30"/>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E1048576">
+      <formula1>Enum_RequirementType</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G2:G1048576">
+      <formula1>Validation_Boolean</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H1048576">
+      <formula1>Validation_Boolean</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2060,7 +2524,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Watchlist</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2097,7 +2561,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Watchlist</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2134,7 +2598,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Watchlist</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2171,7 +2635,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Watchlist</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2182,12 +2646,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G5"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F1048576">
+      <formula1>Enum_VehicleStatus</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2239,12 +2708,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C1048576">
+      <formula1>Enum_Market</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2324,13 +2798,13 @@
       <c r="E2"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="G2"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="I2"/>
@@ -2352,13 +2826,13 @@
       <c r="E3"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>km</t>
+          <t>KM</t>
         </is>
       </c>
       <c r="G3"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="I3"/>
@@ -2380,13 +2854,13 @@
       <c r="E4"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>km</t>
+          <t>KM</t>
         </is>
       </c>
       <c r="G4"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="I4"/>
@@ -2408,13 +2882,13 @@
       <c r="E5"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>kWh</t>
+          <t>KWH</t>
         </is>
       </c>
       <c r="G5"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="I5"/>
@@ -2436,13 +2910,13 @@
       <c r="E6"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>KW</t>
         </is>
       </c>
       <c r="G6"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="I6"/>
@@ -2470,7 +2944,7 @@
       <c r="G7"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="I7"/>
@@ -2482,12 +2956,20 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J7"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F1048576">
+      <formula1>Enum_Unit</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H1048576">
+      <formula1>Enum_Confidence</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2533,12 +3015,20 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D1048576">
+      <formula1>Enum_Availability</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F1048576">
+      <formula1>Enum_Confidence</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2601,7 +3091,7 @@
       <c r="D2"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2629,7 +3119,7 @@
       <c r="D3"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2657,7 +3147,7 @@
       <c r="D4"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -2685,7 +3175,7 @@
       <c r="D5"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2713,7 +3203,7 @@
       <c r="D6"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2741,7 +3231,7 @@
       <c r="D7"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2769,7 +3259,7 @@
       <c r="D8"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2797,7 +3287,7 @@
       <c r="D9"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2825,7 +3315,7 @@
       <c r="D10"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2853,7 +3343,7 @@
       <c r="D11"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2881,7 +3371,7 @@
       <c r="D12"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2909,7 +3399,7 @@
       <c r="D13"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2937,7 +3427,7 @@
       <c r="D14"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2965,7 +3455,7 @@
       <c r="D15"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2993,7 +3483,7 @@
       <c r="D16"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -3021,7 +3511,7 @@
       <c r="D17"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3049,7 +3539,7 @@
       <c r="D18"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3077,7 +3567,7 @@
       <c r="D19"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3105,7 +3595,7 @@
       <c r="D20"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3133,7 +3623,7 @@
       <c r="D21"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -3144,12 +3634,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:F21"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E1048576">
+      <formula1>Validation_Boolean</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3213,12 +3708,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F1048576">
+      <formula1>Enum_Confidence</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3276,6 +3776,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H1048576">
+      <formula1>Enum_Confidence</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Populate Kia EV2 reference vehicle dataset
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -2447,7 +2447,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -2460,37 +2460,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t>VehicleID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t>Manufacturer</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t>ModelYear</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t>Notes</t>
         </is>
@@ -2514,12 +2514,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unknown/EV platform</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2529,118 +2529,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Norske spesifikasjoner kan mates inn manuelt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>RENAULT_4</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Renault</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>4 E-Tech</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>AmpR Small</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Relevant konkurrent til EV2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CITROEN_EC3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Citroën</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ë-C3</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Smart Car</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Lavere pris; må vurderes kritisk på komfort/tech.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SKODA_ELROQ</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Škoda</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Elroq</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>MEB</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Nær maks lengde; praktisk utfordrer.</t>
+          <t>Kia Norway official model list reviewed 2026-07-06; EV2 not listed, so Norwegian lifecycle/configuration data remains unverified.</t>
         </is>
       </c>
     </row>
@@ -2670,37 +2559,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t>ConfigurationID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t>VehicleID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t>Trim</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t>BasePrice</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t>ConfiguredPrice</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t>Notes</t>
         </is>

</xml_diff>

<commit_message>
Populate Tesla Model 3 reference dataset
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -2447,7 +2447,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -2460,37 +2460,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t>VehicleID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t>Manufacturer</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t>ModelYear</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t>Notes</t>
         </is>
@@ -2499,148 +2499,37 @@
     <row r="2" spans="1:7">
       <c r="A2" t="inlineStr">
         <is>
-          <t>KIA_EV2</t>
+          <t>TESLA_MODEL_3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Kia</t>
+          <t>Tesla</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>EV2</t>
+          <t>Model 3</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unknown/EV platform</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>AVAILABLE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Norske spesifikasjoner kan mates inn manuelt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>RENAULT_4</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Renault</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>4 E-Tech</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>AmpR Small</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Relevant konkurrent til EV2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CITROEN_EC3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Citroën</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ë-C3</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Smart Car</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Lavere pris; må vurderes kritisk på komfort/tech.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SKODA_ELROQ</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Škoda</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Elroq</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>MEB</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Nær maks lengde; praktisk utfordrer.</t>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; model year and platform not specified in workbook-supported source fields.</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2546,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -2670,39 +2559,187 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t>ConfigurationID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t>VehicleID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t>Trim</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t>BasePrice</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t>ConfiguredPrice</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Bakhjulsdrift</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Long Range firehjulsdrift</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Long Range bakhjulsdrift</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update framework documentation to version 1.2, enhancing the entity model, implementation contract, relationships model, and workbook schema with new Configuration Status details and clarifications on lifecycle management.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -369,7 +369,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -441,7 +441,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Structure synchronized to Framework Version 1.0. Production data is not introduced by this workbook sync.</t>
+          <t>Configuration Status implemented per ADR-004 (IMPL-002). Structure synchronized to Framework Version 1.2.</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -859,6 +859,164 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Model 3 – Sportslig elektrisk sedan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://www.tesla.com/no_no/model3</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Official Tesla Norway configurator/specification page. Technical values retrieved by switching between the Model 3 (RWD), Premium (Long Range AWD / Long Range RWD) and Performance trim tabs on the live page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SRC_MOTORNO_MODEL3_2024</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Motor har testet nye Tesla Model 3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Motor.no</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://www.motor.no/bil/motor-har-testet-nye-tesla-model-3/262378</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Test av Tesla Model 3 Long Range firehjulsdrift (AWD). Dekker kupestoy, komfort, styring og sikt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SRC_CARSCOM_MODEL3_2024</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2024 Tesla Model 3 Review: My, How You've Improved</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Cars.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://www.cars.com/articles/2024-tesla-model-3-review-my-how-youve-improved-483077/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Test av Tesla Model 3 Long Range. Dekker NVH/stoydemping, fjaering og infotainment-betjening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SRC_MACRUMORS_CARPLAY_2025</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Heres When Tesla is Expected to Add Support for Apple CarPlay</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>MacRumors</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://www.macrumors.com/2025/11/16/tesla-carplay-support-in-coming-months/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2025-11-16</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Rapporterer status og planer for Apple CarPlay-stotte pa Tesla-kjoretoy, inkludert Model 3.</t>
         </is>
       </c>
     </row>
@@ -879,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -934,6 +1092,272 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SCORE_000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>W001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>REV_000001</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>80</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). WeightedScore = RawScore x Weight(8)/100 = 6.4. Traceable to REV_000001 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SCORE_000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>W002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>REV_000002</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>80</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). WeightedScore = RawScore x Weight(7)/100 = 5.6. Traceable to REV_000002 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SCORE_000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>W003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>REV_000003</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). WeightedScore = RawScore x Weight(5)/100 = 3.0. Traceable to REV_000003 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SCORE_000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>W004</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>REV_000004</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>80</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). WeightedScore = RawScore x Weight(5)/100 = 4.0. Traceable to REV_000004 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SCORE_000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>W005</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>REV_000005</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>60</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). WeightedScore = RawScore x Weight(7)/100 = 4.2. Traceable to REV_000005 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SCORE_000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>W007</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>REV_000006</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>20</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Review score 1/5 (normalized RawScore = 20.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). WeightedScore = RawScore x Weight(3)/100 = 0.6. Traceable to REV_000006 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SCORE_000007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>W020</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>REV_000007</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>80</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). WeightedScore = RawScore x Weight(2)/100 = 1.6. Traceable to REV_000007 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -946,7 +1370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1051,6 +1475,43 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>Codex</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DEC_IMPL_002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Implemented Configuration Status (ADR-004 / IMPL-002)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Closed the gap between the documented Configuration Status enumeration and the workbook schema; added Status column to 03_Configurations</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Populated existing Tesla Model 3 configurations as AVAILABLE, backed by the Tesla Norway configurator source already cited in their Notes.</t>
         </is>
       </c>
     </row>
@@ -2659,16 +3120,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2689,20 +3151,25 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Trim</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>BasePrice</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ConfiguredPrice</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2726,14 +3193,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Bakhjulsdrift</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content.</t>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002).</t>
         </is>
       </c>
     </row>
@@ -2755,14 +3225,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Long Range firehjulsdrift</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content.</t>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002).</t>
         </is>
       </c>
     </row>
@@ -2784,14 +3257,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Long Range bakhjulsdrift</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content.</t>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002).</t>
         </is>
       </c>
     </row>
@@ -2813,22 +3289,28 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content.</t>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Enum_Market</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>Enum_ConfigurationStatus</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2841,7 +3323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3037,6 +3519,1491 @@
       <c r="J7" t="inlineStr">
         <is>
           <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TECH_000001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Length</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>4720</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TECH_000002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Width (mirrors unfolded)</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2089</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TECH_000003</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Boot volume</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>682</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TECH_000004</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Height</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1440</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TECH_000005</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Width (mirrors folded)</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1850</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TECH_000006</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ground clearance</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>138</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TECH_000007</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Kerb weight (MRO)</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1847</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TECH_000008</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>WLTP range</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>534</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TECH_000009</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>WLTP consumption</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>13</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>KWH_100KM</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TECH_000010</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>DC max charging</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>175</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TECH_000011</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Height</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1441</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TECH_000012</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Width (mirrors folded)</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1933</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TECH_000013</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Ground clearance</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>138</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TECH_000014</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Kerb weight (MRO)</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1899</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TECH_000015</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>WLTP range</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>660</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TECH_000016</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>WLTP consumption</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>KWH_100KM</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TECH_000017</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>DC max charging</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>250</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TECH_000018</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Height</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1441</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TECH_000019</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Width (mirrors folded)</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1933</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TECH_000020</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Ground clearance</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>138</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TECH_000021</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Kerb weight (MRO)</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1822</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TECH_000022</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>WLTP range (18" wheels)</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>750</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TECH_000023</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>WLTP range (19" wheels)</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>691</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TECH_000024</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>WLTP consumption</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>KWH_100KM</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TECH_000025</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>DC max charging</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>250</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TECH_000026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Height</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1431</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>TECH_000027</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Width (mirrors folded)</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1933</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>TECH_000028</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Ground clearance</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>128</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TECH_000029</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Kerb weight (MRO)</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1929</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>TECH_000030</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>WLTP range</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>571</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>TECH_000031</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>WLTP consumption</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>KWH_100KM</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TECH_000032</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>DC max charging</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>250</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>TECH_000033</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Top speed</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>262</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>KMH</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>1.2</t>
         </is>
       </c>
     </row>
@@ -3723,7 +5690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3781,6 +5748,286 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>FrameworkVersion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>REV_000001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>To uavhengige profesjonelle tester (Motor.no, Cars.com) bekrefter betydelig redusert kupestoy i den oppgraderte Model 3-plattformen sammenlignet med tidligere arsmodeller; dekkstoy fremheves som blant de beste i klassen. Testet pa Long Range AWD/Long Range, men deler karosseri og lydisolasjon med Long Range bakhjulsdrift. [Kriterium W001]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EV_000001,EV_000002</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>REV_000002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Motor.no gir 8/10 for komfort og beskriver fjaeringen som behagelig ved hoyere hastighet; Cars.com bekrefter at det ikke oppstar bra stot takket vaere frekvensavhengige dempere. Testet pa AWD/Long Range-varianter; RWD-spesifikk fjaeringskarakter er ikke uavhengig bekreftet. [Kriterium W002]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EV_000003,EV_000004</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REV_000003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Motor.no rapporterer suveren sikt fremover, men darlig sikt bakover - sistnevnte er en reell praktisk ulempe ved manovrering. Kun en uavhengig kilde funnet. [Kriterium W003]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EV_000006</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>REV_000004</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Motor.no beskriver direkte og relativt tung styrefolelse med umiddelbar respons, og gir 10/10 for kjoreegenskaper. Kun en uavhengig kilde funnet. [Kriterium W004]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EV_000005</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>REV_000005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Cars.com dokumenterer konkrete brukssvakheter: bereringsbaserte blinklysknapper som til tider ikke reagerte, og at telefonnokkelen av og til ikke registrerte foreren. Skjermavhengig betjening omtales som et bevisst, men diskutabelt designvalg. Kun en uavhengig kilde funnet. [Kriterium W005]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EV_000007</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>REV_000006</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>MacRumors bekrefter at Apple CarPlay per undersokelsestidspunkt (juli 2026) fortsatt ikke stottes pa noen Tesla-modell, inkludert Model 3. Tesla har varslet tradlos CarPlay "i lopet av kommende maneder" (kunngjort november 2025), men uten bekreftet lanseringsdato. [Kriterium W007]</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EV_000008</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>REV_000007</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Rekkevidde/lading</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Offisiell spesifikasjon viser 250 kW DC-hurtiglading (opptil 282 km pa 15 minutter) og 13,6 kWh/100km forbruk for denne konfigurasjonen - godt over minimumsbehovet gitt lav estimert arlig kjorelengde (~8000 km/ar), men ladehastighet er uansett lavt vektet i denne kriteriemodellen. [Kriterium W020]</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EV_000009,EV_000010</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>1.2</t>
         </is>
       </c>
     </row>
@@ -3801,7 +6048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3856,6 +6103,326 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>EV_000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Cabin/road noise (2024+ refresh)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Motor.no: tire noise now among the best in class; noise level noticeably lower after the 2024 refresh (tested: Long Range AWD).</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>SRC_MOTORNO_MODEL3_2024</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>EV_000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Cabin/road noise (2024+ refresh)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Cars.com: NVH reduced a claimed 20% vs. previous generation; thicker padding, insulation and new acoustic glass muffle the interior (tested: Long Range).</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SRC_CARSCOM_MODEL3_2024</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EV_000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Ride comfort/suspension</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Motor.no: stiff at low speed, comfortable at higher speeds; scored 8/10 for comfort (tested: Long Range AWD).</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>SRC_MOTORNO_MODEL3_2024</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EV_000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Ride comfort/suspension</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Cars.com: frequency-dependent damper valves adapt to impacts; no jarring hits or unsettledness; tire impacts quieter and less intrusive (tested: Long Range).</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>SRC_CARSCOM_MODEL3_2024</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EV_000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Steering precision</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Motor.no: direct, somewhat heavy steering feel with immediate response to small inputs; awarded 10/10 for driving characteristics (tested: Long Range AWD).</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>SRC_MOTORNO_MODEL3_2024</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EV_000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Forward/rear visibility</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Motor.no: excellent forward visibility, poor rearward visibility (tested: Long Range AWD).</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>SRC_MOTORNO_MODEL3_2024</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EV_000007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Infotainment control scheme</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Cars.com: touch-capacitive turn-signal controls "didn't engage at all" at times, reviewer "often hit the wrong turn direction"; phone key occasionally failed to recognize presence (tested: Long Range).</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>SRC_CARSCOM_MODEL3_2024</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EV_000008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Apple CarPlay availability</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>MacRumors (2025-11-16): CarPlay not currently supported on any Tesla model; Tesla plans standard wireless CarPlay 'in coming months' per Bloomberg's Mark Gurman, appearing as a window within Tesla's interface rather than replacing it.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>SRC_MACRUMORS_CARPLAY_2025</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EV_000009</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DC fast-charging power</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Official Tesla specification: Supercharging-Max rated at 250 kW, adding up to 282 km of range in 15 minutes for the Long Range bakhjulsdrift configuration.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>EV_000010</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Real-world energy consumption</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Official Tesla specification: rated power consumption of 13.6 kWh/100km for Long Range bakhjulsdrift, CO2 efficiency class A.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Update framework documentation to version 1.4, introducing the OverallScore entity and its relationships, enhancing the scoring model with coverage percentages, and refining the garage friendliness criteria. Additionally, update the workbook schema to include OverallScores and clarify the calculation methods for scores.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -18,6 +18,7 @@
     <sheet name="09_Sources" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="10_Scoring" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="11_DecisionLog" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="12_OverallScores" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="Enum_Availability">'README'!$X$2:$X$6</definedName>
@@ -369,7 +370,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -441,7 +442,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -689,7 +690,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Configuration Status implemented per ADR-004 (IMPL-002). Structure synchronized to Framework Version 1.2.</t>
+          <t>Scoring mechanics implemented per ADR-005: 10_Scoring RawScore/WeightedScore are now formulas (1-5 Review.Score scale, documented rounding rule); new 12_OverallScores worksheet aggregates Configuration-level Overall Score with mandatory CoveragePercent.</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
@@ -1115,14 +1116,16 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>80</v>
-      </c>
-      <c r="G2" t="n">
-        <v>6.4</v>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F2">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D2,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>ROUND(F2*INDEX('01_Criteria'!$F:$F,MATCH(C2,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -1153,14 +1156,16 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>80</v>
-      </c>
-      <c r="G3" t="n">
-        <v>5.6</v>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F3">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D3,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>ROUND(F3*INDEX('01_Criteria'!$F:$F,MATCH(C3,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -1191,14 +1196,16 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>60</v>
-      </c>
-      <c r="G4" t="n">
-        <v>3</v>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F4">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D4,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>ROUND(F4*INDEX('01_Criteria'!$F:$F,MATCH(C4,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1229,14 +1236,16 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>80</v>
-      </c>
-      <c r="G5" t="n">
-        <v>4</v>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F5">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D5,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>ROUND(F5*INDEX('01_Criteria'!$F:$F,MATCH(C5,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1267,14 +1276,16 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>60</v>
-      </c>
-      <c r="G6" t="n">
-        <v>4.2</v>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F6">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D6,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>ROUND(F6*INDEX('01_Criteria'!$F:$F,MATCH(C6,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1305,14 +1316,16 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.6</v>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F7">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D7,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>ROUND(F7*INDEX('01_Criteria'!$F:$F,MATCH(C7,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1343,14 +1356,16 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>80</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1.6</v>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F8">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D8,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>ROUND(F8*INDEX('01_Criteria'!$F:$F,MATCH(C8,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1370,7 +1385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1515,9 +1530,223 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DEC_GAP_E_001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Reconciled Garasje category in docs/02_criteria-and-weighting.md</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>The vertical-slice review found 01_Criteria already contains a live, weighted "Garasje" category (W019, weight 3) that docs/02 did not document as its own category - only as a sub-example under Practicality. Documentation-only fix; no weights or 01_Criteria data changed.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Gap E from the post-vertical-slice architecture review. No ADR required (descriptive reconciliation of already-live data, not a methodology change).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DEC_ADR_006</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Implemented ADR-006 (Evidence Schema Reconciliation)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>08_Evidence diverged from documented schema (Claim/Evidence split, unused ReviewID column violating the documented one-way Review-&gt;Evidence flow). Reconciled to the documented Observation column; ReviewID column removed.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Migrated 10 existing Evidence records from the vertical slice to the merged Observation format. Ratified comma-separated EvidenceID on 07_Reviews as the 1:N representation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DEC_ADR_005</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Implemented ADR-005 (Scoring Mechanics)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No documented numeric scale, no calculation engine, and no Overall Score entity/worksheet existed despite implementation-contract.md requiring calculated Overall Scores. Ratified 1-5 Review.Score scale and rounding rule; converted 10_Scoring RawScore/WeightedScore to formulas; added 12_OverallScores with mandatory CoveragePercent.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Regression-checked: the 7 existing vertical-slice Score rows reproduce the known values (25.4 total WeightedScore, 37% coverage) under the new formulas.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>OverallScoreID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ConfigurationID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>FrameworkVersion</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>OverallScore</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>CoveragePercent</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CriteriaScored</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>CriteriaTotal</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>OVSC_000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D2">
+        <f>SUMIFS('10_Scoring'!$G$2:$G$1000,'10_Scoring'!$B$2:$B$1000,B2,'10_Scoring'!$E$2:$E$1000,C2)</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>ROUND(SUMPRODUCT(('10_Scoring'!$B$2:$B$1000=B2)*('10_Scoring'!$E$2:$E$1000=C2)*IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH('10_Scoring'!$C$2:$C$1000,'01_Criteria'!$A$2:$A$1000,0)),0))/SUMIFS('01_Criteria'!$F$2:$F$1000,'01_Criteria'!$E$2:$E$1000,"WEIGHTED",'01_Criteria'!$H$2:$H$1000,"TRUE")*100,2)</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>COUNTIFS('10_Scoring'!$B$2:$B$1000,B2,'10_Scoring'!$E$2:$E$1000,C2)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>COUNTIFS('01_Criteria'!$E$2:$E$1000,"WEIGHTED",'01_Criteria'!$H$2:$H$1000,"TRUE")</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>IF(E2&lt;100,"Partial evaluation - "&amp;F2&amp;" of "&amp;G2&amp;" WEIGHTED+Active criteria scored ("&amp;E2&amp;"% of total weight).","Complete evaluation - all WEIGHTED+Active criteria scored.")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -6052,13 +6281,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="72" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -6079,29 +6306,21 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>ReviewID</t>
+          <t>Observation</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Claim</t>
+          <t>SourceID</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>SourceID</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
           <t>Confidence</t>
         </is>
       </c>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6114,22 +6333,17 @@
           <t>TESLA_MODEL_3</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Cabin/road noise (2024+ refresh): Motor.no: tire noise now among the best in class; noise level noticeably lower after the 2024 refresh (tested: Long Range AWD).</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Cabin/road noise (2024+ refresh)</t>
+          <t>SRC_MOTORNO_MODEL3_2024</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
-        <is>
-          <t>Motor.no: tire noise now among the best in class; noise level noticeably lower after the 2024 refresh (tested: Long Range AWD).</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>SRC_MOTORNO_MODEL3_2024</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -6146,22 +6360,17 @@
           <t>TESLA_MODEL_3</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Cabin/road noise (2024+ refresh): Cars.com: NVH reduced a claimed 20% vs. previous generation; thicker padding, insulation and new acoustic glass muffle the interior (tested: Long Range).</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Cabin/road noise (2024+ refresh)</t>
+          <t>SRC_CARSCOM_MODEL3_2024</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
-        <is>
-          <t>Cars.com: NVH reduced a claimed 20% vs. previous generation; thicker padding, insulation and new acoustic glass muffle the interior (tested: Long Range).</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>SRC_CARSCOM_MODEL3_2024</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -6178,22 +6387,17 @@
           <t>TESLA_MODEL_3</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ride comfort/suspension: Motor.no: stiff at low speed, comfortable at higher speeds; scored 8/10 for comfort (tested: Long Range AWD).</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Ride comfort/suspension</t>
+          <t>SRC_MOTORNO_MODEL3_2024</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
-        <is>
-          <t>Motor.no: stiff at low speed, comfortable at higher speeds; scored 8/10 for comfort (tested: Long Range AWD).</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>SRC_MOTORNO_MODEL3_2024</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -6210,22 +6414,17 @@
           <t>TESLA_MODEL_3</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ride comfort/suspension: Cars.com: frequency-dependent damper valves adapt to impacts; no jarring hits or unsettledness; tire impacts quieter and less intrusive (tested: Long Range).</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ride comfort/suspension</t>
+          <t>SRC_CARSCOM_MODEL3_2024</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
-        <is>
-          <t>Cars.com: frequency-dependent damper valves adapt to impacts; no jarring hits or unsettledness; tire impacts quieter and less intrusive (tested: Long Range).</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>SRC_CARSCOM_MODEL3_2024</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -6242,22 +6441,17 @@
           <t>TESLA_MODEL_3</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Steering precision: Motor.no: direct, somewhat heavy steering feel with immediate response to small inputs; awarded 10/10 for driving characteristics (tested: Long Range AWD).</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Steering precision</t>
+          <t>SRC_MOTORNO_MODEL3_2024</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
-        <is>
-          <t>Motor.no: direct, somewhat heavy steering feel with immediate response to small inputs; awarded 10/10 for driving characteristics (tested: Long Range AWD).</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>SRC_MOTORNO_MODEL3_2024</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -6274,22 +6468,17 @@
           <t>TESLA_MODEL_3</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Forward/rear visibility: Motor.no: excellent forward visibility, poor rearward visibility (tested: Long Range AWD).</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Forward/rear visibility</t>
+          <t>SRC_MOTORNO_MODEL3_2024</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
-        <is>
-          <t>Motor.no: excellent forward visibility, poor rearward visibility (tested: Long Range AWD).</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>SRC_MOTORNO_MODEL3_2024</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -6306,22 +6495,17 @@
           <t>TESLA_MODEL_3</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Infotainment control scheme: Cars.com: touch-capacitive turn-signal controls "didn't engage at all" at times, reviewer "often hit the wrong turn direction"; phone key occasionally failed to recognize presence (tested: Long Range).</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Infotainment control scheme</t>
+          <t>SRC_CARSCOM_MODEL3_2024</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
-        <is>
-          <t>Cars.com: touch-capacitive turn-signal controls "didn't engage at all" at times, reviewer "often hit the wrong turn direction"; phone key occasionally failed to recognize presence (tested: Long Range).</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>SRC_CARSCOM_MODEL3_2024</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -6338,22 +6522,17 @@
           <t>TESLA_MODEL_3</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Apple CarPlay availability: MacRumors (2025-11-16): CarPlay not currently supported on any Tesla model; Tesla plans standard wireless CarPlay 'in coming months' per Bloomberg's Mark Gurman, appearing as a window within Tesla's interface rather than replacing it.</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Apple CarPlay availability</t>
+          <t>SRC_MACRUMORS_CARPLAY_2025</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
-        <is>
-          <t>MacRumors (2025-11-16): CarPlay not currently supported on any Tesla model; Tesla plans standard wireless CarPlay 'in coming months' per Bloomberg's Mark Gurman, appearing as a window within Tesla's interface rather than replacing it.</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>SRC_MACRUMORS_CARPLAY_2025</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -6370,22 +6549,17 @@
           <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>DC fast-charging power: Official Tesla specification: Supercharging-Max rated at 250 kW, adding up to 282 km of range in 15 minutes for the Long Range bakhjulsdrift configuration.</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DC fast-charging power</t>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
-        <is>
-          <t>Official Tesla specification: Supercharging-Max rated at 250 kW, adding up to 282 km of range in 15 minutes for the Long Range bakhjulsdrift configuration.</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -6402,22 +6576,17 @@
           <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Real-world energy consumption: Official Tesla specification: rated power consumption of 13.6 kWh/100km for Long Range bakhjulsdrift, CO2 efficiency class A.</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Real-world energy consumption</t>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
-        <is>
-          <t>Official Tesla specification: rated power consumption of 13.6 kWh/100km for Long Range bakhjulsdrift, CO2 efficiency class A.</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -6426,7 +6595,7 @@
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Enum_Confidence</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update EV Decision Framework workbook to incorporate recent modifications in data structure and scoring model adjustments.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -2721,7 +2721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3048,6 +3048,43 @@
       <c r="G9" t="inlineStr">
         <is>
           <t>Skoda Elroq length (4488mm) passes the 4500mm hard requirement by only 12mm - flagged as a near-miss. A second genuine cross-source disagreement was documented (Motor.no vs What Car? on Elroq road noise), mirroring the Renault comfort discrepancy. Volvo EX30 representative configuration (P8 AWD) was chosen because it matches what Motor.no actually tested, not for cross-vehicle class parity - noted as an asymmetry versus the other 3 vehicles picks (mid-tier RWD/long-range).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DEC_DATA_005</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Populated 05_Equipment using the existing 06_EquipmentDefinitions catalog</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>06_EquipmentDefinitions was already fully authored (20 definitions) - not empty as previously assumed. Mapped 05_Equipment availability to 3 existing definitions (EQ_ACC, EQ_REAR_CAMERA, EQ_CARPLAY) only where already-gathered research provided a sourced answer.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>38 Equipment rows added across Tesla, Renault, Skoda and Volvo configurations, including RENAULT_4_EVOLUTION_URBAN/COMFORT (both EQ_ACC=UNAVAILABLE, formally documenting the Hard Requirement M004 failure already noted in 03_Configurations Notes). Remaining 17 EquipmentDefinitions left unpopulated - no sourced data gathered for them yet.</t>
         </is>
       </c>
     </row>
@@ -11927,7 +11964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11967,6 +12004,1222 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Confidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>EQ_000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_URBAN</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>EQ_000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_COMFORT</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EQ_000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EQ_000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EQ_000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EQ_000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EQ_000007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_ESSENCE_60</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EQ_000008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EQ_000009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_85X</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>EQ_000010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_RS</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EQ_000011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SRC_MOTORNO_EX30_2024</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>EQ_000012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_URBAN</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>EQ_000013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_COMFORT</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>EQ_000014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>EQ_000015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EQ_000016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>EQ_000017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>EQ_000018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_ESSENCE_60</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>EQ_000019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>EQ_000020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_85X</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>EQ_000021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_RS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>EQ_000022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SRC_MACRUMORS_CARPLAY_2025</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EQ_000023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SRC_MACRUMORS_CARPLAY_2025</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>EQ_000024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SRC_MACRUMORS_CARPLAY_2025</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>EQ_000025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SRC_MACRUMORS_CARPLAY_2025</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>EQ_000026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_URBAN</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>EQ_000027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_COMFORT</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>EQ_000028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>EQ_000029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>EQ_000030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>EQ_000031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>EQ_000032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_ESSENCE_60</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>EQ_000033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>EQ_000034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_85X</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>EQ_000035</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_RS</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>EQ_000036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_EX30_2026</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>EQ_000037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_EX30_2026</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>EQ_000038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_EX30_2026</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update EV Decision Framework workbook to reflect recent changes in data structure and scoring model adjustments.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1514,6 +1514,191 @@
       <c r="H18" t="inlineStr">
         <is>
           <t>UK professional review. Covers CarPlay, steering, ride comfort, cabin noise, and outward visibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Tilbud: Kia EV2 FWD Long Range GT Line</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Bertel O. Steen Lorenskog (authorized Kia dealer)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Official dealer sales quote (PDF), valid to 2026-07-12. Covers configuration, trim/equipment list, and full pricing breakdown for the specific GT Line configuration. No battery/range/charging/dimension figures included. Customer contact details in the source document deliberately excluded from this citation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SRC_KIA_NETTBUTIKK_EV2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>EV2 FWD Long Range GT Line - Oppsummering (Kia nettbutikk)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Kia Norge</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://nettbutikk.kia.no/ev2/oppsummering</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Official Kia Norway configurator, saved configuration code A2231F29 (verified directly by fetching the live page 2026-07-06 - matches text supplied by user exactly). Technical data section contains confirmed unit-label errors on Kia's own page template: "Bagasjerom"/"Frunk" labeled kg (should be L, volume), "Forbruk" labeled kWh/km (should be kWh/100km - confirmed by cross-check: 62kWh battery / 15.2kWh-per-100km implies ~408km range, consistent with the stated 453km WLTP figure; taken literally as kWh/km the range would be ~4km, which is physically absurd), "Batterikapasitet" labeled kW (should be kWh, energy not power - same cross-check applies). Numeric values are trusted (official source, tied to a specific saved configuration); unit labels corrected based on physical plausibility and internal arithmetic consistency, not assumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SRC_MOTORNO_EV2_2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Prøvekjørt: Kia EV2, nå begynner smått å bli virkelig godt</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Motor.no</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.motor.no/aktuelt/provekjort-kia-ev2-na-begynner-smatt-a-bli-virkelig-godt/350785</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Test av Kia EV2 Standard Range (42.2 kWh, 147 hk), testet i Lisboa. Dekker fjaering/komfort og sikt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_EV2_2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Kia EV2 Review 2026, Price &amp; Specs</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>What Car?</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.whatcar.com/kia/ev2/hatchback/review/n28833</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>UK professional review. Covers CarPlay, steering, ride comfort, cabin noise and outward visibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SRC_RAC_EV2_2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Kia EV2 Review 2026: Prices, specs and verdict</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>RAC Drive</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://www.rac.co.uk/drive/car-reviews/kia/ev2/ev2/</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>UK professional review. Covers infotainment/touchscreen quality.</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2709,6 +2894,286 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SCORE_000030</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>W001</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>REV_000029</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F30">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D30,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G30">
+        <f>ROUND(F30*INDEX('01_Criteria'!$F:$F,MATCH(C30,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000029 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SCORE_000031</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>W002</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>REV_000030</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F31">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D31,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G31">
+        <f>ROUND(F31*INDEX('01_Criteria'!$F:$F,MATCH(C31,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000030 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SCORE_000032</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>W003</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>REV_000031</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F32">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D32,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G32">
+        <f>ROUND(F32*INDEX('01_Criteria'!$F:$F,MATCH(C32,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000031 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SCORE_000033</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>W004</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>REV_000032</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F33">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D33,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G33">
+        <f>ROUND(F33*INDEX('01_Criteria'!$F:$F,MATCH(C33,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000032 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SCORE_000034</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>W005</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>REV_000033</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F34">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D34,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G34">
+        <f>ROUND(F34*INDEX('01_Criteria'!$F:$F,MATCH(C34,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000033 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SCORE_000035</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>W007</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>REV_000034</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F35">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D35,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G35">
+        <f>ROUND(F35*INDEX('01_Criteria'!$F:$F,MATCH(C35,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000034 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SCORE_000036</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>W020</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>REV_000035</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F36">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D36,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G36">
+        <f>ROUND(F36*INDEX('01_Criteria'!$F:$F,MATCH(C36,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000035 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2721,7 +3186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3088,6 +3553,117 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DEC_DATA_006</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Populated Kia EV2 from a real dealer sales quote (user-supplied PDF)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>A genuine, dated Bertel O. Steen (Kia dealer) sales quote for EV2 FWD Long Range GT Line reconciled the earlier "not on Kia Norway model list" uncertainty - Vehicle status updated from UNKNOWN to AVAILABLE.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Added KIA_EV2_FWD_LONG_RANGE_GT_LINE configuration with BasePrice/ConfiguredPrice split (trim price vs. this specific buyers customized quote incl. 4-seat conversion and winter wheels), and 14 Equipment rows from the itemized equipment list. No Technical (battery/range/charging/dimensions) facts were available in the quote document - explicitly left Unknown rather than assumed. Customer personal contact details deliberately excluded from all workbook citations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DEC_DATA_007</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Populated Kia EV2 Technical facts from Kia official web store, correcting unit-label errors</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Verified nettbutikk.kia.no/ev2/oppsummering directly (config code A2231F29). Confirmed the page itself mislabels several units (kg instead of L for boot/frunk, kW instead of kWh for battery, kWh/km instead of kWh/100km for consumption) - a bug on Kia's own site, not a user transcription error.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>7 Technical rows added. Battery net (62kWh) and WLTP consumption (15.2kWh/100km) corrections verified via arithmetic cross-check against the stated 453km range - high confidence in the correction logic. Boot/Frunk volume corrections (kg-&gt;L) recorded at LOW confidence since no independent cross-check was available for those two.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DEC_DATA_008</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Added Kia EV2 Evidence/Review/Score - now 5th vehicle in the thin-slice comparison</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Completed the same 7-criterion pipeline (Motor.no, What Car?, RAC Drive) for KIA_EV2_FWD_LONG_RANGE_GT_LINE, alongside Tesla, Renault, Skoda and Volvo.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>DC fast-charging power was never stated on the Kia configurator - W020 scored at reduced (LOW) confidence reflecting this gap. A third genuine cross-source ride-comfort disagreement was documented (Motor.no tested Standard Range as stiff/bouncy; What Car? found the suspension soft or supple) - same pattern as Renault and Skoda.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3100,7 +3676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3300,6 +3876,43 @@
       </c>
       <c r="H5">
         <f>IF(E5&lt;100,"Partial evaluation - "&amp;F5&amp;" of "&amp;G5&amp;" WEIGHTED+Active criteria scored ("&amp;E5&amp;"% of total weight).","Complete evaluation - all WEIGHTED+Active criteria scored.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>OVSC_000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D6">
+        <f>SUMIFS('10_Scoring'!$G$2:$G$1000,'10_Scoring'!$B$2:$B$1000,B6,'10_Scoring'!$E$2:$E$1000,C6)</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>ROUND(SUMPRODUCT(('10_Scoring'!$B$2:$B$1000=B6)*('10_Scoring'!$E$2:$E$1000=C6)*IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH('10_Scoring'!$C$2:$C$1000,'01_Criteria'!$A$2:$A$1000,0)),0))/SUMIFS('01_Criteria'!$F$2:$F$1000,'01_Criteria'!$E$2:$E$1000,"WEIGHTED",'01_Criteria'!$H$2:$H$1000,"TRUE")*100,2)</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>COUNTIFS('10_Scoring'!$B$2:$B$1000,B6,'10_Scoring'!$E$2:$E$1000,C6)</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>COUNTIFS('01_Criteria'!$E$2:$E$1000,"WEIGHTED",'01_Criteria'!$H$2:$H$1000,"TRUE")</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>IF(E6&lt;100,"Partial evaluation - "&amp;F6&amp;" of "&amp;G6&amp;" WEIGHTED+Active criteria scored ("&amp;E6&amp;"% of total weight).","Complete evaluation - all WEIGHTED+Active criteria scored.")</f>
         <v/>
       </c>
     </row>
@@ -4844,12 +5457,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>AVAILABLE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Kia Norway official model list reviewed 2026-07-06; EV2 not listed, so Norwegian lifecycle/configuration data remains unverified.</t>
+          <t>Official dealer sales quote from Bertel O. Steen Lorenskog (authorized Kia dealer), quote valid to 2026-07-12, reviewed 2026-07-06 - supersedes the earlier "not listed on Kia Norway model list" observation with concrete, dated transactional evidence of market availability. Configuration: EV2 FWD Long Range GT Line, 135 hk, forhjulsdrift. No battery capacity, WLTP range, charging power, or dimensions were stated anywhere in the quote document.</t>
         </is>
       </c>
     </row>
@@ -5018,7 +5631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5692,6 +6305,44 @@
       <c r="H18" t="inlineStr">
         <is>
           <t>Volvo Norway official specifications page reviewed 2026-07-06. Same Hard Requirement notes as P5. This is the configuration actually tested by Motor.no (Evidence directly applicable, not inferred across trims).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>KIA_EV2</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>FWD Long Range GT Line, 135 hk</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>346417</v>
+      </c>
+      <c r="G19" t="n">
+        <v>423340</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Official Bertel O. Steen (Kia dealer) sales quote reviewed 2026-07-06, valid to 2026-07-12. BasePrice (346417 kr) = base EV2 FWD Long Range (251655 kr) + GT Line package (94762 kr), i.e. the trim as sold. ConfiguredPrice (423340 kr) = this specific quote total, which additionally includes buyer-selected options not part of the base GT Line trim: 4-seat sliding-seat conversion (+3200 kr), 16" Nokian studded winter wheels (+23603 kr), plus delivery (12500 kr), VAT (21430 kr) and registration tax/vrakpant (16190 kr). Colour (Frost Blue - Solid) and interior (Grey/Black) were no-cost selections. No battery capacity, WLTP range, charging power, or vehicle dimensions were stated in the source document - these remain Unknown pending a manufacturer specification sheet.</t>
         </is>
       </c>
     </row>
@@ -5715,7 +6366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J141"/>
+  <dimension ref="A1:J148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11939,6 +12590,321 @@
         </is>
       </c>
       <c r="J141" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>TECH_000135</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>WLTP range</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>453</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>SRC_KIA_NETTBUTIKK_EV2</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>TECH_000136</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>WLTP consumption</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>KWH_100KM</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>SRC_KIA_NETTBUTIKK_EV2</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>TECH_000137</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>AC max charging</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>11</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>SRC_KIA_NETTBUTIKK_EV2</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>TECH_000138</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Battery net</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>62</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>KWH</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>SRC_KIA_NETTBUTIKK_EV2</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>TECH_000139</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Max trailer weight</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>750</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>SRC_KIA_NETTBUTIKK_EV2</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>TECH_000140</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Boot volume</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>362</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>SRC_KIA_NETTBUTIKK_EV2</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>TECH_000141</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Frunk volume</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>15</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>SRC_KIA_NETTBUTIKK_EV2</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -11964,7 +12930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -13220,6 +14186,454 @@
       <c r="F39" t="inlineStr">
         <is>
           <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>EQ_000039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>EQ_CARPLAY</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>EQ_000040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>EQ_360</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>EQ_000041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>EQ_000042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>EQ_OTA</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>EQ_000043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>EQ_000044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>EQ_LANE_CENTER</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>EQ_000045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>EQ_DIGITAL_KEY</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>EQ_000046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>EQ_HEATPUMP</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>EQ_000047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>EQ_WIRELESS_CHARGE</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>EQ_000048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>EQ_AUDIO</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>EQ_000049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>EQ_V2L</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>EQ_000050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>EQ_VENT_SEATS</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>EQ_000051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>EQ_AMBIENT</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>EQ_000052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>EQ_APP</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -13843,7 +15257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -15019,6 +16433,286 @@
         </is>
       </c>
       <c r="I29" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>REV_000029</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>4</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>What Car? rapporterer lite motorstoy, lite dekkstoy pa motorvei og lite fjaeringsstoy i by. Kun en uavhengig kilde funnet. [Kriterium W001]</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EV_000040</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>REV_000030</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Motor.no rapporterer at bilen rister over brostein og oppleves spretten i hoyere hastighet pa Standard Range-varianten, med dempere beskrevet som stive og "ikke spesielt sofistikerte." What Car? rapporterer motsatt at fjaeringen er relativt myk og glatter ut humper, om enn med krengning i svinger. Direkte motstridende funn - dokumentert som uenighet, ikke lost. [Kriterium W002]</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>EV_000041,EV_000042</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>REV_000031</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Motor.no og What Car? er begge enige om god sikt: firkantet form med store glassflater og oppreiste stolper gir god oversikt i alle retninger. To uavhengige kilder enige. [Kriterium W003]</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>EV_000043</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>REV_000032</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>What Car? beskriver styringen som "a bit vague," satt opp for enkelhet fremfor styrefolelse eller engasjement. Kun en uavhengig kilde funnet, men et klart negativt funn. [Kriterium W004]</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>EV_000044</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>REV_000033</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>RAC Drive: skjermen er "responsive... easy to understand... has all the latest features," men matcher ikke Renaults visuelle polish. Beholder fysiske knapper for temperatur/vifte/setevarme/volum. Kun en uavhengig kilde funnet. [Kriterium W005]</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>EV_000045</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>REV_000034</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>What Car? bekrefter at "Apple CarPlay and Android Auto are standard on all versions." Samme positive funn som Renault 4, Skoda Elroq og Volvo EX30; motsatt funn av Tesla Model 3 Long Range RWD. [Kriterium W007]</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>EV_000046</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>REV_000035</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Rekkevidde/lading</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Offisiell konfigurator viser 11 kW AC-lading og 15,2 kWh/100km forbruk for denne konfigurasjonen. DC-hurtigladeeffekt var ikke oppgitt pa kildesiden, noe som begrenser vurderingen av reell ladeegenskap sammenlignet med de andre bilene. [Kriterium W020]</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>EV_000047</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -15041,7 +16735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16139,6 +17833,222 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>EV_000040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>KIA_EV2</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Cabin/road noise: What Car?: "very little electric motor whine under acceleration. There isn't much tyre noise on the motorway, either, or suspension noise around town."</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_EV2_2026</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>EV_000041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>KIA_EV2</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Ride comfort/suspension: Motor.no: "Det rister godt over brostein, og humper og dumper i litt hoyere hastigheter gir en vel spretten folelse" (shakes noticeably over cobblestones, bouncy over bumps at higher speed); dampers described as stiff and "not particularly sophisticated" (tested: Standard Range, 42.2 kWh).</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SRC_MOTORNO_EV2_2026</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>EV_000042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>KIA_EV2</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Ride comfort/suspension: What Car?: "relatively soft suspension helps smother ridges and small potholes," though the car exhibits "plenty of lean when going around corners quickly" - directly contrasts with Motor.no's "stiff" characterization on the Standard Range.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_EV2_2026</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>EV_000043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>KIA_EV2</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Outward visibility: Motor.no: angular shape with large glass surfaces gives good sightlines from the driver seat (tested: Standard Range). What Car?: "upright pillars and tall, oblong windows give you a great view out in all directions." Two independent sources agree.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SRC_MOTORNO_EV2_2026</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>EV_000044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>KIA_EV2</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Steering precision: What Car?: "the steering is a bit vague," set up for ease rather than steering feel or engagement.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_EV2_2026</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>EV_000045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>KIA_EV2</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Infotainment/software quality: RAC Drive: touchscreen is "responsive and the menu layout is easy to understand, while it has all the latest features," though "doesn't quite manage to look as slick as Renault's infotainment system." Retains physical switchgear for temperature/fan/seat heating/volume.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SRC_RAC_EV2_2026</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>EV_000046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>KIA_EV2</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Apple CarPlay availability: What Car?: "Apple CarPlay and Android Auto are standard on all versions."</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_EV2_2026</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>EV_000047</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>AC charging power and real-world energy consumption: Official Kia nettbutikk configurator: 11 kW three-phase onboard AC charger, rated consumption 15.2 kWh/100km (corrected from a mislabeled kWh/km unit on the source page). DC fast-charging power not stated on the source page.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SRC_KIA_NETTBUTIKK_EV2</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Update EV Decision Framework workbook to include further refinements in data structure and scoring model adjustments.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1699,6 +1699,127 @@
       <c r="H23" t="inlineStr">
         <is>
           <t>UK professional review. Covers infotainment/touchscreen quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_VOLVO_EX30_WINTER</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Vintertest av Volvo EX30: Denne bilen forteller deg om batterihelsen sin</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Norsk elbilforening (elbil.no)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://elbil.no/vinter-test-av-volvo-ex30-denne-bilen-forteller-deg-om-batterihelsen-sin/</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2025-02-26</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Independent winter test (Tier A: independent winter testing). Tested Twin Performance (dual-motor AWD Ultra) - matches VOLVO_EX30_P8_AWD powertrain. Estimated ~75% of WLTP range retained under real winter conditions (down to approx. -20C) after accounting for a mid-route fast-charge stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_RENAULT4_TEST</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Test av Renault 4: Billig sjarmklump som fort blir dyr</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Norsk elbilforening (elbil.no)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://elbil.no/test-av-renault-4/</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2025-11-05</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>General road test, not a dedicated winter cold-chamber test. Tested Iconic trim (52kWh, same powertrain as Techno, different equipment level) at highway consumption of 1.81 kWh/mil (18.1 kWh/100km) at constant 100km/h in 5-7C conditions - not extreme winter cold. Measured range at this consumption: 287km. Used as a cautious proxy only, explicitly flagged as trim- and condition-mismatched to the Techno configuration and to true deep-winter conditions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_DESIGN</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Design din Model 3 | Tesla</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://www.tesla.com/no_no/model3/design</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Official Tesla Norway configurator. Verified total price for Long Range bakhjulsdrift (Long Range RWD) with no optional extras selected: 369990 kr excl. VAT/fees, 400539 kr incl. VAT and fees.</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3174,6 +3295,206 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SCORE_000037</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>W017</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>REV_000036</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F37">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D37,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G37">
+        <f>ROUND(F37*INDEX('01_Criteria'!$F:$F,MATCH(C37,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000036 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SCORE_000038</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>W017</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>REV_000037</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F38">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D38,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G38">
+        <f>ROUND(F38*INDEX('01_Criteria'!$F:$F,MATCH(C38,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000037 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SCORE_000039</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>W017</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>REV_000038</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F39">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D39,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G39">
+        <f>ROUND(F39*INDEX('01_Criteria'!$F:$F,MATCH(C39,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000038 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SCORE_000040</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>W017</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>REV_000039</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F40">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D40,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G40">
+        <f>ROUND(F40*INDEX('01_Criteria'!$F:$F,MATCH(C40,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000039 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SCORE_000041</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>W017</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>REV_000040</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F41">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D41,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G41">
+        <f>ROUND(F41*INDEX('01_Criteria'!$F:$F,MATCH(C41,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000040 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3186,7 +3507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3661,6 +3982,80 @@
       <c r="G13" t="inlineStr">
         <is>
           <t>DC fast-charging power was never stated on the Kia configurator - W020 scored at reduced (LOW) confidence reflecting this gap. A third genuine cross-source ride-comfort disagreement was documented (Motor.no tested Standard Range as stiff/bouncy; What Car? found the suspension soft or supple) - same pattern as Renault and Skoda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DEC_M003_VERIFY</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Attempted M003 (winter highway range hard requirement) verification for all 5 scored configurations</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Only 1 of 5 (Volvo EX30 P8 AWD) had a clean, trim-matched independent winter test (elbil.no) - passes comfortably at ~338km. Renault 4 Techno has a flagged, non-matching proxy data point (287km, wrong trim, mild not winter conditions) that is a concerning signal, not a confirmed pass. Skoda Elroq, Tesla Model 3, and Kia EV2 have no reliable independent winter data at all.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Per user direction: Renault proxy recorded with explicit caveats rather than discarded; the other 3 remain genuinely Unknown rather than assumed. No configuration was removed from scoring - none was confirmed to fail M003, so all 5 proceed to Del 2 (Price/Value) as planned. Winter range verification for Skoda/Tesla/Kia should be revisited when better sources become available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DEC_W017_SCORE</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Scored Price/Value (W017, weight 10) for all 5 configurations</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Judged price relative to range/charging/equipment delivered in class per user direction, not pure price ranking. Discovered and fixed a real gap: Tesla Model 3 Long Range RWD had no price data at all since DATA-001 - fetched 400539 kr from the official Tesla configurator.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Coverage now 47% (8 of 20 weighted criteria). Volvo EX30 P8 AWD scored lowest on this criterion - its price premium goes toward performance (0-100 time), which the framework explicitly excludes as a meaningful ownership factor, so that premium is not counted as good value here.</t>
         </is>
       </c>
     </row>
@@ -5776,9 +6171,15 @@
           <t>Long Range bakhjulsdrift</t>
         </is>
       </c>
+      <c r="F4" t="n">
+        <v>400539</v>
+      </c>
+      <c r="G4" t="n">
+        <v>400539</v>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002).</t>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002). M003 (winter highway range): Not verified. Two winter tests were found but both are unreliable matches: a 2022 test used a superseded pre-refresh Model 3 generation with a WLTP figure (614km) that matches no current trim, and a NAF winter 2025 test reports 702km WLTP (matching none of this workbook's four recorded Model 3 configurations) without specifying which trim was tested. Remains genuinely Unknown. Price verified 2026-07-06 via official Tesla Norway configurator (SRC_TESLA_NO_MODEL3_DESIGN): 400539 kr incl. VAT/fees, no optional extras selected (previously unpriced under DATA-001).</t>
         </is>
       </c>
     </row>
@@ -5924,7 +6325,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Renault Norway official price list (Versjon 2, 01-06-2026) reviewed 2026-07-06. Meets all checked Hard Requirements (BEV, length 4140mm, Intelligent cruise control multi target = adaptive, standard rearview camera). M003 (winter highway range) remains Unknown - no winter test data reviewed.</t>
+          <t>Renault Norway official price list (Versjon 2, 01-06-2026) reviewed 2026-07-06. Meets all checked Hard Requirements (BEV, length 4140mm, Intelligent cruise control multi target = adaptive, standard rearview camera). M003 (winter highway range) remains Unknown - no winter test data reviewed. M003 (winter highway range): No dedicated deep-winter test found for this exact configuration. Closest available data point (elbil.no, Iconic trim - same 52kWh/150hk powertrain as Techno, but a different equipment level) measured 287 km at constant 100km/h highway driving in mild 5-7C conditions - NOT true winter cold. Since colder conditions would be expected to reduce range further, this data point is a concerning signal rather than a confident pass: the hard requirement remains genuinely uncertain, possibly at risk of failing, for this configuration. Flagged for the user's attention rather than resolved either way.</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6515,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Skoda Norway official price list (2027-modell, 29.06.2026) reviewed 2026-07-06. Reportedly the most popular Elroq variant per Skoda. Meets all checked Hard Requirements (see Essence 60 note; same length/ACC/camera). M003 remains Unknown.</t>
+          <t>Skoda Norway official price list (2027-modell, 29.06.2026) reviewed 2026-07-06. Reportedly the most popular Elroq variant per Skoda. Meets all checked Hard Requirements (see Essence 60 note; same length/ACC/camera). M003 remains Unknown. M003 (winter highway range): Not verified. NAF's El Prix winter 2026 test included only the Elroq RS variant (different chassis/suspension/power tier), and the results table was rendered as an image, not extractable as text. Searched but found no dedicated winter test for Selection 60 specifically. Remains genuinely Unknown, not assumed.</t>
         </is>
       </c>
     </row>
@@ -6304,7 +6705,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Volvo Norway official specifications page reviewed 2026-07-06. Same Hard Requirement notes as P5. This is the configuration actually tested by Motor.no (Evidence directly applicable, not inferred across trims).</t>
+          <t>Volvo Norway official specifications page reviewed 2026-07-06. Same Hard Requirement notes as P5. This is the configuration actually tested by Motor.no (Evidence directly applicable, not inferred across trims). M003 (winter highway range): Independent test (elbil.no, matching Twin Performance/dual-motor AWD powertrain) estimated ~75% of the 450km WLTP figure retained in real winter conditions (~-20C), i.e. approximately 338 km. This comfortably passes the ~300km hard requirement.</t>
         </is>
       </c>
     </row>
@@ -6342,7 +6743,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Official Bertel O. Steen (Kia dealer) sales quote reviewed 2026-07-06, valid to 2026-07-12. BasePrice (346417 kr) = base EV2 FWD Long Range (251655 kr) + GT Line package (94762 kr), i.e. the trim as sold. ConfiguredPrice (423340 kr) = this specific quote total, which additionally includes buyer-selected options not part of the base GT Line trim: 4-seat sliding-seat conversion (+3200 kr), 16" Nokian studded winter wheels (+23603 kr), plus delivery (12500 kr), VAT (21430 kr) and registration tax/vrakpant (16190 kr). Colour (Frost Blue - Solid) and interior (Grey/Black) were no-cost selections. No battery capacity, WLTP range, charging power, or vehicle dimensions were stated in the source document - these remain Unknown pending a manufacturer specification sheet.</t>
+          <t>Official Bertel O. Steen (Kia dealer) sales quote reviewed 2026-07-06, valid to 2026-07-12. BasePrice (346417 kr) = base EV2 FWD Long Range (251655 kr) + GT Line package (94762 kr), i.e. the trim as sold. ConfiguredPrice (423340 kr) = this specific quote total, which additionally includes buyer-selected options not part of the base GT Line trim: 4-seat sliding-seat conversion (+3200 kr), 16" Nokian studded winter wheels (+23603 kr), plus delivery (12500 kr), VAT (21430 kr) and registration tax/vrakpant (16190 kr). Colour (Frost Blue - Solid) and interior (Grey/Black) were no-cost selections. No battery capacity, WLTP range, charging power, or vehicle dimensions were stated in the source document - these remain Unknown pending a manufacturer specification sheet. M003 (winter highway range): Not verified. No independent winter test was found for the Kia EV2 - likely because the model is too new to the Norwegian market to have been included in a winter test cycle yet. Remains genuinely Unknown.</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J148"/>
+  <dimension ref="A1:J150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12905,6 +13306,96 @@
         </is>
       </c>
       <c r="J148" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>TECH_000142</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Winter highway range estimate</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>338</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_VOLVO_EX30_WINTER</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>TECH_000143</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Winter highway range estimate</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>287</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_RENAULT4_TEST</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -15257,7 +15748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16713,6 +17204,206 @@
         </is>
       </c>
       <c r="I36" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>REV_000036</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Økonomi</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Beste pris per kilometer rekkevidde av alle fem (ca. 534-580 kr/km avhengig av felgvalg, mot 837-1042 kr/km for de andre), kombinert med raskest DC-lading (250 kW) og lavest forbruk (13,6 kWh/100km). Merprisen sammenlignet med Renault forsvares tydelig av vesentlig bedre rekkevidde/lading/effektivitet. [Kriterium W017]</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>EV_000048</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>REV_000037</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Økonomi</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Lavest totalpris av de fem (364 900 kr), men ogsa kortest rekkevidde og tregest DC-lading utenom sammenligningen med Tesla. Grei, men ikke fremragende, verdi for pengene - billig inngangsbillett, men leverer ikke uforholdsmessig mye rekkevidde/lading for prisen sammenlignet med Skoda rett over. [Kriterium W017]</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>EV_000049</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>REV_000038</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Økonomi</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>4</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Kun ca. 10 000 kr dyrere enn Renault 4 Techno, men gir 50 km mer rekkevidde og marginalt raskere lading - beste rekkevidde-per-krone av ikke-Tesla-alternativene. Merprisen forsvares tydelig av det den gir tilbake. [Kriterium W017]</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>EV_000050</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>REV_000039</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Økonomi</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Dyrest av de fem (468 900 kr) og samtidig minst effektiv (17,5 kWh/100km, hoyest forbruk i utvalget) uten tilsvarende mer rekkevidde. Merprisen gar hovedsakelig til firehjulsdrift og ytelse (0-100 pa 3,6 sek), som rammeverket eksplisitt ekskluderer som en meningsfull faktor for langsiktig eierskap. Svakest verdi for pengene av de fem. [Kriterium W017]</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>EV_000051</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>REV_000040</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Økonomi</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Grunnprisen for selve GT Line-trimmen (346 417 kr) er faktisk lavest av alle fem, for nest-best rekkevidde (453 km) og det mest omfattende standardutstyret registrert i dette datasettet. Totalprisen i det spesifikke tilbudet (423 340 kr) reflekterer kjoperens egne tilvalg (4-seter, vinterhjul) og er ikke representativt for trimmens egen verdi. Vurdert pa grunnprisen: sterk verdi for pengene. [Kriterium W017]</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>EV_000052</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -16735,7 +17426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -18049,6 +18740,141 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>EV_000048</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Price positioning: 400539 kr incl. VAT/fees (official Tesla configurator, no options), for 691-750km WLTP range (wheel-dependent), 250kW DC charging and 13.6 kWh/100km consumption - the best price-per-km-range and fastest charging of the five compared configurations.</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_DESIGN</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>EV_000049</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Price positioning: 364900 kr incl. VAT/fees (official Renault price list), for 398km WLTP range and 100kW DC charging - the lowest absolute price of the five, but also the shortest range and slowest charging outside of Tesla's advantage.</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>EV_000050</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Price positioning: 374900 kr incl. VAT/fees (official Skoda price list), for 448km WLTP range and 105kW DC charging - only ~10000 kr above Renault 4 Techno for 50km more range and marginally faster charging.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>EV_000051</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Price positioning: 468900 kr incl. VAT/fees (official Volvo specification page), for 450km WLTP range and 17.5 kWh/100km consumption - the highest price and least efficient consumption of the five, with the premium going primarily toward dual-motor performance rather than range or efficiency.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>SRC_VOLVO_NO_EX30_SPECS</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>EV_000052</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Price positioning: BasePrice 346417 kr incl. VAT/fees for the GT Line trim itself (official Kia configurator/dealer quote), for 453km WLTP range - the second-best range of the five at the lowest trim price, with the richest standard equipment list gathered in this dataset. ConfiguredPrice (423340 kr) reflects this buyer's personal options (4-seat conversion, winter wheels) and is not representative of the trim's own value.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>SRC_KIA_NETTBUTIKK_EV2</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Update EV Decision Framework workbook to implement additional refinements in data structure and scoring model.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1820,6 +1820,43 @@
       <c r="H26" t="inlineStr">
         <is>
           <t>Official Tesla Norway configurator. Verified total price for Long Range bakhjulsdrift (Long Range RWD) with no optional extras selected: 369990 kr excl. VAT/fees, 400539 kr incl. VAT and fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SRC_KIA_UK_SPECS_PDF</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>The Kia EV2 Specifications (Kia UK)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Kia UK</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://www.kia.com/content/dam/kwcms/kme/uk/en/assets/vehicles/ev2/ev2-specifications.pdf</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Official Kia UK specifications PDF. GT Line/GT Line S trim: Length 4065mm, Wheelbase 2565mm, Width 1800mm, Height 1585mm. UK market document, not Norway-specific, but physical dimensions are not expected to differ by market for the same generation/trim.</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3495,6 +3532,206 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SCORE_000042</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>W019</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>REV_000041</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F42">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D42,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G42">
+        <f>ROUND(F42*INDEX('01_Criteria'!$F:$F,MATCH(C42,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000041 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SCORE_000043</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>W019</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>REV_000042</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F43">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D43,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G43">
+        <f>ROUND(F43*INDEX('01_Criteria'!$F:$F,MATCH(C43,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000042 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SCORE_000044</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>W019</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>REV_000043</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F44">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D44,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G44">
+        <f>ROUND(F44*INDEX('01_Criteria'!$F:$F,MATCH(C44,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000043 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SCORE_000045</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>W019</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>REV_000044</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F45">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D45,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G45">
+        <f>ROUND(F45*INDEX('01_Criteria'!$F:$F,MATCH(C45,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000044 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SCORE_000046</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>W019</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>REV_000045</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F46">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D46,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G46">
+        <f>ROUND(F46*INDEX('01_Criteria'!$F:$F,MATCH(C46,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000045 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3507,7 +3744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4056,6 +4293,80 @@
       <c r="G15" t="inlineStr">
         <is>
           <t>Coverage now 47% (8 of 20 weighted criteria). Volvo EX30 P8 AWD scored lowest on this criterion - its price premium goes toward performance (0-100 time), which the framework explicitly excludes as a meaningful ownership factor, so that premium is not counted as good value here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DEC_M002_VIOLATION</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CRITICAL: Discovered Tesla Model 3 fails Hard Requirement M002 (length 4720mm &gt; 4500mm limit) - all 4 configurations affected</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>While scoring Garasje (W019), cross-checked recorded vehicle lengths against the M002 hard requirement for the first time this session. Tesla Model 3 length (4720mm, sourced from Tesla's own official page early in the session) exceeds the 4500mm maximum by 220mm. Per docs/02_criteria-and-weighting.md, failing configurations should not proceed to weighted evaluation - yet TESLA_MODEL_3_LONG_RANGE_RWD has been scored on 8 criteria throughout this session.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Per user direction: all 4 Tesla configurations kept in 03_Configurations and the comparison, but explicitly flagged in both Configuration Notes and 12_OverallScores.Notes as hard-requirement non-compliant. No Score/Review rows were deleted or altered - existing history remains intact and traceable. User will personally weigh the 220mm overage rather than have it silently resolved. This is a process gap worth addressing going forward: Hard Requirements should be checked before, not after, weighted scoring begins for a new vehicle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DEC_W019_SCORE</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Scored Garasje (W019, weight 3) for all 5 configurations - purely computed from Length margin vs 4500mm</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Deterministic scoring based on official Length figures already gathered (or newly sourced for Kia EV2: 4065mm from official Kia UK spec PDF). Rubric: &gt;=400mm margin=5, 250-399mm=4, 100-249mm=3, 1-99mm=2, &lt;=0mm(over limit)=1.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>This is what surfaced the Tesla M002 violation (see DEC_M002_VIOLATION) - Tesla scored 1/5 since it EXCEEDS the limit, not just has minimal margin. Skoda scored only 2/5 despite passing M002, since its 12mm margin is negligible in practice. Kia scored 5/5 with the largest margin (435mm) of the five.</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4470,7 @@
         <v/>
       </c>
       <c r="H2">
-        <f>IF(E2&lt;100,"Partial evaluation - "&amp;F2&amp;" of "&amp;G2&amp;" WEIGHTED+Active criteria scored ("&amp;E2&amp;"% of total weight).","Complete evaluation - all WEIGHTED+Active criteria scored.")</f>
+        <f>"HARD REQUIREMENT FAILED (M002: length 4720mm &gt; 4500mm) - NOT ELIGIBLE, kept only for user comparison. "&amp;IF(E2&lt;100,"Partial evaluation - "&amp;F2&amp;" of "&amp;G2&amp;" WEIGHTED+Active criteria scored ("&amp;E2&amp;"% of total weight).","Complete evaluation - all WEIGHTED+Active criteria scored.")</f>
         <v/>
       </c>
     </row>
@@ -6109,7 +6420,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002).</t>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002). HARD REQUIREMENT FAILED (M002): Official length is 4720mm, 220mm over the 4500mm maximum. Per docs/02_criteria-and-weighting.md, "Configurations failing a mandatory requirement shall not proceed to weighted evaluation." This was not caught until the length figure was cross-checked against M002 during Garasje (W019) scoring. Kept in the comparison table at the users explicit request so they can personally weigh the 220mm overage, but this configuration is NOT hard-requirement-compliant and all its existing Reviews/Scores/OverallScore should be read with that in mind.</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6452,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002).</t>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002). HARD REQUIREMENT FAILED (M002): Official length is 4720mm, 220mm over the 4500mm maximum. Per docs/02_criteria-and-weighting.md, "Configurations failing a mandatory requirement shall not proceed to weighted evaluation." This was not caught until the length figure was cross-checked against M002 during Garasje (W019) scoring. Kept in the comparison table at the users explicit request so they can personally weigh the 220mm overage, but this configuration is NOT hard-requirement-compliant and all its existing Reviews/Scores/OverallScore should be read with that in mind.</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6490,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002). M003 (winter highway range): Not verified. Two winter tests were found but both are unreliable matches: a 2022 test used a superseded pre-refresh Model 3 generation with a WLTP figure (614km) that matches no current trim, and a NAF winter 2025 test reports 702km WLTP (matching none of this workbook's four recorded Model 3 configurations) without specifying which trim was tested. Remains genuinely Unknown. Price verified 2026-07-06 via official Tesla Norway configurator (SRC_TESLA_NO_MODEL3_DESIGN): 400539 kr incl. VAT/fees, no optional extras selected (previously unpriced under DATA-001).</t>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002). M003 (winter highway range): Not verified. Two winter tests were found but both are unreliable matches: a 2022 test used a superseded pre-refresh Model 3 generation with a WLTP figure (614km) that matches no current trim, and a NAF winter 2025 test reports 702km WLTP (matching none of this workbook's four recorded Model 3 configurations) without specifying which trim was tested. Remains genuinely Unknown. Price verified 2026-07-06 via official Tesla Norway configurator (SRC_TESLA_NO_MODEL3_DESIGN): 400539 kr incl. VAT/fees, no optional extras selected (previously unpriced under DATA-001). HARD REQUIREMENT FAILED (M002): Official length is 4720mm, 220mm over the 4500mm maximum. Per docs/02_criteria-and-weighting.md, "Configurations failing a mandatory requirement shall not proceed to weighted evaluation." This was not caught until the length figure was cross-checked against M002 during Garasje (W019) scoring. Kept in the comparison table at the users explicit request so they can personally weigh the 220mm overage, but this configuration is NOT hard-requirement-compliant and all its existing Reviews/Scores/OverallScore should be read with that in mind.</t>
         </is>
       </c>
     </row>
@@ -6211,7 +6522,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002).</t>
+          <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002). HARD REQUIREMENT FAILED (M002): Official length is 4720mm, 220mm over the 4500mm maximum. Per docs/02_criteria-and-weighting.md, "Configurations failing a mandatory requirement shall not proceed to weighted evaluation." This was not caught until the length figure was cross-checked against M002 during Garasje (W019) scoring. Kept in the comparison table at the users explicit request so they can personally weigh the 220mm overage, but this configuration is NOT hard-requirement-compliant and all its existing Reviews/Scores/OverallScore should be read with that in mind.</t>
         </is>
       </c>
     </row>
@@ -6767,7 +7078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -13396,6 +13707,51 @@
         </is>
       </c>
       <c r="J150" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>TECH_000144</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Length</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>4065</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>SRC_KIA_UK_SPECS_PDF</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -15748,7 +16104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -17404,6 +17760,206 @@
         </is>
       </c>
       <c r="I41" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>REV_000041</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Garasje</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Lengde 4720mm OVERSKRIDER 4500mm-grensen med 220mm. Denne konfigurasjonen oppfyller ikke engang minstekravet (M002), langt mindre gir den margin utover det. Laveste mulige score, og et symptom pa at denne konfigurasjonen ikke skulle vaert vektet evaluert i utgangspunktet (se DecisionLog DEC_M002_VIOLATION). [Kriterium W019]</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>EV_000053</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>REV_000042</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Garasje</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Lengde 4140mm gir 360mm margin under 4500mm-grensen - en komfortabel margin, i tradisjonens andre halvdel av utvalget. [Kriterium W019]</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>EV_000054</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>REV_000043</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Garasje</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Lengde 4488mm gir kun 12mm margin under 4500mm-grensen - den klart minste marginen i utvalget, og i praksis neglisjerbar. [Kriterium W019]</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>EV_000055</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>REV_000044</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Garasje</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>4</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Lengde 4233mm gir 267mm margin under 4500mm-grensen - komfortabel margin. [Kriterium W019]</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>EV_000056</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>REV_000045</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Garasje</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Lengde 4065mm gir 435mm margin under 4500mm-grensen - storst margin av alle fem, og eneste konfigurasjon med over 400mm margin. [Kriterium W019]</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>EV_000057</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -17426,7 +17982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -18875,6 +19431,141 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>EV_000053</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Garage length margin: official length 4720mm EXCEEDS the 4500mm hard-requirement maximum by 220mm - this configuration does not meet the minimum requirement, let alone have margin beyond it.</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>EV_000054</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Garage length margin: official length 4140mm, giving a 360mm margin below the 4500mm hard-requirement maximum.</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PAGE</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>EV_000055</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Garage length margin: official length 4488mm, giving a 12mm margin below the 4500mm hard-requirement maximum.</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_GLOBAL_TECHDATA</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>EV_000056</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Garage length margin: official length 4233mm, giving a 267mm margin below the 4500mm hard-requirement maximum.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>SRC_VOLVO_NO_EX30_SPECS</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>EV_000057</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Garage length margin: official length 4065mm, giving a 435mm margin below the 4500mm hard-requirement maximum.</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>SRC_KIA_UK_SPECS_PDF</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Volvo EX30 P8 AWD on W008 (Førerassistenter kvalitet)
Reuses existing Motor.no evidence (EV_000036) on ACC winter-driving
issues, previously only linked to the W005 infotainment review, to
add REV_000046 / SCORE_000047.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -1877,7 +1877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3729,6 +3729,46 @@
       <c r="H46" t="inlineStr">
         <is>
           <t>Traceable to REV_000045 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SCORE_000047</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>W008</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>REV_000046</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F47">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D47,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G47">
+        <f>ROUND(F47*INDEX('01_Criteria'!$F:$F,MATCH(C47,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000046 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -16104,7 +16144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -17960,6 +18000,46 @@
         </is>
       </c>
       <c r="I46" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>REV_000046</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Motor.no: ACC beskrives som "lunefull på norske vinterveier" - å justere hastighet/intervall "viste seg i praksis umulig" under vinterkjøring. Isolert praktisk svakhet ved førerassistanse i norske vinterforhold under spesifikke forhold, ikke en total systemsvikt. [Kriterium W008]</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>EV_000036</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>

</xml_diff>

<commit_message>
Score Tesla Model 3 LR RWD on W006, W008, W009
W006 (OTA): self-verified on Tesla's Norwegian configurator that
Autosteer is now paywalled behind the FSD subscription, corroborated
by Electrek's Jan/May 2026 coverage of the EU rollout - scored 3/5,
strong OTA delivery undercut by feature-paywalling risk.

W008 (driver-assist quality): no independent Norwegian/Nordic winter
test of standard Autopilot exists; scored 3/5 at LOW confidence with
the evidence gap explicitly flagged in the review rather than left
silently unscored.

W009 (camera): Tesla's own owner's manual confirms rear + side camera
views only, no stitched 360-degree composite - scored 2/5.

Adds supporting Equipment rows (ACC standard, lane-centering optional/
paywalled, rear camera standard, 360 unavailable, OTA standard) and
four new Sources (Tesla owner's manual, Tesla winter driving tips,
Electrek, elbilforum.no).
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1857,6 +1857,159 @@
       <c r="H27" t="inlineStr">
         <is>
           <t>Official Kia UK specifications PDF. GT Line/GT Line S trim: Length 4065mm, Wheelbase 2565mm, Width 1800mm, Height 1585mm. UK market document, not Norway-specific, but physical dimensions are not expected to differ by market for the same generation/trim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_OWNERSMANUAL_MODEL3_NO</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Tesla Model 3 Owner's Manual (Norwegian)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://www.tesla.com/ownersmanual/model3/no_no/GUID-3598EF55-6B1D-462B-88D8-704DB0896DD1.html</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Official Tesla owner's manual, camera/parking section. Confirms rear-view camera plus side-pillar camera views, no stitched 360-degree/bird's-eye composite view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SRC_ELECTREK_TESLA_AUTOPILOT_PAYWALL</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Tesla cuts standard Autopilot, paywalls basic safety feature behind FSD subscription</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Electrek</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://electrek.co/2026/01/23/tesla-cuts-standard-autopilot-paywalls-basic-safety-feature-behind-fsd-subscription/</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Reports Tesla removing 'Basic Autopilot' (TACC+Autosteer bundle) from new North American orders in Jan 2026, later expanded to EU markets (Netherlands May 2026; one-time FSD purchase deadline May 21 2026 per follow-up Electrek coverage). Corroborates the paywall pattern later self-verified on Tesla's own Norwegian configurator (SRC_TESLA_NO_MODEL3_DESIGN).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_WINTER_DRIVING_TIPS</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Winter driving tips</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://www.tesla.com/support/winter-driving-tips</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Official Tesla guidance warning that Traffic-Aware Cruise Control/Autopilot should not be used on icy or slippery road surfaces. Generic safety boilerplate, not Norway-specific or comparative to other manufacturers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SRC_ELBILFORUM_MODEL3_AUTOPILOT_WINTER</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>COMMUNITY</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Model 3 Autopilot på norske vinterveier - brukertråd</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>elbilforum.no</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://elbilforum.no/</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Anecdotal, mixed user reports on standard Autopilot/TACC behavior on Norwegian winter roads - some describe it as reliable in winter conditions, others report late reactions on icy side roads. Forum anecdote only, not editorial/independent testing.</t>
         </is>
       </c>
     </row>
@@ -1877,7 +2030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3769,6 +3922,126 @@
       <c r="H47" t="inlineStr">
         <is>
           <t>Traceable to REV_000046 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SCORE_000048</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>W006</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>REV_000047</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F48">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D48,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G48">
+        <f>ROUND(F48*INDEX('01_Criteria'!$F:$F,MATCH(C48,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000047 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SCORE_000049</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>W008</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>REV_000048</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F49">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D49,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G49">
+        <f>ROUND(F49*INDEX('01_Criteria'!$F:$F,MATCH(C49,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000048 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SCORE_000050</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>W009</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>REV_000049</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F50">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D50,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G50">
+        <f>ROUND(F50*INDEX('01_Criteria'!$F:$F,MATCH(C50,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000049 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -13817,7 +14090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -15521,6 +15794,166 @@
       <c r="F53" t="inlineStr">
         <is>
           <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>EQ_000053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_DESIGN</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>EQ_000054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>EQ_LANE_CENTER</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_DESIGN</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>EQ_000055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_OWNERSMANUAL_MODEL3_NO</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>EQ_000056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>EQ_360</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_OWNERSMANUAL_MODEL3_NO</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>EQ_000057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>EQ_OTA</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>SRC_ELECTREK_TESLA_AUTOPILOT_PAYWALL</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -16144,7 +16577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -18040,6 +18473,126 @@
         </is>
       </c>
       <c r="I47" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>REV_000047</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Tesla leverer hyppige og reelle OTA-oppdateringer, men et dokumentert og nå Norge-bekreftet mønster av å flytte tidligere inkluderte førerassistanse-funksjoner (Autostyring) bak et betalt abonnement svekker forutsigbarheten for et 8-10-års eierskap. Sterk oppdateringsmotor, men fremtidssikringen er ikke garantert gratis. [Kriterium W006]</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>EV_000058,EV_000059</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>REV_000048</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Ingen uavhengig norsk/nordisk test av standard Autopilot/TACC sin kvalitet på vinterforhold ble funnet - kun generisk produsentadvarsel og sprikende anekdotiske brukerrapporter. Score satt nøytralt grunnet reell kunnskapsmangel, ikke grunnet bekreftet gjennomsnittlig ytelse; bør revurderes hvis en dedikert test dukker opp. [Kriterium W008]</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>EV_000060,EV_000061</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>REV_000049</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>2</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Tesla sin egen brukermanual bekrefter kun ryggekamera og sidekameraer - ingen sammenstilt 360-graders visning. Fungerende grunnleggende parkeringskamera, men mangler den spesifikke 360-verdien kriteriet fremhever. [Kriterium W009]</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>EV_000062</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -18062,7 +18615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -19646,6 +20199,141 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>EV_000058</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>OTA/fremtidssikring: Tesla sin egen norske konfigurator (selv-verifisert 2026-07-06) viser at Autostyring (Autosteer) nå kun er tilgjengelig i det betalte tillegget 'Fremtidig selvkjørende funksjoner' (1090 kr/mnd eller engangskjøp) - ikke som standardutstyr. Trafikkoppmerksom cruisekontroll (TACC) forblir standard.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_DESIGN</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>EV_000059</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>OTA/fremtidssikring: Electrek rapporterer at Tesla fjernet gratis 'Basic Autopilot' (TACC+Autosteer) fra nye Nord-Amerika-bestillinger 23. januar 2026, og utvidet dette til EU-markeder (Nederland mai 2026, med frist 21. mai 2026 for engangskjøp av FSD i øvrige europeiske markeder). Bekrefter et gjentakende mønster av å legge tidligere inkluderte funksjoner bak abonnement.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>SRC_ELECTREK_TESLA_AUTOPILOT_PAYWALL</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>EV_000060</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Førerassistenter kvalitet: Tesla sin egen support-side advarer om at Trafikkoppmerksom cruisekontroll/Autopilot ikke bør brukes på isete eller glatte veier. Generisk sikkerhetsdisclaimer, ikke Norge-spesifikk eller sammenlignende.</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_WINTER_DRIVING_TIPS</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>EV_000061</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Førerassistenter kvalitet: Anekdotiske og sprikende brukerrapporter fra elbilforum.no om standard Autopilot/TACC på norske vinterveier - noen beskriver systemet som pålitelig i vinterforhold, andre rapporterer sen reaksjon på glatte sideveier. Ingen redaksjonell eller uavhengig test funnet.</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>SRC_ELBILFORUM_MODEL3_AUTOPILOT_WINTER</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>EV_000062</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Kamera/parkering: Tesla sin offisielle norske brukermanual bekrefter ryggekamera pluss sidekameraer (B-stolpe), men ingen sammenstilt 360-graders/fugleperspektiv-visning. Direkte sitat: 'Model 3 har et ryggekamera... Model 3 viser også bilder fra sidekameraene (hvis utstyrt).'</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_OWNERSMANUAL_MODEL3_NO</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Renault 4 Techno on W006, W008, W009
W006 (OTA): Renault Group confirms FOTA capability via embedded 4G;
electrive.com corroborates a real shipped update (Google Gemini AI,
June 2026), no workshop visit needed - scored 4/5.

W008 (driver-assist quality): elbil.no's Norwegian test confirms ACC
"works surprisingly well on the motorway" on Techno/Iconic trims -
scored 4/5, brief mention rather than a deep winter test.

W009 (camera): elbil.no confirms the 360-degree camera and auto-park
are Iconic-exclusive (+20,000 kr); Techno gets rear camera + front
sensors only - scored 2/5, consistent with Tesla's treatment.

Adds EQ_OTA equipment row and two new Sources (Renault Group FOTA
article, electrive.com); reuses existing SRC_ELBIL_RENAULT4_TEST for
W008/W009.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2010,6 +2010,85 @@
       <c r="H31" t="inlineStr">
         <is>
           <t>Anecdotal, mixed user reports on standard Autopilot/TACC behavior on Norwegian winter roads - some describe it as reliable in winter conditions, others report late reactions on icy side roads. Forum anecdote only, not editorial/independent testing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_GROUP_FOTA</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>FOTA: updates are in the air</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Renault Group</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://www.renaultgroup.com/en/magazine/our-group-news/fota-updates-are-in-the-air/</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Official Renault Group article confirming Firmware-Over-The-Air (FOTA) update capability via embedded 4G, no workshop visit required. Applies to OpenR Link-equipped models including Renault 4 E-Tech.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SRC_ELECTRIVE_RENAULT_GEMINI_OTA</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Renault introduces Google Gemini via OTA update</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>electrive.com</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://www.electrive.com/2026/07/03/renault-introduces-google-gemini-via-ota-update/</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Independent corroboration of a real, dated shipped OTA update: Google Gemini AI assistant rolled out free to all OpenR Link-equipped models starting mid-June 2026, no workshop visit required.</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4042,6 +4121,126 @@
       <c r="H50" t="inlineStr">
         <is>
           <t>Traceable to REV_000049 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SCORE_000051</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>W006</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>REV_000050</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F51">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D51,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G51">
+        <f>ROUND(F51*INDEX('01_Criteria'!$F:$F,MATCH(C51,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000050 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SCORE_000052</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>W008</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>REV_000051</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F52">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D52,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G52">
+        <f>ROUND(F52*INDEX('01_Criteria'!$F:$F,MATCH(C52,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000051 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SCORE_000053</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>W009</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>REV_000052</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F53">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D53,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G53">
+        <f>ROUND(F53*INDEX('01_Criteria'!$F:$F,MATCH(C53,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000052 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -14090,7 +14289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -15952,6 +16151,38 @@
         </is>
       </c>
       <c r="F58" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>EQ_000058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>EQ_OTA</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_GROUP_FOTA</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -16577,7 +16808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -18593,6 +18824,126 @@
         </is>
       </c>
       <c r="I50" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>REV_000050</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Renault leverer bekreftet FOTA-kapasitet og har allerede sendt en reell, datert oppdatering (Google Gemini AI, juni 2026) uten verkstedbesok. Ingen tegn til betalingsmur eller fjerning av funksjoner, i motsetning til enkelte konkurrenter. [Kriterium W006]</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>EV_000063,EV_000064</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>REV_000051</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>4</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>elbil.no sin norske test gir en positiv, direkte vurdering av adaptiv cruise control - 'fungerer overraskende greit pa motorvei.' Kort omtale fremfor en dyptgaende vinterspesifikk test, men et reelt norsk testverdikt. [Kriterium W008]</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>EV_000065</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>REV_000052</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>2</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Techno-trimmet far kun ryggekamera og parkeringssensorer foran - 360-graders kamera og automatisk parkering er reservert Iconic-varianten (+20 000 kr). Fungerende grunnutstyr, men mangler den spesifikke 360-verdien kriteriet fremhever. [Kriterium W009]</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>EV_000066</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -18615,7 +18966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -20334,6 +20685,114 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>EV_000063</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>OTA/fremtidssikring: Renault Group bekrefter FOTA (Firmware-Over-The-Air) via innebygd 4G-tilkobling, uten behov for verkstedbesok. Gjelder OpenR Link-utstyrte modeller, inkludert Renault 4 E-Tech.</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_GROUP_FOTA</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>EV_000064</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>OTA/fremtidssikring: electrive.com bekrefter et reelt, datert OTA-levert oppdatering - Google Gemini AI-assistent ble rullet ut gratis til alle OpenR Link-utstyrte modeller fra medio juni 2026, uten behov for verkstedbesok.</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>SRC_ELECTRIVE_RENAULT_GEMINI_OTA</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>EV_000065</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Forerassistenter kvalitet: elbil.no sin norske test bekrefter adaptiv cruise control er standard pa Techno (og Iconic), og at den fungerer 'overraskende greit pa motorvei'. Kort omtale, ikke en dyptgaende vintertest.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_RENAULT4_TEST</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>EV_000066</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Kamera/parkering: elbil.no bekrefter at 360-graders kamera og automatisk parkering kun finnes pa Iconic-varianten (+20 000 kr over Techno). Techno far ryggekamera og parkeringssensorer foran, men ingen 360-visning.</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_RENAULT4_TEST</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Skoda Elroq Selection 60 on W006, W008, W009
W006 (OTA): MEB/CARIAD platform supports OTA and has matured past the
early ID.3/ID.4 software problems, but per CarExpert's review of the
equivalent export-market trim, OTA is tied to a Connected Services
subscription not standard on this trim - scored 3/5, single-source
and not Norway-specific so confidence is MEDIUM.

W008 (driver-assist quality): consistently praised across independent
European reviews as "highly competent," compared favorably to
Mercedes Distronic Plus; general positive Norwegian endorsement
(elbil.no) too, but no dedicated winter-specific test - scored 4/5.

W009 (camera): rear-view camera only standard on Selection 60;
360-degree Area View gated to higher trims/packages - scored 2/5,
consistent with Tesla/Renault's treatment.

Adds two new Sources (CarExpert, elbil.no Elroq test) and EQ_OTA/
EQ_360 equipment rows.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2089,6 +2089,85 @@
       <c r="H33" t="inlineStr">
         <is>
           <t>Independent corroboration of a real, dated shipped OTA update: Google Gemini AI assistant rolled out free to all OpenR Link-equipped models starting mid-June 2026, no workshop visit required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SRC_CAREXPERT_ELROQ_60SELECT</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026 Skoda Elroq 60 Select review (quick drive)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>CarExpert</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://www.carexpert.com.au/car-reviews/2026-skoda-elroq-60-select-review-quick-drive</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Review of the '60 Select' trim, the closest export-market analog to the Norwegian Selection 60. Confirms Connected Services (incl. OTA updates) is not standard on this trim, praises Travel Assist/ACC quality, and confirms rear-view-only camera as standard with 360-degree Area View reserved for higher trims/packages. Not Norway-specific.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_ELROQ_TEST</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Test av Skoda Elroq</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Norsk elbilforening (elbil.no)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://elbil.no/</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Norwegian test of the Skoda Elroq 60. Brief general endorsement of driver-assist systems ('holder orden i sysakene hvis du blir overivrig') - no dedicated winter-specific ACC deep-dive.</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4241,6 +4320,126 @@
       <c r="H53" t="inlineStr">
         <is>
           <t>Traceable to REV_000052 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SCORE_000054</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>W006</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>REV_000053</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F54">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D54,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G54">
+        <f>ROUND(F54*INDEX('01_Criteria'!$F:$F,MATCH(C54,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000053 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SCORE_000055</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>W008</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>REV_000054</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F55">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D55,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G55">
+        <f>ROUND(F55*INDEX('01_Criteria'!$F:$F,MATCH(C55,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000054 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SCORE_000056</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>W009</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>REV_000055</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F56">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D56,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G56">
+        <f>ROUND(F56*INDEX('01_Criteria'!$F:$F,MATCH(C56,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000055 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -14289,7 +14488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16183,6 +16382,70 @@
         </is>
       </c>
       <c r="F59" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>EQ_000059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>EQ_OTA</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>SRC_CAREXPERT_ELROQ_60SELECT</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>EQ_000060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>EQ_360</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>SRC_CAREXPERT_ELROQ_60SELECT</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -16808,7 +17071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -18944,6 +19207,126 @@
         </is>
       </c>
       <c r="I53" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>REV_000053</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>3</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>MEB/CARIAD-plattformen støtter OTA og har modnet betydelig siden tidlige ID.3/ID.4-problemer, men Connected Services (som OTA inngår i) er ikke standard på denne trimmen ifølge en eksportmarked-gjennomgang - ikke Norge-spesifikk kilde. [Kriterium W006]</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>EV_000067</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>REV_000054</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>4</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Gjennomgående positiv omtale av Travel Assist/adaptiv cruise control i flere uavhengige europeiske tester ('highly competent', bedre finjustert enn Mercedes Distronic Plus), understøttet av en generell positiv norsk omtale (elbil.no). Ingen dedikert vinterspesifikk test funnet. [Kriterium W008]</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>EV_000068,EV_000069</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>REV_000055</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>2</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Selection 60 får kun ryggekamera som standard - 360-graders Area View er reservert høyere trimmer/pakker. Fungerende grunnutstyr, men mangler den spesifikke 360-verdien kriteriet fremhever, i tråd med Tesla og Renault sin vurdering. [Kriterium W009]</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>EV_000070</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -18966,7 +19349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -20793,6 +21176,114 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>EV_000067</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>OTA/fremtidssikring: CarExpert sin gjennomgang av '60 Select' (nærmeste eksportmarked-ekvivalent til norske Selection 60) bekrefter at Connected Services - som inkluderer OTA-oppdateringer - ikke er standard på denne trimmen. MEB/CARIAD-plattformen har for øvrig modnet betydelig siden de tidlige ID.3/ID.4-problemene.</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>SRC_CAREXPERT_ELROQ_60SELECT</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>EV_000068</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Førerassistenter kvalitet: CarExpert beskriver Predictive Adaptive Cruise Control/Travel Assist som 'highly competent' og kalibrert til å være hjelpsom uten å være påtrengende. Andre uavhengige europeiske tester (aggregert) beskriver systemet som mer finjustert enn Mercedes' Distronic Plus.</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>SRC_CAREXPERT_ELROQ_60SELECT</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>EV_000069</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Førerassistenter kvalitet: elbil.no sin norske test gir en generell positiv omtale av kjøreassistentene ('holder orden i sysakene hvis du blir overivrig'), men uten en dyptgående vinterspesifikk vurdering av adaptiv cruise control.</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_ELROQ_TEST</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>EV_000070</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Kamera/parkering: CarExpert bekrefter at Selection/60 Select-trimmen kun får ryggekamera som standard - 360-graders Area View er reservert høyere trimmer/pakker (f.eks. '130 Years Edition').</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>SRC_CAREXPERT_ELROQ_60SELECT</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Volvo EX30 P8 AWD on W006 and W009
W006 (OTA): Volvo delivered "the largest OTA update in history" across
~2.5M vehicles reworking the UX, with Gemini AI planned via a future
OTA - but the EX30 also launched with severe software bugs (black
screens, keyless-entry failures, reported power loss) serious enough
to trigger UK consumer-rights returns, taking roughly a year of OTA
patching to resolve - scored 3/5.

W009 (camera): verified this specific configuration (Twin Performance
AWD, 468,900 kr) is Plus trim, not Ultra - the 360-degree camera/Park
Pilot is Ultra-exclusive (~505,900 kr for the same powertrain) -
scored 2/5, consistent with Tesla/Renault/Skoda's treatment.

Adds four new Sources (WardsAuto, InsideEVs, elbil.no trim test,
Frydenbo dealer comparison) and EQ_OTA/EQ_360 equipment rows.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2168,6 +2168,154 @@
       <c r="H35" t="inlineStr">
         <is>
           <t>Norwegian test of the Skoda Elroq 60. Brief general endorsement of driver-assist systems ('holder orden i sysakene hvis du blir overivrig') - no dedicated winter-specific ACC deep-dive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SRC_WARDSAUTO_VOLVO_OTA</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Volvo Delivers Biggest OTA Software Update in Company History</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>WardsAuto</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://www.wardsauto.com/news/volvo-biggest-ota-update-software-comapny-history-google-maps-android-automotive-os/813588/</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Reports Volvo pushed its largest-ever OTA update to ~2.5 million vehicles (EX30 included), reworking the UX, with Google Gemini-based conversational AI planned via a further OTA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SRC_INSIDEEVS_VOLVO_EX30_BUGS</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Volvo EX30 launch software issues</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>InsideEVs</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://insideevs.com/news/785621/volvo-ex60-launch-issues/</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Reports the EX30 launched with severe software bugs (black screens, keyless-entry failures, reported power loss), serious enough that UK customers exercised consumer-rights returns; Volvo spent roughly a year patching issues via OTA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_VOLVO_EX30_TRIM</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Prøvekjøring av Volvo EX30</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Norsk elbilforening (elbil.no)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://elbil.no/provekjoring-av-volvo-ex30/</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Confirms 360-degree camera, automatic parking assist, panoramic roof, and powered seats/lumbar are Ultra-trim-exclusive, not included on Plus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SRC_FRYDENBO_VOLVO_EX30_TRIMCOMPARE</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Volvo EX30 trim level comparison</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Frydenbø (Volvo dealer, Norway)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://www.frydenbo.no/</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Independently corroborates that at the Twin Performance AWD powertrain, Plus trim (468,900 NOK) excludes the 360-degree camera/Park Pilot, which is only added at Ultra trim (~505,900 NOK) for the same powertrain.</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4440,6 +4588,86 @@
       <c r="H56" t="inlineStr">
         <is>
           <t>Traceable to REV_000055 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SCORE_000057</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>W006</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>REV_000056</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F57">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D57,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G57">
+        <f>ROUND(F57*INDEX('01_Criteria'!$F:$F,MATCH(C57,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000056 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>SCORE_000058</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>W009</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>REV_000057</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F58">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D58,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G58">
+        <f>ROUND(F58*INDEX('01_Criteria'!$F:$F,MATCH(C58,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000057 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -14488,7 +14716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16446,6 +16674,70 @@
         </is>
       </c>
       <c r="F61" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>EQ_000061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>EQ_OTA</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>SRC_WARDSAUTO_VOLVO_OTA</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>EQ_000062</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>EQ_360</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_VOLVO_EX30_TRIM</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -17071,7 +17363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -19327,6 +19619,86 @@
         </is>
       </c>
       <c r="I56" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>REV_000056</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>3</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Volvo har levert en reelt substansiell OTA-oppdatering (største i selskapets historie, ~2,5 mill. biler) og planlegger Gemini-AI via fremtidig OTA - men EX30 lanserte med alvorlige programvarefeil (sorte skjermer, nøkkelfri-svikt, rapportert strømtap) alvorlig nok til å utløse forbrukerrettighetsreturer i Storbritannia, og det tok omtrent et år å rette dette via OTA. Reell leveringsevne, men reell kvalitetsrisiko ved lansering. [Kriterium W006]</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>EV_000071,EV_000072</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>REV_000057</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>2</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Denne konfigurasjonen (Twin Performance AWD, 468 900 kr) er Plus-utstyrsnivå, ikke Ultra - 360-graders kamera og automatisk parkeringsassistent er forbeholdt Ultra (ca. 505 900 kr for samme drivlinje). Mangler den spesifikke 360-verdien kriteriet fremhever, i tråd med Tesla, Renault og Skoda sin vurdering. [Kriterium W009]</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>EV_000073</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -19349,7 +19721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -21284,6 +21656,87 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>EV_000071</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>OTA/fremtidssikring: WardsAuto rapporterer at Volvo sendte den største OTA-oppdateringen i selskapets historie til ca. 2,5 millioner biler (inkludert EX30), med omfattende UX-omarbeiding, og at Google Gemini-basert samtale-AI er planlagt via en fremtidig OTA.</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>SRC_WARDSAUTO_VOLVO_OTA</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>EV_000072</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>OTA/fremtidssikring: InsideEVs rapporterer at EX30 ble lansert med alvorlige programvarefeil (sorte skjermer, feil på nøkkelfri adgang, rapportert strømtap), alvorlig nok til at britiske kunder benyttet seg av forbrukerrettigheter for å returnere bilen. Volvo brukte omtrent et år på å rette feil via OTA.</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>SRC_INSIDEEVS_VOLVO_EX30_BUGS</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>EV_000073</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Kamera/parkering: elbil.no bekrefter at 360-graders kamera og automatisk parkeringsassistent er forbeholdt Ultra-utstyrsnivå - ikke inkludert på Plus. Uavhengig bekreftet av Frydenbø sin trimnivå-sammenligning: samme drivlinje (Twin Performance AWD) til 468 900 kr er Plus uten 360-kamera, mens Ultra (ca. 505 900 kr) inkluderer det.</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_VOLVO_EX30_TRIM</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Tesla Model 3 LR RWD on W014, W015
W014 (produsent-/modellrisiko): Model 3 var Norges mest solgte
bilmodell i 2020 og 2021, og over 60 000 eksemplarer er registrert i
Norge i dag - klart lengst og mest dokumentert sporhistorikk av de
fem konfigurasjonene. Scoret 5/5.

W015 (garanti/serviceapparat): Tesla oppgir 4 års/80 000 km generell
garanti - kortest av de fem - pluss 8 års batterigaranti (minst 70 %
kapasitet) og 12 års rustgaranti. Serviceapparatet er også strukturelt
annerledes (fåtall faste servicesentre + mobil service, ikke
tradisjonelt forhandlernett). Scoret 3/5: solide batterivilkår, men
svakest generell garanti og tynnere fysisk serviceapparat.

Legger til to nye kilder (Tesla garantiside, NRK/ITavisen om
salgshistorikk).
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2553,6 +2553,80 @@
       <c r="H45" t="inlineStr">
         <is>
           <t>EV2-specific Danish test. Notes the adaptive cruise/lane-assist system 'holder usædvanligt hårdt i rattet' (holds unusually firmly on the wheel), requiring deliberate steering input to override - an over-intervention complaint, not a performance failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_WARRANTY</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Bilgaranti | Tesla-støtte Norge</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://www.tesla.com/no_no/support/vehicle-warranty</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Official Tesla Norway warranty page. Direct fetch returned HTTP 403; terms corroborated via search-result synthesis (4 års/80 000 km generell nybilgaranti, 8 års batterigaranti med garantert minst 70 % kapasitet, 12 års rustgjennomtæringsgaranti uten kilometergrense). Bør verifiseres direkte ved behov for presisjon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_MODEL3_NO_SALES_HISTORY</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Rekordår i salg av nye biler: Tesla er Norges mest solgte bil</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>NRK / ITavisen (basert på OFV-tall)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://www.nrk.no/norge/rekordar-i-salg-av-nye-biler_-tesla-er-norges-mest-solgte-bil-1.15793772</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Nyhetsdekning av offisiell registreringsstatistikk fra OFV (Opplysningsrådet for Veitrafikken). Model 3 var Norges mest solgte bilmodell i 2020 og 2021 (over 12 000 solgte i 2021 alene), og over 60 000 eksemplarer er i dag registrert i Norge; OFV-tall for november 2025 viser 2 562 nyregistrerte Model 3 i den ene måneden alene.</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5025,6 +5099,86 @@
       <c r="H61" t="inlineStr">
         <is>
           <t>Traceable to REV_000060 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>SCORE_000062</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>W014</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>REV_000061</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F62">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D62,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G62">
+        <f>ROUND(F62*INDEX('01_Criteria'!$F:$F,MATCH(C62,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000061 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>SCORE_000063</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>W015</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>REV_000062</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F63">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D63,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G63">
+        <f>ROUND(F63*INDEX('01_Criteria'!$F:$F,MATCH(C63,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000062 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -17720,7 +17874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -20176,6 +20330,86 @@
         </is>
       </c>
       <c r="I61" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>REV_000061</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>5</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Model 3 har vært Norges mest solgte bilmodell i flere år (2020 og 2021, med over 12 000 solgte i 2021 alene), og over 60 000 eksemplarer ruller på norske skilter i dag - den desidert lengste og mest dokumenterte sporhistorikken av de fem konfigurasjonene. Både produsent og modell fremstår som lavest mulig risiko i denne sammenligningen. [Kriterium W014]</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>EV_000081</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>REV_000062</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>3</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Tesla tilbyr 4 års/80 000 km generell nybilgaranti - kortest av de fem konfigurasjonene - samt 8 års batterigaranti (minst 70 % kapasitet) og 12 års rustgaranti uten kilometergrense. Serviceapparatet er også strukturelt annerledes enn de øvrige: færre faste servicesentre (Bærum og Oslo), supplert med mobil service fremfor et tradisjonelt forhandlernett. Solide batterivilkår, men svakest generell garanti og et tynnere fysisk serviceapparat enn konkurrentene. [Kriterium W015]</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>EV_000082</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -20198,7 +20432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -22403,6 +22637,60 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>EV_000081</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Modellrisiko: Tesla Model 3 var Norges mest solgte bilmodell i 2020 og 2021 (over 12 000 solgte i 2021), og over 60 000 eksemplarer er i dag registrert på norske skilter. Ifølge OFV ble det registrert 2 562 nye Model 3 i november 2025 alene.</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_MODEL3_NO_SALES_HISTORY</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>EV_000082</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Garanti: Tesla oppgir 4 års/80 000 km generell nybilgaranti, 8 års batterigaranti (minst 70 % kapasitet beholdt) og 12 års rustgjennomtæringsgaranti uten kilometergrense. Serviceapparatet i Norge er strukturert rundt et fåtall faste servicesentre (Bærum, Oslo) supplert med mobil service, ikke et tradisjonelt forhandlernett.</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_WARRANTY</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Renault 4 Techno on W014, W015
W014 (produsent-/modellrisiko): 4 E-Tech er tilgjengelig i Norge fra
høsten 2025 - under ett år på markedet ved vurderingstidspunktet, på
en helt ny plattform (AmpR Small) uten egen lang sporhistorikk.
Produsenten selv er langt fra ny, men konfigurasjonens ferskhet
tilsier en forsiktig middels vurdering. Scoret 3/5.

W015 (garanti/serviceapparat): Renault innførte fra mai 2025 5
år/150 000 km generell garanti på alle nye elbiler, pluss 8 år/
160 000 km batterigaranti (minst 70 % SOH). Vilkårene er bekreftet
via en dansk Renault-kilde (paneuropeisk politikk, ikke direkte
bekreftet på en norsk side), kombinert med et langt etablert
forhandlernett i Norge. Scoret 4/5.

Legger til to nye kilder (Renault EV-garanti, Renault 4 Norge-side).
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2627,6 +2627,80 @@
       <c r="H47" t="inlineStr">
         <is>
           <t>Nyhetsdekning av offisiell registreringsstatistikk fra OFV (Opplysningsrådet for Veitrafikken). Model 3 var Norges mest solgte bilmodell i 2020 og 2021 (over 12 000 solgte i 2021 alene), og over 60 000 eksemplarer er i dag registrert i Norge; OFV-tall for november 2025 viser 2 562 nyregistrerte Model 3 i den ene måneden alene.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_EV_WARRANTY_2025</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Renault garanti – hvor længe og hvad er dækket?</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Renault (Danmark, renault.dk)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://www.renault.dk/kob/garanti</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Dansk Renault-garantiside. Beskriver en paneuropeisk garantiendring fra mai 2025: 5 år/150 000 km generell garanti på alle nye elektriske Renault-modeller, samt 8 år/160 000 km batterigaranti (minst 70 % SOH garantert). Ikke uavhengig bekreftet på en norsk Renault-side; behandlet som MEDIUM-konfidens for det norske markedet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_4_NO_LAUNCH</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Renault 4 E-Tech electric</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Renault Norge</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://www.renault.no/personbil/renault-4-e-tech-electric</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Offisiell Renault Norge-produktside bekrefter at 4 E-Tech Electric kommer tilbake for 2025 som en helelektrisk modell ("tilbake i 2025, 100 % elektrisk"); eksakt norsk lanseringsdato er ikke oppgitt på selve siden. Samlet søkeresultat (ikke uavhengig reverifisert) plasserer markedstilgjengelighet til høsten 2025.</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5179,6 +5253,86 @@
       <c r="H63" t="inlineStr">
         <is>
           <t>Traceable to REV_000062 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>SCORE_000064</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>W014</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>REV_000063</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F64">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D64,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G64">
+        <f>ROUND(F64*INDEX('01_Criteria'!$F:$F,MATCH(C64,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000063 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>SCORE_000065</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>W015</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>REV_000064</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F65">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D65,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G65">
+        <f>ROUND(F65*INDEX('01_Criteria'!$F:$F,MATCH(C65,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000064 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -17874,7 +18028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -20410,6 +20564,86 @@
         </is>
       </c>
       <c r="I63" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>REV_000063</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>3</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Renault 4 E-Tech er tilgjengelig i Norge fra høsten 2025 - under ett år på markedet ved vurderingstidspunktet, og en helt ny plattform (AmpR Small) uten egen lang sporhistorikk. Produsenten selv er langt fra ny (over 125 år i bilbransjen, lang nordisk tilstedeværelse), men den konkrete konfigurasjonens ferskhet tilsier en forsiktig middels vurdering. [Kriterium W014]</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>EV_000083</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>REV_000064</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>4</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Renault innførte fra mai 2025 5 års/150 000 km generell garanti på alle nye elbiler, i tillegg til 8 års/160 000 km batterigaranti (minst 70 % SOH). Vilkårene ble bekreftet via dansk Renault-kilde (samme paneuropeiske elbilpolitikk gjelder trolig Norge, men ikke direkte bekreftet på en norsk side) - solid garanti kombinert med et langt etablert forhandler- og serviceapparat i Norge. [Kriterium W015]</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>EV_000084</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -20432,7 +20666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -22691,6 +22925,60 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>EV_000083</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Modellrisiko: Renault 4 E-Tech Electric ble tilgjengelig i det norske markedet fra høsten 2025 - under ett år på markedet ved vurderingstidspunktet (juli 2026). Bygget på Renaults nye AmpR Small-plattform uten egen lang driftshistorikk.</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_4_NO_LAUNCH</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>EV_000084</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Garanti: Renault innførte fra mai 2025 5 års/150 000 km generell nybilgaranti på alle nye elbiler, samt 8 års/160 000 km batterigaranti (minst 70 % SOH-kapasitet garantert). Bekreftet via dansk Renault-kilde som del av en paneuropeisk garantiendring; ikke direkte bekreftet på en norsk kildeside.</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_EV_WARRANTY_2025</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Skoda Elroq Selection 60 on W014, W015
W014 (produsent-/modellrisiko): Elroq gikk i produksjon januar 2025
med leveranser fra tidlig 2025 - rundt halvannet år på markedet.
Viktigere: den er den andre Skoda-modellen på Volkswagen-konsernets
MEB-plattform, som deler arkitektur med Enyaq, ID.3, ID.4/ID.5 og
Audi Q4 e-tron - flere års reell driftserfaring på tvers av merker
veier tyngre enn Elroqs egen korte modellhistorikk. Scoret 4/5.

W015 (garanti/serviceapparat): Skoda-Norge (importert av Harald A.
Møller AS) oppgir 5 år/100 000 km generell garanti samt 8 år/
160 000 km batterigaranti (minst 70 % kapasitet). Kortere
kilometergrense enn Renault og Kia, men fortsatt god margin for en
familiebil med begrenset årlig kjørelengde, og et langt etablert
forhandlernett via Møller. Scoret 4/5.

Legger til to nye kilder (Skoda Norge-garantiside, Wikipedia om
Elroq-produksjon/MEB-plattform).
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2701,6 +2701,80 @@
       <c r="H49" t="inlineStr">
         <is>
           <t>Offisiell Renault Norge-produktside bekrefter at 4 E-Tech Electric kommer tilbake for 2025 som en helelektrisk modell ("tilbake i 2025, 100 % elektrisk"); eksakt norsk lanseringsdato er ikke oppgitt på selve siden. Samlet søkeresultat (ikke uavhengig reverifisert) plasserer markedstilgjengelighet til høsten 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_WARRANTY</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Garanti | Gode garantiordninger</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Skoda Norge (Harald A. Møller AS)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://www.skoda-auto.no/eie/garantier</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Offisiell Skoda Norge-garantiside, hentet direkte. "5 års Norgesgaranti": 5 år/100 000 km generell garanti (biler førstegangsregistrert etter 2011-01-01, importert av Harald A. Møller AS). Alle nye ladbare hybrider og elbiler: 8 år/160 000 km batteripakkegaranti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_ELROQ_WIKIPEDIA_PLATFORM</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>COMMUNITY</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Škoda Elroq</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/%C5%A0koda_Elroq</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Bekrefter at Elroq gikk i produksjon januar 2025 med de første kundeleveransene tidlig i 2025, etter å ha blitt vist frem på Paris Motor Show oktober 2024. Er den andre Skoda-modellen på Volkswagen-konsernets MEB-plattform, som deles med Enyaq, ID.3, ID.4/ID.5 og Audi Q4 e-tron.</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5333,6 +5407,86 @@
       <c r="H65" t="inlineStr">
         <is>
           <t>Traceable to REV_000064 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>SCORE_000066</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>W014</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>REV_000065</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F66">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D66,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G66">
+        <f>ROUND(F66*INDEX('01_Criteria'!$F:$F,MATCH(C66,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000065 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>SCORE_000067</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>W015</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>REV_000066</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F67">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D67,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G67">
+        <f>ROUND(F67*INDEX('01_Criteria'!$F:$F,MATCH(C67,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000066 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -18028,7 +18182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -20644,6 +20798,86 @@
         </is>
       </c>
       <c r="I65" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>REV_000065</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>4</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Elroq gikk i produksjon januar 2025 med leveranser fra tidlig 2025 - rundt halvannet år på markedet. Viktigere: den er den andre Skoda-modellen bygget på Volkswagen-konsernets MEB-plattform, som også deler arkitektur med Enyaq, ID.3, ID.4/ID.5 og Audi Q4 e-tron - en plattform med flere års reell driftserfaring på tvers av merker. Modenheten i den delte plattformen veier tyngre enn Elroqs egen korte modellhistorikk. [Kriterium W014]</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>EV_000085</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>REV_000066</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>4</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Skoda-Norge (importert av Harald A. Møller AS) tilbyr 5 års/100 000 km generell nybilgaranti samt 8 års/160 000 km batterigaranti (minst 70 % kapasitet) på alle nye elbiler. Kortere kilometergrense enn Renault og Kia, men fortsatt god margin for en familiebil med begrenset årlig kjørelengde (jf. W018), og et langt etablert, landsdekkende forhandlernett via Møller-apparatet. [Kriterium W015]</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>EV_000086</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -20666,7 +20900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -22979,6 +23213,60 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>EV_000085</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Modellrisiko: Elroq gikk i produksjon januar 2025 med kundeleveranser fra tidlig 2025, etter å ha blitt vist frem på Paris Motor Show oktober 2024. Er den andre Skoda-modellen på Volkswagen-konsernets MEB-plattform, som deler arkitektur med Enyaq, ID.3, ID.4/ID.5 og Audi Q4 e-tron.</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_ELROQ_WIKIPEDIA_PLATFORM</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>EV_000086</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Garanti: Skoda-Norge (importert av Harald A. Møller AS) oppgir 5 års/100 000 km generell nybilgaranti, samt 8 års/160 000 km batterigaranti (minst 70 % kapasitet) på alle nye elbiler og ladbare hybrider.</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_WARRANTY</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Tesla Model 3 LR RWD on W016
W016 (Nordisk modenhet): Model 3 har deltatt i NAF/Motor sin årlige
vintertest hvert år siden 2020, med jevnt sterke og forbedrede
resultater (faktisk kjørt distanse ca. 521-548 km over ulike
vintertester, WLTP-oppgitt rekkevidde økt fra 560 til 614 km over
generasjoner). Klart lengste og mest kontinuerlig verifiserte
vinterhistorikk av de fem konfigurasjonene. Scoret 5/5.

Legger til én ny kilde (bil24.no-dekning av NAF/Motor sin
El Prix-vintertest).
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2886,6 +2886,43 @@
       <c r="H54" t="inlineStr">
         <is>
           <t>Offisiell Kia-pressemelding distribuert via NTB. Bekrefter produksjonsstart for alle EV2-batterialternativer 2026-06-25, og en oppfølgende pressemelding bekrefter at salget av EV2 formelt startet 2026-07-02 - få dager før denne vurderingen. GT Line tilbys blant de første variantene i salg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SRC_NAF_TESLA_MODEL3_VINTERTEST</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Verdens største vintertest: Tesla Model 3 gikk lengst</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>bil24.no (dekning av NAF/Motor sin El Prix-vintertest)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://bil24.no/verdens-storste-vintertest-tesla-model-3-gikk-lengst/</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Dekker NAF/Motor sin årlige El Prix-vintertest, der Tesla Model 3 har deltatt hvert år siden 2020 med jevnt sterke resultater (WLTP-oppgitt rekkevidde økt fra 560 til 614 km over generasjoner; faktisk kjørt distanse har variert mellom ca. 521 og 548 km i ulike vintertester, gjennomgående blant de beste i klassen).</t>
         </is>
       </c>
     </row>
@@ -2906,7 +2943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5758,6 +5795,46 @@
       <c r="H71" t="inlineStr">
         <is>
           <t>Traceable to REV_000070 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>SCORE_000072</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>W016</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>REV_000071</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F72">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D72,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G72">
+        <f>ROUND(F72*INDEX('01_Criteria'!$F:$F,MATCH(C72,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000071 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -18453,7 +18530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -21309,6 +21386,46 @@
         </is>
       </c>
       <c r="I71" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>REV_000071</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>5</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Model 3 har den desidert lengste og mest kontinuerlig dokumenterte vinterhistorikken av de fem konfigurasjonene: testet av NAF/Motor hvert år siden 2020, med jevnt sterke og forbedrede resultater (521-548 km faktisk kjørt over ulike vintertester, WLTP økt fra 560 til 614 km). Et reelt, flerårig "over tid"-bevis for nordisk klimaegnethet. [Kriterium W016]</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>EV_000090</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -21331,7 +21448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -23779,6 +23896,33 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>EV_000090</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Nordisk modenhet: Tesla Model 3 har deltatt i NAF/Motor sin årlige vintertest hvert år siden 2020, med jevnt sterke og forbedrede resultater (WLTP-rekkevidde økt fra 560 til 614 km over generasjoner; faktisk kjørt distanse ca. 521-548 km i ulike vintertester) - den klart lengste, mest kontinuerlig verifiserte vinterhistorikken av de fem konfigurasjonene.</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>SRC_NAF_TESLA_MODEL3_VINTERTEST</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Renault 4 Techno on W016
W016 (Nordisk modenhet): Renault 4 E-Tech bygger på en helt ny
plattform (AmpR Small, jf. W014) uten egen vinterhistorikk. Den
eneste tilgjengelige "over tid"-dokumentasjonen for merket er
forgjengeren Zoe, som har en reell, dokumentert historikk med
varmepumpe-/varmeelementsvikt og rekkeviddetap på opptil 40 % i kulde
- riktignok bedret i senere generasjoner (R110/R135). Uten egen
modellspesifikk vinterdata og med en historisk blandet
merkebakgrunn på nettopp dette punktet, gir dette den svakeste
vurderingen av de fem. Scoret 2/5.

Legger til én ny kilde (om Zoes historiske varmepumpeproblemer i
kulde).
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2923,6 +2923,43 @@
       <c r="H55" t="inlineStr">
         <is>
           <t>Dekker NAF/Motor sin årlige El Prix-vintertest, der Tesla Model 3 har deltatt hvert år siden 2020 med jevnt sterke resultater (WLTP-oppgitt rekkevidde økt fra 560 til 614 km over generasjoner; faktisk kjørt distanse har variert mellom ca. 521 og 548 km i ulike vintertester, gjennomgående blant de beste i klassen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_ZOE_HEATPUMP_COLD_ISSUES</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Renault Zoe lader ikke og andre problemer og feil</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Bildelerekspert</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://www.bildelerekspert.co.no/blogg/renault-zoe-lader-ikke-og-andre-problemer-og-feil-2559</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Dokumenterer tilbakevendende svikt i varmepumpe/varmeelement på Renault Zoe (Renaults forrige generasjons elbil) etter 20 000-30 000 km, som kan redusere rekkevidden i kulde med opptil 40 %. Nyere generasjoner (R110/R135) med aktiv batteritemperaturstyring håndterer dette 'vesentlig bedre' enn de tidligste modellene. Gjelder en annen, eldre Renault-elbilplattform enn den helt nye Renault 4 (AmpR Small), men representerer Renaults dokumenterte merkehistorikk i nordisk kulde over tid.</t>
         </is>
       </c>
     </row>
@@ -2943,7 +2980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5835,6 +5872,46 @@
       <c r="H72" t="inlineStr">
         <is>
           <t>Traceable to REV_000071 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>SCORE_000073</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>W016</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>REV_000072</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F73">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D73,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G73">
+        <f>ROUND(F73*INDEX('01_Criteria'!$F:$F,MATCH(C73,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000072 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -18530,7 +18607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -21426,6 +21503,46 @@
         </is>
       </c>
       <c r="I72" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>REV_000072</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>2</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Renault 4 E-Tech bygger på en helt ny plattform (AmpR Small, jf. W014) uten egen vinterhistorikk. Den eneste tilgjengelige "over tid"-dokumentasjonen for merket er forgjengeren Zoe, som har en reell, dokumentert historikk med varmepumpe-/varmeelementsvikt og rekkeviddetap på opptil 40 % i kulde - riktignok bedret i senere generasjoner. Uten egen modellspesifikk vinterdata og med en historisk blandet merkebakgrunn på nettopp dette punktet, gir dette den svakeste vurderingen av de fem. [Kriterium W016]</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>EV_000091</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -21448,7 +21565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -23923,6 +24040,33 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>EV_000091</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Nordisk modenhet: Renaults forrige generasjons elbil (Zoe) har en dokumentert historikk med svikt i varmepumpe/varmeelement etter 20 000-30 000 km, med rekkeviddetap i kulde på opptil 40 % i de tidligste modellene - om enn betydelig bedret i senere generasjoner (R110/R135). Renault 4 E-Tech bygger på en helt ny plattform (AmpR Small) uten egen vinterhistorikk, så den eneste tilgjengelige 'over tid'-dokumentasjonen for merket er denne blandede Zoe-historikken.</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_ZOE_HEATPUMP_COLD_ISSUES</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Skoda Elroq Selection 60 on W016
W016 (Nordisk modenhet): Elroq Selection 60 selv mangler egen
flerårig vinterhistorikk, men MEB-plattformen den deler med VW ID.4
og Skoda Enyaq har vært testet av NAF/Motor siden januar 2022 med
gjennomgående sterke resultater (kun 11-15 % under WLTP, blant de
beste i feltet sammen med Tesla Model 3/Y og Kia EV6). Plattformens
dokumenterte, flerårige nordiske vintermodenhet veier tungt selv om
Elroq-modellen selv er ferskere. Scoret 4/5.

Legger til én ny kilde (NAF sin vintertest 2022, ID.4/Enyaq-resultater
på MEB-plattformen).
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2960,6 +2960,43 @@
       <c r="H56" t="inlineStr">
         <is>
           <t>Dokumenterer tilbakevendende svikt i varmepumpe/varmeelement på Renault Zoe (Renaults forrige generasjons elbil) etter 20 000-30 000 km, som kan redusere rekkevidden i kulde med opptil 40 %. Nyere generasjoner (R110/R135) med aktiv batteritemperaturstyring håndterer dette 'vesentlig bedre' enn de tidligste modellene. Gjelder en annen, eldre Renault-elbilplattform enn den helt nye Renault 4 (AmpR Small), men representerer Renaults dokumenterte merkehistorikk i nordisk kulde over tid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SRC_NAF_MEB_WINTER_ID4_ENYAQ</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>NAF Vintertest av rekkevidde på elbil 2022</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>NAF (Norges Automobil-Forbund)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://www.naf.no/elbil/bruke-elbil/test-rekkevidde-vinter-2022</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>NAF/Motor sin vintertest fra januar 2022 inkluderte VW ID.4 og Skoda Enyaq (samme MEB-plattform som Elroq), samt Tesla Model 3/Model Y og Kia EV6. Konklusjonen for ID.4 var 'rekkevidden holder seg godt i kulde, selv om varmepumpen sliter litt på de kaldeste dagene' - blant flere modeller som kun tapte 11-15 % av WLTP-rekkevidden. Representerer flere års gjentatt, konsistent MEB-plattformytelse i norsk vinterklima, selv om Elroq Selection 60 ikke selv var inkludert i denne konkrete testen.</t>
         </is>
       </c>
     </row>
@@ -2980,7 +3017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5912,6 +5949,46 @@
       <c r="H73" t="inlineStr">
         <is>
           <t>Traceable to REV_000072 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>SCORE_000074</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>W016</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>REV_000073</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F74">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D74,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G74">
+        <f>ROUND(F74*INDEX('01_Criteria'!$F:$F,MATCH(C74,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000073 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -18607,7 +18684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -21543,6 +21620,46 @@
         </is>
       </c>
       <c r="I73" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>REV_000073</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>4</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Elroq Selection 60 selv mangler egen flerårig vinterhistorikk, men MEB-plattformen den deler med VW ID.4 og Skoda Enyaq har vært testet av NAF/Motor siden januar 2022 med gjennomgående sterke resultater (kun 11-15 % under WLTP, blant de beste i feltet). Plattformens dokumenterte, flerårige nordiske vintermodenhet veier tungt selv om Elroq-modellen selv er ferskere. [Kriterium W016]</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>EV_000092</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -21565,7 +21682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H92"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -24067,6 +24184,33 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>EV_000092</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Nordisk modenhet: VW ID.4 og Skoda Enyaq (samme MEB-plattform som Elroq) ble testet av NAF/Motor i vintertesten fra januar 2022 med sterke resultater ('rekkevidden holder seg godt i kulde'), kun 11-15 % under WLTP - blant de beste i feltet sammen med Tesla Model 3/Y og Kia EV6. Flere års konsistent plattformytelse i norsk vinterklima, om enn ikke Elroq Selection 60 spesifikt.</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>SRC_NAF_MEB_WINTER_ID4_ENYAQ</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Volvo EX30 P8 AWD on W016
W016 (Nordisk modenhet): EX30 Twin Performance (samme drivlinje som
P8 AWD) har ett solid, uavhengig vintertestresultat: elbil.no anslo
omtrent 75 % av WLTP-rekkevidden beholdt ned mot -20°C. Dette er
reell, modellspesifikk evidens, men fra kun én vintersesong -
kortere dokumentert historikk enn både Tesla og MEB-plattformen, om
enn understøttet av Volvos lange generelle tilstedeværelse i det
nordiske markedet. Scoret 4/5.

Ingen nye kilder - gjenbruker eksisterende elbil.no-vintertest
(SRC_ELBIL_VOLVO_EX30_WINTER) som tidligere kun var referert i
Configurations-notatene, nå formalisert som Evidence for dette
kriteriet.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -3017,7 +3017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5989,6 +5989,46 @@
       <c r="H74" t="inlineStr">
         <is>
           <t>Traceable to REV_000073 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>SCORE_000075</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>W016</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>REV_000074</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F75">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D75,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G75">
+        <f>ROUND(F75*INDEX('01_Criteria'!$F:$F,MATCH(C75,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000074 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -18684,7 +18724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -21660,6 +21700,46 @@
         </is>
       </c>
       <c r="I74" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>REV_000074</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>4</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>EX30 Twin Performance (samme drivlinje som P8 AWD) har ett solid, uavhengig vintertestresultat: elbil.no anslo omtrent 75 % av WLTP-rekkevidden beholdt ned mot -20°C. Dette er reell, modellspesifikk evidens, men fra kun én vintersesong - kortere dokumentert historikk enn både Tesla og MEB-plattformen, om enn understøttet av Volvos lange generelle tilstedeværelse i det nordiske markedet. [Kriterium W016]</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>EV_000093</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -21682,7 +21762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -24211,6 +24291,33 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>EV_000093</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Nordisk modenhet: elbil.no sin uavhengige vintertest av EX30 Twin Performance (samme drivlinje som P8 AWD) anslo at bilen beholdt rundt 75 % av WLTP-rekkevidden under reelle vinterforhold ned mot -20°C, etter et mellomstopp for hurtiglading. Ett solid, modellspesifikt datapunkt, men fra kun én vintersesong - kortere dokumentert historikk enn Tesla og MEB-plattformen.</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_VOLVO_EX30_WINTER</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Kia EV2 GT-Line on W016
W016 (Nordisk modenhet): EV2 GT Line selv har ingen driftshistorikk
(jf. W014), men to uavhengige datapunkter trekker vurderingen
tydelig opp: (1) en lang, positiv merkehistorikk for
varmepumpeassistert kuldeytelse på søskenmodellene e-Niro og EV6,
og (2) et faktisk NAF-verifisert vintertestresultat for en
EV2-prototyp med samme 61 kWh-batteri (310,6 km i temperaturer ned
mot -31°C, kun 24,8 % under WLTP, samt sterk hurtigladeytelse i
ekstrem kulde). Det siste er reell modellspesifikk evidens, om enn
fra en prototyp og ikke en levert kundebil - vesentlig sterkere enn
et rent merke-fallback alene ville gitt. Scoret 4/5.

Legger til to nye kilder (elbil24.no om Kia e-Niro/EV6-vintertester,
InsideEVs om EV2-prototypens NAF-vintertest) og fullfører denne
rundens W016-scoring på tvers av alle fem konfigurasjoner (15/20
kriterier, 77 % dekning).
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2997,6 +2997,80 @@
       <c r="H57" t="inlineStr">
         <is>
           <t>NAF/Motor sin vintertest fra januar 2022 inkluderte VW ID.4 og Skoda Enyaq (samme MEB-plattform som Elroq), samt Tesla Model 3/Model Y og Kia EV6. Konklusjonen for ID.4 var 'rekkevidden holder seg godt i kulde, selv om varmepumpen sliter litt på de kaldeste dagene' - blant flere modeller som kun tapte 11-15 % av WLTP-rekkevidden. Representerer flere års gjentatt, konsistent MEB-plattformytelse i norsk vinterklima, selv om Elroq Selection 60 ikke selv var inkludert i denne konkrete testen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL24_KIA_EV6_ENIRO_WINTER</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Vintertest: Kia EV6 i norsk sprengkulde</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>elbil24.no</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://www.elbil24.no/tester/vintertest-kia-ev6-i-norsk-sprengkulde/74846150</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>NAF/Motor-vintertester av Kia e-Niro og EV6 viser sterk varmepumpeassistert kuldeytelse ('uvanlig behagelig i kulden'; e-Niro tapte kun rundt 10 % rekkevidde). EV6 gikk fra 481 til 341 km ved rundt -10°C, men rangerte likevel høyt, med varm kupé og upåvirket infotainmentskjerm selv i sterk kulde.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>SRC_INSIDEEVS_KIA_EV2_WINTER_PROTOTYPE</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Freezing Temps Crush Range. But Kia's Newest EV Dominated This Test</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>InsideEVs</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://insideevs.com/news/786909/ev2-prototype-winter-range-tests/</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>En Kia EV2-prototyp (61 kWh Long Range) deltok i NAFs El Prix-vintertest i Norge, februar 2026, i temperaturer mellom -8°C og -31°C: kjørte 310,6 km, kun 24,8 % under WLTP-oppgitt rekkevidde - blant de beste i testfeltet. Hurtiglading 8 %→80 % på under 37 minutter (97 kW effekttopp, 74 kW snitt) selv i ekstrem kulde. Gjelder en produksjonsnær prototyp, ikke en levert kundebil.</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6029,6 +6103,46 @@
       <c r="H75" t="inlineStr">
         <is>
           <t>Traceable to REV_000074 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>SCORE_000076</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>W016</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>REV_000075</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F76">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D76,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G76">
+        <f>ROUND(F76*INDEX('01_Criteria'!$F:$F,MATCH(C76,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000075 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -18724,7 +18838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -21740,6 +21854,46 @@
         </is>
       </c>
       <c r="I75" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>REV_000075</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>4</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>EV2 GT Line selv har ingen driftshistorikk (jf. W014), men to uavhengige datapunkter trekker vurderingen opp: (1) en lang, positiv merkehistorikk for varmepumpeassistert kuldeytelse på søskenmodellene e-Niro og EV6, og (2) et faktisk NAF-verifisert vintertestresultat for en EV2-prototyp med samme 61 kWh-batteri (310,6 km i temperaturer ned mot -31°C, kun 24,8 % under WLTP, samt sterk hurtigladeytelse i ekstrem kulde). Sistnevnte er reell modellspesifikk evidens, om enn fra en prototyp og ikke en levert kundebil, og det trekker vurderingen tydelig over det rene merke-fallbacket. [Kriterium W016]</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>EV_000094,EV_000095</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -21762,7 +21916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -24318,6 +24472,60 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>EV_000094</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Nordisk modenhet (merkenivå): NAF/Motor-vintertester av søskenmodellene Kia e-Niro og EV6 viser sterk varmepumpeassistert kuldeytelse over flere år ('uvanlig behagelig i kulden'; EV6 gikk fra 481 til 341 km ved rundt -10°C, men rangerte fortsatt høyt, med varm kupé og upåvirket infotainment). Ingen av disse modellene er EV2, men de representerer en lang, positiv merkehistorikk i nordisk vinterklima.</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL24_KIA_EV6_ENIRO_WINTER</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>EV_000095</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Nordisk modenhet (modellspesifikk): En Kia EV2-prototyp (61 kWh Long Range, samme batteri som denne konfigurasjonen) deltok i NAFs egen vintertest i Norge februar 2026, i temperaturer fra -8°C til -31°C: kjørte 310,6 km, kun 24,8 % under WLTP - blant de beste i testfeltet, med sterk hurtigladeytelse i ekstrem kulde (8 %→80 % på under 37 minutter). Faktisk NAF-verifisert, modellspesifikk vintertest, om enn på en produksjonsnær prototyp fremfor en levert kundebil.</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>SRC_INSIDEEVS_KIA_EV2_WINTER_PROTOTYPE</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Tesla Model 3 LR RWD on W018
Praktisk bruk/bagasje: 682L combined boot+frunk, flat rear floor,
60/40 split-fold seats, and ISOFIX on both outer rear seats support
family use, offset by the narrow saloon boot opening and a somewhat
cramped rear knee position. Scored 4/5, MEDIUM confidence.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3737,6 +3737,80 @@
       <c r="H77" t="inlineStr">
         <is>
           <t>Oppsummerer pålitelighetsdata for Kias nylige elbilportefølje: EV6 (2022-2026 årsmodeller) har en gjennomsnittlig pålitelighetsscore på 75/100 (JD Power/Consumer Reports-baserte kilder), med tidlige modeller som hadde elektriske/drivverk-problemer, men betydelig forbedring fra 2025-årsmodellen. EV9 (større, mer kompleks 3-seters SUV) scorer lavere, 67/100, under gjennomsnittet for nye biler. EV2 er nærmere EV6/Niro EV i segment og kompleksitet enn EV9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_OWNERSMANUAL_MODEL3_NO_BARNESIKRING</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Model 3 Brukerhåndbok – Barnesikringsutstyr</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>https://www.tesla.com/ownersmanual/model3/no_no/GUID-BD88652C-E641-4889-B7DF-6A4E32727388.html</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Offisiell norsk brukerhåndbok, avsnitt om barnesikringsutstyr/ISOFIX. Bekrefter ISOFIX/i-Size-forankring i begge ytre baksetene, ingen ISOFIX-forankring i forsetet, og at beltebaserte barneseter kan monteres i alle passasjerseter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_TESLA_MODEL3_PRACTICALITY</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Tesla Model 3 review – Space &amp; practicality</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>What Car?</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>https://www.whatcar.com/tesla/model-3/saloon/review/n19010/space-practicality</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Bekrefter 594 L bagasjerom bak + 88 L frunk (682 L kombinert, samsvarer med Teslas eget totaltall), flatt bakgulv uten sentertunnel, 60/40-delt nedfellbar rygglene, samt at sedan-bagasjeromsåpningen er mindre fleksibel enn en femdørs/stasjonsvogn og at baksetets kne-høye sittestilling oppleves noe ubehagelig på lengre turer.</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H96"/>
+  <dimension ref="A1:H97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7609,6 +7683,46 @@
       <c r="H96" t="inlineStr">
         <is>
           <t>Traceable to REV_000095 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>SCORE_000097</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>W018</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>REV_000096</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F97">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D97,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G97">
+        <f>ROUND(F97*INDEX('01_Criteria'!$F:$F,MATCH(C97,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000096 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -20304,7 +20418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -24160,6 +24274,46 @@
         </is>
       </c>
       <c r="I96" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>REV_000096</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Praktisk bruk</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>4</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Kombinert bagasjerom på 682 liter (594 L bagasjerom bak + 88 L frunk foran) er stort for segmentet, med flatt bakgulv uten sentertunnel og 60/40-delt nedfellbar rygglene for å utvide lastekapasiteten ved behov. ISOFIX/i-Size-forankring er bekreftet på begge ytre baksetene (ikke forsetet), som dekker standard barnesetebehov for en familiebil. Den smale sedan-bagasjeromsåpningen - i motsetning til en femdørs/stasjonsvogn - begrenser noe hvor praktisk store gjenstander som barnevogn er å laste, og baksetets kne-høye sittestilling er av uavhengige anmeldere beskrevet som noe ubehagelig på lengre turer. Samlet solid, men ikke optimal, praktisk bruk for familiens hovedbil med begrenset årlig kjørelengde. [Kriterium W018]</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>EV_000117,EV_000118</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -24182,7 +24336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:H119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -27359,6 +27513,60 @@
         </is>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>EV_000117</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Praktisk bruk/bagasje: Uavhengig anmeldelse bekrefter et kombinert bagasjerom på 682 liter, fordelt på 594 liter i bagasjerommet bak og 88 liter i frunken foran (samsvarer med Teslas offisielle totaltall). Baksetet har flatt gulv uten sentertunnel å knå over, og 60/40-delt rygglene som kan felles for å utvide lastekapasiteten. Sedan-utformingen gir imidlertid en smalere bagasjeromsåpning enn en femdørs/stasjonsvogn, noe som kan begrense praktisk lasting av store gjenstander som barnevogn. Baksetets kne-høye sittestilling beskrives som noe ubehagelig for voksne på lengre turer.</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_TESLA_MODEL3_PRACTICALITY</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>EV_000118</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Barnesikring: Teslas offisielle norske brukerhåndbok bekrefter at ISOFIX/i-Size-forankringspunkter kan monteres i begge de ytre baksetene, mens forsetet (passasjersetet) ikke har ISOFIX-forankring. Beltebaserte barneseter kan monteres i alle passasjerseter. Dette dekker standardbehovet for en familiebil med barn i barnesete/beltestol.</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_OWNERSMANUAL_MODEL3_NO_BARNESIKRING</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Renault 4 Techno on W018
Praktisk bruk/bagasje: 420L boot (1405L folded), low load threshold,
wide opening, and a hands-free tailgate give strong everyday
practicality; rear legroom beats class average thanks to the longer
wheelbase, and ISOFIX is confirmed on both outer rear seats. Offset
by a cramped rear footwell from battery intrusion and a folded-seat
step from the lack of a two-level boot floor. Scored 4/5, MEDIUM
confidence.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3811,6 +3811,80 @@
       <c r="H79" t="inlineStr">
         <is>
           <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Bekrefter 594 L bagasjerom bak + 88 L frunk (682 L kombinert, samsvarer med Teslas eget totaltall), flatt bakgulv uten sentertunnel, 60/40-delt nedfellbar rygglene, samt at sedan-bagasjeromsåpningen er mindre fleksibel enn en femdørs/stasjonsvogn og at baksetets kne-høye sittestilling oppleves noe ubehagelig på lengre turer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_BAGASJEROM</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Romslig bagasjerom med modulært interiør</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Renault (via mobile.no)</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>https://mobile.no/nybil/personbil/renault/renault-4-e-tech-electric/romslig-bagasjerom-med-modulaert-interior</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Norsk markedsartikkel som gjengir Renaults offisielle spesifikasjoner for Renault 4 E-Tech: bagasjerom på 420 liter (1405 liter med nedfelt baksete), 40/60-delt nedfellbar baksete, hands-free bakluke, lav terskel og bred åpning, samt 23,3 liter oppbevaringsplass i kupeen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>SRC_CARWOW_RENAULT4_SPECS</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Renault 4 E-Tech | Specifications &amp; Dimensions</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Carwow</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>https://www.carwow.co.uk/renault/4-e-tech/specifications</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Britisk profesjonell anmeldelse/spesifikasjonsside (ikke Norge-spesifikk). Bekrefter ISOFIX-forankring i begge ytre baksetene (tre ISOFIX-kompatible posisjoner totalt), 60/40-delt rygglene uten gjennomlastingsluke, samt at fotplassen bak er trang fordi batteriet stikker inn i fotrommet - ingen fotplass under forsetene. Noterer også at det mangler et to-nivås bagasjeromsgulv, som skaper et trinn ved nedfelte seter.</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H97"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7723,6 +7797,46 @@
       <c r="H97" t="inlineStr">
         <is>
           <t>Traceable to REV_000096 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>SCORE_000098</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>W018</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>REV_000097</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F98">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D98,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G98">
+        <f>ROUND(F98*INDEX('01_Criteria'!$F:$F,MATCH(C98,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000097 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -11072,7 +11186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:J152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -17746,6 +17860,51 @@
         </is>
       </c>
       <c r="J151" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>TECH_000145</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Boot volume</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>420</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_BAGASJEROM</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -20418,7 +20577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -24314,6 +24473,46 @@
         </is>
       </c>
       <c r="I97" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>REV_000097</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Praktisk bruk</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>4</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Bagasjerom på 420 liter, som utvides til 1405 liter med nedfelt baksete (40/60-delt), lav lasteterskel, bred åpning og elektrisk bakluke på Techno gir solid og fleksibel hverdagspraktisk last for en familiebil. Baksetets benplass er bedre enn gjennomsnittet for klassen takket være et lengre akselavstand enn Renault 5, og ISOFIX-forankring er bekreftet på begge ytre baksetene. Trekkes noe ned av trang fotplass bak (batteriet stikker inn i fotrommet) og et lite trinn ved nedfelte seter grunnet manglende to-nivås bagasjeromsgulv. Samlet solid praktisk bruk for familiens hovedbil med begrenset årlig kjørelengde. [Kriterium W018]</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>EV_000119,EV_000120</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -24336,7 +24535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H119"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -27567,6 +27766,60 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>EV_000119</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Praktisk bruk/bagasje: Offisiell norsk kilde bekrefter et bagasjerom på 420 liter, som utvides til 1405 liter med baksetene nedfelt (40/60-delt rygglene). Bagasjerommet har lav terskel og bred åpning, og Techno-utgaven har elektrisk (hands-free) bakluke. Dette gir god fleksibilitet for en familiebil med varierende lastebehov.</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_BAGASJEROM</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>EV_000120</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Barnesikring og baksete: Uavhengig anmeldelse bekrefter ISOFIX-forankring i begge de ytre baksetene. Baksetets benplass beskrives som bedre enn gjennomsnittet for klassen takket være et 8 cm lengre akselavstand enn Renault 5, men fotplassen bak er noe trang på grunn av at batteriet stikker inn i fotrommet - det er ikke fotplass under forsetene. Ved nedfelling av baksetene (60/40-delt) mangler det et to-nivås bagasjeromsgulv, som skaper et lite trinn mellom bagasjerommet og de nedfelte setene.</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>SRC_CARWOW_RENAULT4_SPECS</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Skoda Elroq Selection 60 on W018
Praktisk bruk/bagasje: 470L boot (1580L folded) is among the largest
in class, and a wheelbase matching the larger Enyaq despite a 160mm
shorter body gives unusually good rear legroom. ISOFIX is confirmed
on both outer rear seats plus the front passenger seat - three points,
more than Tesla or Renault in this comparison - backed by Simply
Clever touches (adjustable parcel shelf, ice scraper, umbrella
holder, cable storage). No material practicality drawbacks surfaced.
Scored 5/5, MEDIUM confidence.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3885,6 +3885,80 @@
       <c r="H81" t="inlineStr">
         <is>
           <t>Britisk profesjonell anmeldelse/spesifikasjonsside (ikke Norge-spesifikk). Bekrefter ISOFIX-forankring i begge ytre baksetene (tre ISOFIX-kompatible posisjoner totalt), 60/40-delt rygglene uten gjennomlastingsluke, samt at fotplassen bak er trang fordi batteriet stikker inn i fotrommet - ingen fotplass under forsetene. Noterer også at det mangler et to-nivås bagasjeromsgulv, som skaper et trinn ved nedfelte seter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>SRC_MOBILE_NO_ELROQ_BAGASJEROM</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Størrelse og bagasjerom i Škoda Elroq</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Skoda (via mobile.no)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>https://mobile.no/nybil/personbil/skoda/elroq/storrelse-og-bagasjerom-i-koda-elroq</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Norsk markedsartikkel som gjengir Skodas offisielle spesifikasjoner for Elroq: bagasjerom på 470 liter (1580 liter med nedfelte seter), kabeloppbevaring under hattehyllen, og samme akselavstand som den større Enyaq til tross for 160 mm kortere karosseri, som gir svært god benplass i baksetet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>SRC_PARKERS_ELROQ_PRACTICALITY</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Skoda Elroq (2026) boot space &amp; practicality</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Parkers</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>https://www.parkers.co.uk/skoda/elroq/review/practicality/</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Bekrefter ISOFIX-forankring i begge ytre baksetene og i forsetet (tre punkter totalt), et flatt baksete som gir plass til en voksen midt bak, en hattehylle som kan plasseres i to høyder for å dele opp bagasjerommet, samt Simply Clever-detaljer (isskrape i bakluken, paraplyholder i førerdøren, hjørnehyller mot forskyvning av last).</t>
         </is>
       </c>
     </row>
@@ -3905,7 +3979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H98"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7837,6 +7911,46 @@
       <c r="H98" t="inlineStr">
         <is>
           <t>Traceable to REV_000097 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>SCORE_000099</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>W018</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>REV_000098</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F99">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D99,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G99">
+        <f>ROUND(F99*INDEX('01_Criteria'!$F:$F,MATCH(C99,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000098 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -20577,7 +20691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I98"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -24513,6 +24627,46 @@
         </is>
       </c>
       <c r="I98" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>REV_000098</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Praktisk bruk</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>5</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Bagasjerom på 470 liter (1580 liter med nedfelte seter) er blant det største i klassen, og samme akselavstand som den større Enyaq gir uvanlig god benplass i baksetet til tross for en 160 mm kortere karosseri. ISOFIX-forankring er bekreftet i begge ytre baksetene og i forsetet - totalt tre punkter, mer enn både Tesla og Renault i denne sammenligningen. Simply Clever-detaljer (justerbar/delt hattehylle, isskrape, paraplyholder, kabeloppbevaring) understøtter hverdagsbruk ytterligere. Ingen vesentlige praktiske svakheter funnet for en familiebil med begrenset årlig kjørelengde. [Kriterium W018]</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>EV_000121,EV_000122</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -24535,7 +24689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -27820,6 +27974,60 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>EV_000121</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Praktisk bruk/bagasje: Bagasjerommet rommer 470 liter, utvidbart til 1580 liter med nedfelte seter - blant de største i klassen for kompakte elektriske SUV-er. Samme akselavstand som den større Enyaq (til tross for at Elroq er 160 mm kortere) gir svært god benplass i baksetet. Kabeloppbevaring er integrert under hattehyllen.</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>SRC_MOBILE_NO_ELROQ_BAGASJEROM</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>EV_000122</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Barnesikring og Simply Clever-løsninger: Uavhengig anmeldelse bekrefter ISOFIX-forankring i begge ytre baksetene, samt i forsetet (passasjersetet) - totalt tre monteringspunkter, mer enn de fleste konkurrenter. Baksetet er beskrevet som flatt nok til at også en voksen kan sitte komfortabelt i midten. Hattehyllen kan plasseres i to ulike høyder for å dele opp bagasjerommet, og Simply Clever-detaljer som isskrape i bakluken og paraplyholder i førerdøren understøtter hverdagsbruk.</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>SRC_PARKERS_ELROQ_PRACTICALITY</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Volvo EX30 P8 AWD on W018
Praktisk bruk/bagasje: 318L boot is the smallest of the five
configurations compared (roughly 900-1000L folded), and ISOFIX is
limited to the outer rear seats only. Independent reviews describe
the rear cabin as tight for feet and knees with a taller driver and
recommend the car mainly for occasional rather than regular family
use, directly contradicting Volvo's own more positive description of
the same rear seat - documented as a source disagreement rather than
resolved. Scored 2/5, MEDIUM confidence, the weakest practicality
package of the five so far.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3959,6 +3959,117 @@
       <c r="H83" t="inlineStr">
         <is>
           <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Bekrefter ISOFIX-forankring i begge ytre baksetene og i forsetet (tre punkter totalt), et flatt baksete som gir plass til en voksen midt bak, en hattehylle som kan plasseres i to høyder for å dele opp bagasjerommet, samt Simply Clever-detaljer (isskrape i bakluken, paraplyholder i førerdøren, hjørnehyller mot forskyvning av last).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>SRC_VOLVO_NO_EX30_BAGASJEROM</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>EX30 Bagasjerom og oppbevaring av last</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Volvo</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>https://www.volvocars.com/no/support/car/ex30/article/47d2c97fd33effd3c0a8cc3718c999b7-2200e9f555c43bb3c0a8b0975816a437-8664b2fa77a7e089c0a8296870d1a409/</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Offisiell norsk Volvo-støtteside. Direkte henting ga HTTP 403; innhold bekreftet via søkeresultat-syntese. Oppgir bagasjerom på 318 liter, utvidbart til opptil 1000 liter med nedfelte bakseter (40/60-delt), inkludert et eget rom på 61 liter under lastegulvet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>SRC_CARBUYER_EX30_PRACTICALITY</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Volvo EX30 review – Boot space, practicality &amp; boot dimensions</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Carbuyer</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>https://www.carbuyer.co.uk/volvo/ex30/practicality</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Oppgir 318 liter bagasjerom / 904 liter med nedfelte seter (60/40-delt) - noe lavere enn Volvos eget nedfelt-tall, trolig grunnet ulik målemetode. Beskriver baksetet som trangt for fot- og knehøyde ved en over gjennomsnittlig høy fører, bemerker at et stort barnesete kan være vanskelig å montere bak, og gir bagasjerom/praktisk bruk 3,0 av 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>SRC_VOLVO_NO_EX30_BAKSETER</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>EX30 Bakseter</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Volvo</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>https://www.volvocars.com/no/support/car/ex30/article/47d2c97fd33effd3c0a8cc3718c999b7-efd89bccd31a1370c0a8b04a2c4e0bc2-8664b2fa77a7e089c0a8296870d1a409/</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Offisiell norsk Volvo-støtteside. Beskriver baksetet mer positivt enn uavhengige anmeldere: tilstrekkelig benplass til å strekke bena under forsetene, svært god hodeplass takket være panoramatak, komfortable seter med god korsryggstøtte, og plass til to barneseter eller to langbeinte voksne bak.</t>
         </is>
       </c>
     </row>
@@ -3979,7 +4090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7951,6 +8062,46 @@
       <c r="H99" t="inlineStr">
         <is>
           <t>Traceable to REV_000098 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>SCORE_000100</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>W018</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>REV_000099</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F100">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D100,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G100">
+        <f>ROUND(F100*INDEX('01_Criteria'!$F:$F,MATCH(C100,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000099 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -20691,7 +20842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I99"/>
+  <dimension ref="A1:I100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -24667,6 +24818,46 @@
         </is>
       </c>
       <c r="I99" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>REV_000099</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Praktisk bruk</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>2</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Bagasjerommet på 318 liter er det minste av de fem konfigurasjonene i denne sammenligningen, selv om det kan utvides til rundt 900-1000 liter med nedfelte seter (40/60-delt) pluss et 61-liters rom under lastegulvet. ISOFIX-forankring finnes kun i de ytre baksetene, ikke i forsetet. Uavhengige anmeldere beskriver baksetet som trangt for fot- og knehøyde ved en høyere fører og anbefaler bilen fremst for sporadisk bruk eller mindre familier - i direkte motsetning til Volvos egen, mer positive omtale av baksetet. Denne uenigheten er dokumentert, ikke løst. Samlet den svakeste praktiske pakken av de fem for en "familiens hovedbil"-rolle, til tross for lav estimert årlig kjørelengde. [Kriterium W018]</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>EV_000123,EV_000124,EV_000125</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -24689,7 +24880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H123"/>
+  <dimension ref="A1:H126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -28028,6 +28219,87 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>EV_000123</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Praktisk bruk/bagasje: Volvos offisielle norske støtteside oppgir et bagasjerom på 318 liter, utvidbart til opptil 1000 liter med nedfelte bakseter (40/60-delt), inkludert et eget rom på 61 liter under lastegulvet. Dette er det minste bagasjevolumet av de fem konfigurasjonene i denne sammenligningen. En uavhengig kilde (Carbuyer) oppgir et noe lavere nedfelt volum på 904 liter - trolig grunnet ulik målemetode, men grunntallet på 318 liter i bagasjerommet er samstemt.</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>SRC_VOLVO_NO_EX30_BAGASJEROM</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>EV_000124</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Baksete og barnesikring: Uavhengig anmeldelse beskriver plassen bak som trang for fot- og knehøyde dersom føreren er over gjennomsnittlig høy, og bemerker at det kan være vanskelig å montere et stort barnesete bak. ISOFIX-forankring er kun tilgjengelig i de ytre baksetene, ikke i forsetet. Anmeldelsen gir bagasjerom/praktisk bruk en score på 3,0 av 5 og konkluderer med at baksetet egner seg for sporadisk bruk fremfor jevnlig familiebruk.</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>SRC_CARBUYER_EX30_PRACTICALITY</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>EV_000125</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Motstridende kilde (produsent): Volvos egen norske støtteside beskriver baksetet mer positivt - tilstrekkelig benplass til å strekke bena under forsetene, svært god hodeplass takket være panoramatak, komfortable seter med god korsryggstøtte, og plass til to barneseter eller to langbeinte voksne. Dette står i direkte motsetning til uavhengige anmelderes vurdering av samme baksete som trangt - dokumentert som uenighet mellom kilder, ikke løst ved å velge en foretrukket versjon.</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>SRC_VOLVO_NO_EX30_BAKSETER</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Score Kia EV2 GT-Line on W018
Praktisk bruk/bagasje: 362L boot (plus 15L frunk) trails Tesla,
Renault and Skoda but beats Volvo; independent reviews praise the
flat, lip-free load floor with a removable false floor, 60/40 split
folding, and better head-/kneeroom than several rivals in the
standard 5-seat layout. This exact priced configuration, however,
was ordered with the optional 4-seat sliding-seat conversion per the
dealer quote - useful flexibility, but it costs the car its fifth
seat, a real tradeoff for a household needing full 5-seat capacity.
No source confirms ISOFIX count/placement for the EV2, so that is
left genuinely unknown rather than assumed. Scored 3/5, MEDIUM
confidence.

This completes W018 for all 5 tracked configurations, bringing the
framework to 100% coverage on FrameworkVersion 1.4.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4070,6 +4070,80 @@
       <c r="H86" t="inlineStr">
         <is>
           <t>Offisiell norsk Volvo-støtteside. Beskriver baksetet mer positivt enn uavhengige anmeldere: tilstrekkelig benplass til å strekke bena under forsetene, svært god hodeplass takket være panoramatak, komfortable seter med god korsryggstøtte, og plass til to barneseter eller to langbeinte voksne bak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_KIA_EV2_PRACTICALITY</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Kia EV2 Review 2026, Price &amp; Specs</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>What Car?</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://www.whatcar.com/kia/ev2/hatchback/review/n28833</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Bekrefter 362 liter bagasjerom pluss 15 liter frunk foran, en flyttbar falskbunn under lastegulvet, 60/40-delt rygglene med minimal terskel/trinn ved nedfelling, helt flatt gulv uten sentertunnel, bedre hodeplass enn Renault 4 og mer knebplass enn Jeep Avenger Electric - men trangt for tre voksne ved siden av hverandre bak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>SRC_AUTOCAR_KIA_EV2_REVIEW</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Tested: 2026 Kia EV2 - Full review, price &amp; features</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Autocar</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>https://www.autocar.co.uk/car-review/kia/ev2</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Oppgir 362 liter bagasjerom (mot 420 liter i Renault 4), "fairly generous" hodeplass bak, og "just enough" knebplass for en 183 cm passasjer, med trang midtsete. Bekrefter at en 4-seters variant med skyvbar bakbenk finnes i enkelte europeiske markeder (ikke bekreftet for Storbritannia), beskrevet som "nyttig".</t>
         </is>
       </c>
     </row>
@@ -4090,7 +4164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8102,6 +8176,46 @@
       <c r="H100" t="inlineStr">
         <is>
           <t>Traceable to REV_000099 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>SCORE_000101</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>W018</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>REV_000100</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F101">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D101,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G101">
+        <f>ROUND(F101*INDEX('01_Criteria'!$F:$F,MATCH(C101,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Traceable to REV_000100 -&gt; supporting Evidence -&gt; cited Source. RawScore/WeightedScore computed via the ADR-005 formula engine.</t>
         </is>
       </c>
     </row>
@@ -20842,7 +20956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I100"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -24858,6 +24972,46 @@
         </is>
       </c>
       <c r="I100" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>REV_000100</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Praktisk bruk</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>3</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Bagasjerommet på 362 liter (pluss 15 liter frunk) er mindre enn Tesla, Renault og Skoda i denne sammenligningen, men noe større enn Volvo. Uavhengige anmeldelser roser en flat, terskelfri løsning med flyttbar falskbunn, 60/40-delt rygglene, og bedre hodeplass/knebplass enn flere konkurrenter i standard 5-seters oppsett. Den faktiske forhandlerkvitteringen for denne konfigurasjonen viser imidlertid at kjøperen har valgt en 4-seters skyvesetekonvertering (+3200 kr) - en reell nyttig fleksibilitet for kne-/bagasjeplass, men den koster bilen dens femte sete, noe som er relevant dersom husstanden trenger full 5-seters kapasitet. Ingen kilde ble funnet som bekrefter ISOFIX-antall eller -plassering spesifikt for EV2 - dette forblir genuint ukjent, ikke antatt. Samlet middels praktisk bruk for familiens hovedbil, med en reell avveining i denne spesifikke konfigurasjonen. [Kriterium W018]</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>EV_000126,EV_000127</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -24880,7 +25034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H126"/>
+  <dimension ref="A1:H128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -28300,6 +28454,60 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>EV_000126</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Praktisk bruk/bagasje: Uavhengige anmeldelser bekrefter et bagasjerom på 362 liter (pluss 15 liter frunk foran til ladekabler), med en flyttbar falskbunn som gir tilgang til ekstra oppbevaringsplass under - kan enten fylles med vesker eller fjernes helt. 60/40-delt rygglene gir tilnærmet ingen terskel eller trinn ved nedfelling. Baksetegulvet er helt flatt uten sentertunnel, med bedre hodeplass enn Renault 4 og mer knebplass enn Jeep Avenger Electric ifølge samme kilder - men tre voksne ved siden av hverandre bak vil oppleves trangt.</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_KIA_EV2_PRACTICALITY</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>EV_000127</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Konfigurasjonsspesifikk endring: Den faktiske forhandlerkvitteringen for denne konfigurasjonen viser at kjøperen har valgt en 4-seters skyvesetekonvertering (+3200 kr) som tilleggsutstyr utover standard GT Line-utstyr. Dette omgjør baksetet fra en standard 3-seters benk til en 4-seters løsning der de to gjenværende baksetene kan skyves frem/tilbake for å prioritere enten knebplass eller bagasjeromsplass. Uavhengig anmeldelse (Autocar) bekrefter at en slik skyvbar bakbenk finnes i enkelte europeiske markeder (ikke i Storbritannia), og beskriver den som nyttig. Ulempen er at bilen dermed mister sitt femte sete - relevant for en "familiens hovedbil" dersom husstanden trenger full 5-seters kapasitet. Ingen kilde ble funnet som bekrefter ISOFIX-antall eller -plassering spesifikt for EV2 - forblir genuint ukjent, ikke antatt.</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Revise Kia EV2 W018 score from 3/5 to 4/5
The user clarified this is their main car with no children in the
household, and that the 4-seat sliding-seat conversion was a
deliberate choice to trade the fifth seat for flexibility between
adult passengers (friends/family) and extra cargo space - not a
capacity shortfall. The original score treated losing the fifth seat
as a con and ISOFIX as an open gap, both of which assumed a
child-carrying use case that doesn't apply here.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -24994,7 +24994,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -25003,7 +25003,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Bagasjerommet på 362 liter (pluss 15 liter frunk) er mindre enn Tesla, Renault og Skoda i denne sammenligningen, men noe større enn Volvo. Uavhengige anmeldelser roser en flat, terskelfri løsning med flyttbar falskbunn, 60/40-delt rygglene, og bedre hodeplass/knebplass enn flere konkurrenter i standard 5-seters oppsett. Den faktiske forhandlerkvitteringen for denne konfigurasjonen viser imidlertid at kjøperen har valgt en 4-seters skyvesetekonvertering (+3200 kr) - en reell nyttig fleksibilitet for kne-/bagasjeplass, men den koster bilen dens femte sete, noe som er relevant dersom husstanden trenger full 5-seters kapasitet. Ingen kilde ble funnet som bekrefter ISOFIX-antall eller -plassering spesifikt for EV2 - dette forblir genuint ukjent, ikke antatt. Samlet middels praktisk bruk for familiens hovedbil, med en reell avveining i denne spesifikke konfigurasjonen. [Kriterium W018]</t>
+          <t>Bagasjerommet på 362 liter (pluss 15 liter frunk) er mindre enn Tesla, Renault og Skoda i denne sammenligningen, men noe større enn Volvo. Uavhengige anmeldelser roser en flat, terskelfri løsning med flyttbar falskbunn, 60/40-delt rygglene, og bedre hodeplass/knebplass enn flere konkurrenter i standard 5-seters oppsett. Revurdert: den opprinnelige vurderingen (3/5) trakk ned for at den faktiske 4-seters skyvesetekonverteringen (+3200 kr, jf. forhandlerkvitteringen) "koster bilen dens femte sete" og antok et behov for full 5-seters/barnesetekapasitet. Brukeren har presisert at dette er brukerens hovedbil uten barn i husstanden, og at skyvesetene ble bevisst valgt for å kunne prioritere enten voksne passasjerer (venner/familie) eller bagasjeplass etter behov - en reell fordel for akkurat denne bruksprofilen, ikke en mangel. ISOFIX-antall/plassering for EV2 ble ikke funnet i noen kilde, men er irrelevant for denne husstanden. Justert opp fra opprinnelig 3/5 til 4/5 (uendret MEDIUM konfidens - selve bagasjevolumet er fortsatt nest minst av de fem). [Kriterium W018]</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -28494,7 +28494,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Konfigurasjonsspesifikk endring: Den faktiske forhandlerkvitteringen for denne konfigurasjonen viser at kjøperen har valgt en 4-seters skyvesetekonvertering (+3200 kr) som tilleggsutstyr utover standard GT Line-utstyr. Dette omgjør baksetet fra en standard 3-seters benk til en 4-seters løsning der de to gjenværende baksetene kan skyves frem/tilbake for å prioritere enten knebplass eller bagasjeromsplass. Uavhengig anmeldelse (Autocar) bekrefter at en slik skyvbar bakbenk finnes i enkelte europeiske markeder (ikke i Storbritannia), og beskriver den som nyttig. Ulempen er at bilen dermed mister sitt femte sete - relevant for en "familiens hovedbil" dersom husstanden trenger full 5-seters kapasitet. Ingen kilde ble funnet som bekrefter ISOFIX-antall eller -plassering spesifikt for EV2 - forblir genuint ukjent, ikke antatt.</t>
+          <t>Konfigurasjonsspesifikk endring: Den faktiske forhandlerkvitteringen for denne konfigurasjonen viser at kjøperen har valgt en 4-seters skyvesetekonvertering (+3200 kr) som tilleggsutstyr utover standard GT Line-utstyr. Dette omgjør baksetet fra en standard 3-seters benk til en 4-seters løsning der de to gjenværende baksetene kan skyves frem/tilbake for å prioritere enten knebplass til voksne passasjerer (venner/familie) eller bagasjeromsplass, alt etter behov. Eieren har ingen barn i husstanden, så dette er en bevisst, aktiv tilpasning til faktisk bruksmønster - ikke et tap av nødvendig kapasitet. Uavhengig anmeldelse (Autocar) bekrefter at en slik skyvbar bakbenk finnes i enkelte europeiske markeder (ikke i Storbritannia), og beskriver den som nyttig. ISOFIX-antall/plassering for EV2 ble ikke funnet i noen kilde, men er ikke utslagsgivende for denne husstanden.</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">

</xml_diff>

<commit_message>
Revise Skoda and Volvo W018 reasoning for no-children household
Following the Kia W018 revision, re-examined Skoda's and Volvo's
reviews since both leaned on child-specific framing (ISOFIX point
count as a differentiator, "family use" language implying child-seat
capacity needs). Reworded both to focus on adult-passenger and cargo
flexibility instead, which is what actually matters for this
household. Neither score changes: Skoda's 5/5 already stood on its
boot/legroom/storage merits alone, and Volvo's 2/5 reflects a
genuinely small boot and rear seat tightness for adult passengers
that isn't specific to carrying children.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -24923,7 +24923,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Bagasjerom på 470 liter (1580 liter med nedfelte seter) er blant det største i klassen, og samme akselavstand som den større Enyaq gir uvanlig god benplass i baksetet til tross for en 160 mm kortere karosseri. ISOFIX-forankring er bekreftet i begge ytre baksetene og i forsetet - totalt tre punkter, mer enn både Tesla og Renault i denne sammenligningen. Simply Clever-detaljer (justerbar/delt hattehylle, isskrape, paraplyholder, kabeloppbevaring) understøtter hverdagsbruk ytterligere. Ingen vesentlige praktiske svakheter funnet for en familiebil med begrenset årlig kjørelengde. [Kriterium W018]</t>
+          <t>Bagasjerom på 470 liter (1580 liter med nedfelte seter) er blant det største i klassen, og samme akselavstand som den større Enyaq gir uvanlig god benplass i baksetet til tross for en 160 mm kortere karosseri - svært godt egnet til å frakte voksne passasjerer (venner/familie), ikke bare barn. Simply Clever-detaljer (justerbar/delt hattehylle, isskrape, paraplyholder, kabeloppbevaring) understøtter hverdagsbruk ytterligere. Revurdert: den opprinnelige vurderingen fremhevet ISOFIX-forankring i tre punkter (begge ytre bakseter + forsetet) som en sentral fordel sammenlignet med konkurrentene. Brukeren har presisert at det ikke er barn i husstanden, så ISOFIX-antallet er ikke utslagsgivende for denne beslutningen - det registreres fortsatt som et faktum, men er ikke lenger en del av begrunnelsen for scoren. Scoren forblir uendret på 5/5: den generøse bagasjeplassen, det eksepsjonelt gode benrommet for voksne passasjerer, og Simply Clever-detaljene er alene nok til å begrunne toppscore, uten at ISOFIX trengs som argument. Ingen vesentlige praktiske svakheter funnet. [Kriterium W018]</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -24963,7 +24963,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Bagasjerommet på 318 liter er det minste av de fem konfigurasjonene i denne sammenligningen, selv om det kan utvides til rundt 900-1000 liter med nedfelte seter (40/60-delt) pluss et 61-liters rom under lastegulvet. ISOFIX-forankring finnes kun i de ytre baksetene, ikke i forsetet. Uavhengige anmeldere beskriver baksetet som trangt for fot- og knehøyde ved en høyere fører og anbefaler bilen fremst for sporadisk bruk eller mindre familier - i direkte motsetning til Volvos egen, mer positive omtale av baksetet. Denne uenigheten er dokumentert, ikke løst. Samlet den svakeste praktiske pakken av de fem for en "familiens hovedbil"-rolle, til tross for lav estimert årlig kjørelengde. [Kriterium W018]</t>
+          <t>Bagasjerommet på 318 liter er det minste av de fem konfigurasjonene i denne sammenligningen, selv om det kan utvides til rundt 900-1000 liter med nedfelte seter (40/60-delt) pluss et 61-liters rom under lastegulvet. Uavhengige anmeldere beskriver baksetet som trangt for fot- og knehøyde ved en høyere fører - en fysisk plassbegrensning som gjelder voksne passasjerer generelt (venner/familie), ikke spesifikt barn - og konkluderer at bilen passer best til sporadisk bruk med full passasjerlast, i direkte motsetning til Volvos egen, mer positive omtale av samme baksete. Denne uenigheten er dokumentert, ikke løst. Revurdert: den opprinnelige vurderingen la også vekt på at ISOFIX kun finnes i de ytre baksetene (ikke forsetet) som et minuspunkt, og brukte "familiebruk"-språk som antydet et behov for barnesetekapasitet. Brukeren har presisert at det ikke er barn i husstanden, så ISOFIX-antallet er ikke utslagsgivende. Scoren forblir likevel uendret på 2/5: det minste bagasjerommet av de fem og en dokumentert, fra flere uavhengige kilder bekreftet trang baksete for voksne passasjerer er reelle, barneuavhengige svakheter for en bil som skal kunne frakte voksne venner/familie og bagasje regelmessig. Fortsatt den svakeste praktiske pakken av de fem. [Kriterium W018]</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -28359,7 +28359,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Barnesikring og Simply Clever-løsninger: Uavhengig anmeldelse bekrefter ISOFIX-forankring i begge ytre baksetene, samt i forsetet (passasjersetet) - totalt tre monteringspunkter, mer enn de fleste konkurrenter. Baksetet er beskrevet som flatt nok til at også en voksen kan sitte komfortabelt i midten. Hattehyllen kan plasseres i to ulike høyder for å dele opp bagasjerommet, og Simply Clever-detaljer som isskrape i bakluken og paraplyholder i førerdøren understøtter hverdagsbruk.</t>
+          <t>Simply Clever-løsninger: Uavhengig anmeldelse bekrefter ISOFIX-forankring i begge ytre baksetene samt i forsetet (tre punkter totalt) - et faktum registrert for fullstendighetens skyld, men ikke utslagsgivende for denne husstanden uten barn. Mer relevant her: baksetet er beskrevet som flatt nok til at også en voksen kan sitte komfortabelt i midten, noe som gjør bilen godt egnet til å frakte voksne passasjerer (venner/familie). Hattehyllen kan plasseres i to ulike høyder for å dele opp bagasjerommet, og Simply Clever-detaljer som isskrape i bakluken og paraplyholder i førerdøren understøtter hverdagsbruk uavhengig av passasjertype.</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -28413,7 +28413,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Baksete og barnesikring: Uavhengig anmeldelse beskriver plassen bak som trang for fot- og knehøyde dersom føreren er over gjennomsnittlig høy, og bemerker at det kan være vanskelig å montere et stort barnesete bak. ISOFIX-forankring er kun tilgjengelig i de ytre baksetene, ikke i forsetet. Anmeldelsen gir bagasjerom/praktisk bruk en score på 3,0 av 5 og konkluderer med at baksetet egner seg for sporadisk bruk fremfor jevnlig familiebruk.</t>
+          <t>Baksete: Uavhengig anmeldelse beskriver plassen bak som trang for fot- og knehøyde dersom føreren er over gjennomsnittlig høy - en fysisk plassbegrensning som gjelder voksne passasjerer generelt, uavhengig av om husstanden har barn. ISOFIX-forankring er kun tilgjengelig i de ytre baksetene, ikke i forsetet - registrert for fullstendighetens skyld, men ikke utslagsgivende for denne husstanden uten barn. Anmeldelsen gir bagasjerom/praktisk bruk en score på 3,0 av 5 og konkluderer med at baksetet egner seg best for sporadisk bruk med full passasjerlast fremfor jevnlig bruk med flere voksne om bord.</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">

</xml_diff>

<commit_message>
Clarify Review ownership boundary vs Scoring (ADR-008)
ARCH-008 found Review/Scoring separation structurally sound - Review.Score
(1-5 conclusion) is correctly distinct from Scoring's weight/normalization/
total-score, and Category never drifts from its linked Criterion across all
100 Reviews checked. Two small gaps remained: entity-model.md's Review Owns
list omitted score entirely, contradicting ADR-005; and two Review Summaries
(REV_000007, REV_000041) restated Criterion Weight and Hard-Requirement
pipeline status in prose instead of pointing to where that already lives.
Fixes both, adds a documented convention against the pattern recurring, and
corrects lingering ASCII-substituted diacritics in the two reworded cells.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -8232,7 +8232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8892,6 +8892,43 @@
       <c r="G18" t="inlineStr">
         <is>
           <t>Migrated 145 existing Technical rows: TechnicalField values converted from free text to 17 canonical TechnicalFieldID codes; Qualifier populated for the 5 known measurement-condition variants. Deleted 6 orphaned FrameworkVersion-1.0 template rows (no Vehicle/Configuration reference, no Value, no Source) that violated the Technical referential-integrity rule. No measured value was altered - reformatting only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DEC_ADR_008</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Reworded REV_000007 and REV_000041 to remove weight/pipeline-eligibility reasoning (ADR-008)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ARCH-008 found these two Review Summaries restating Criterion Weight (W020) and Hard-Requirement/pipeline status (W019, Tesla M002) in prose - information that already has a queryable home in 01_Criteria.Weight and 11_DecisionLog/12_OverallScores.Notes respectively.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Score, Confidence, Category, EvidenceID and FrameworkVersion unchanged for both rows - wording correction only, not a re-evaluation. entity-model.md's Review Owns list also corrected to include score, reconciling it with ADR-005 and workbook-schema.md.</t>
         </is>
       </c>
     </row>
@@ -21664,7 +21701,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Offisiell spesifikasjon viser 250 kW DC-hurtiglading (opptil 282 km pa 15 minutter) og 13,6 kWh/100km forbruk for denne konfigurasjonen - godt over minimumsbehovet gitt lav estimert arlig kjorelengde (~8000 km/ar), men ladehastighet er uansett lavt vektet i denne kriteriemodellen. [Kriterium W020]</t>
+          <t>Offisiell spesifikasjon viser 250 kW DC-hurtiglading (opptil 282 km på 15 minutter) og 13,6 kWh/100km forbruk for denne konfigurasjonen - godt over minimumsbehovet gitt lav estimert årlig kjørelengde (~8000 km/år). [Kriterium W020]</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -23024,7 +23061,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Lengde 4720mm OVERSKRIDER 4500mm-grensen med 220mm. Denne konfigurasjonen oppfyller ikke engang minstekravet (M002), langt mindre gir den margin utover det. Laveste mulige score, og et symptom pa at denne konfigurasjonen ikke skulle vaert vektet evaluert i utgangspunktet (se DecisionLog DEC_M002_VIOLATION). [Kriterium W019]</t>
+          <t>Lengde 4720mm OVERSKRIDER 4500mm-grensen (M002) med 220mm - konfigurasjonen oppfyller ikke minstekravet. Laveste mulige score for dette kriteriet. Se DecisionLog DEC_M002_VIOLATION for hvordan dette håndteres i evalueringen. [Kriterium W019]</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">

</xml_diff>

<commit_message>
Add Hard Requirement Result model (ADR-009)
ARCH-009 found every Hard Requirement fact (length, winter range, ACC,
rear camera) already existed as structured data in 04_Technical/05_Equipment,
but was never joined into a queryable PASS/FAIL/UNKNOWN answer - only Notes
prose, which had already missed the Tesla M002 violation for 8+ criteria and
left several configurations silently unassessed for M004/M005. Introduces
14_HardRequirementResults (contributor-authored like Review, not a pure
formula like Scoring - a naive threshold check on Renault 4 Techno's winter
range data would confidently misjudge a weak proxy measurement as a fail).
Backfills all 90 rows (18 configs x 5 criteria) from existing facts, and adds
Configuration.HardRequirementOverride to represent "confirmed FAIL kept for
comparison" (Tesla) distinctly from a default exclusion (Renault Evolution
Urban/Comfort). FrameworkVersion 1.5 -> 1.6.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -20,6 +20,7 @@
     <sheet name="11_DecisionLog" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="12_OverallScores" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="13_TechnicalFieldDefinitions" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="14_HardRequirementResults" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="Enum_Availability">'README'!$X$2:$X$6</definedName>
@@ -34,6 +35,7 @@
     <definedName name="Enum_FrameworkStatus">'README'!$AG$2:$AG$5</definedName>
     <definedName name="Enum_DecisionStatus">'README'!$AH$2:$AH$5</definedName>
     <definedName name="Validation_Boolean">'README'!$AI$2:$AI$3</definedName>
+    <definedName name="Enum_HardRequirementResult">'README'!$AJ$2:$AJ$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_Criteria'!$A$1:$J$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_Vehicles'!$A$1:$G$5</definedName>
@@ -272,7 +274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI13"/>
+  <dimension ref="A1:AJ13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -362,6 +364,11 @@
           <t>Validation_Boolean</t>
         </is>
       </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>Enum_HardRequirementResult</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -371,7 +378,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -432,6 +439,11 @@
       <c r="AI2" t="inlineStr">
         <is>
           <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -443,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -504,6 +516,11 @@
       <c r="AI3" t="inlineStr">
         <is>
           <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -571,6 +588,11 @@
       <c r="AH4" t="inlineStr">
         <is>
           <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
         </is>
       </c>
     </row>
@@ -8232,7 +8254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8929,6 +8951,43 @@
       <c r="G19" t="inlineStr">
         <is>
           <t>Score, Confidence, Category, EvidenceID and FrameworkVersion unchanged for both rows - wording correction only, not a re-evaluation. entity-model.md's Review Owns list also corrected to include score, reconciling it with ADR-005 and workbook-schema.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DEC_ADR_009</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Introduced 14_HardRequirementResults and Configuration.HardRequirementOverride (ADR-009)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ARCH-009 found every Hard Requirement fact (length, winter range, ACC, rear camera) already existed as structured data in 04_Technical/05_Equipment, but was never joined into a queryable PASS/FAIL/UNKNOWN answer - only Notes prose, which had already missed the Tesla M002 violation for 8+ criteria and left several Configurations silently unassessed for M004/M005.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Backfilled 90 rows (18 Configurations x 5 Hard Requirement criteria M001-M005) from existing Technical/Equipment facts and the judgment already recorded in Configuration Notes - no new research performed. Renault 4 Techno's M003 kept as UNKNOWN (not a naive FAIL) per the mismatched -trim/mild-conditions caveat already on record. HardRequirementOverride set TRUE for the 4 Tesla configurations (kept scored despite confirmed M002 FAIL, per the user's standing instruction), FALSE for all others.</t>
         </is>
       </c>
     </row>
@@ -9600,6 +9659,3625 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H91"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>HardRequirementResultID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ConfigurationID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CriterionID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>SourceID</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>FrameworkVersion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>HRR_000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HRR_000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HRR_000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HRR_000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HRR_000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_URBAN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>HRR_000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_COMFORT</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HRR_000007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HRR_000008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HRR_000009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HRR_000010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HRR_000011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_ESSENCE_60</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HRR_000012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HRR_000013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_85X</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HRR_000014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_RS</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>HRR_000015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>HRR_000016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>HRR_000017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>HRR_000018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>HRR_000019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4720mm overskrider 4500mm-grensen med 220mm (se DecisionLog DEC_M002_VIOLATION).</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>HRR_000020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4720mm overskrider 4500mm-grensen med 220mm (se DecisionLog DEC_M002_VIOLATION).</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>HRR_000021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4720mm overskrider 4500mm-grensen med 220mm (se DecisionLog DEC_M002_VIOLATION).</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>HRR_000022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4720mm overskrider 4500mm-grensen med 220mm (se DecisionLog DEC_M002_VIOLATION).</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>HRR_000023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_URBAN</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4140mm er godt innenfor 4500mm-grensen.</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PAGE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>HRR_000024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_COMFORT</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4140mm er godt innenfor 4500mm-grensen.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PAGE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>HRR_000025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4140mm er godt innenfor 4500mm-grensen.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PAGE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>HRR_000026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4140mm er godt innenfor 4500mm-grensen.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PAGE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>HRR_000027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4140mm er godt innenfor 4500mm-grensen.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PAGE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>HRR_000028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4140mm er godt innenfor 4500mm-grensen.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PAGE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>HRR_000029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_ESSENCE_60</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4488mm er innenfor 4500mm-grensen, men med kun 12mm margin - tett, men bestått.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_GLOBAL_TECHDATA</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>HRR_000030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4488mm er innenfor 4500mm-grensen, men med kun 12mm margin - tett, men bestått.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_GLOBAL_TECHDATA</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>HRR_000031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_85X</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4488mm er innenfor 4500mm-grensen, men med kun 12mm margin - tett, men bestått.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_GLOBAL_TECHDATA</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>HRR_000032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_RS</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4488mm er innenfor 4500mm-grensen, men med kun 12mm margin - tett, men bestått.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_GLOBAL_TECHDATA</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>HRR_000033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4233mm er godt innenfor 4500mm-grensen.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>SRC_VOLVO_NO_EX30_SPECS</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>HRR_000034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4233mm er godt innenfor 4500mm-grensen.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>SRC_VOLVO_NO_EX30_SPECS</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>HRR_000035</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4233mm er godt innenfor 4500mm-grensen.</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>SRC_VOLVO_NO_EX30_SPECS</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>HRR_000036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4065mm er godt innenfor 4500mm-grensen.</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>SRC_KIA_UK_SPECS_PDF</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>HRR_000037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>To vintertester funnet, men begge er upålitelige treff: en 2022-test brukte en utgått pre-facelift-generasjon, og en NAF-vintertest 2025 rapporterer 702km WLTP som ikke matcher noen av de fire registrerte Model 3-konfigurasjonene. Forblir reelt ukjent.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>HRR_000038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Ingen konfigurasjonsspesifikk vintertest vurdert for denne varianten; se TESLA_MODEL_3_LONG_RANGE_RWD for detaljert vurdering av tilgjengelige, men ikke-treffende, datapunkter.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>HRR_000039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Ingen konfigurasjonsspesifikk vintertest vurdert for denne varianten; se TESLA_MODEL_3_LONG_RANGE_RWD for detaljert vurdering av tilgjengelige, men ikke-treffende, datapunkter.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>HRR_000040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Ingen konfigurasjonsspesifikk vintertest vurdert for denne varianten; se TESLA_MODEL_3_LONG_RANGE_RWD for detaljert vurdering av tilgjengelige, men ikke-treffende, datapunkter.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>HRR_000041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_URBAN</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Ingen vintertest vurdert for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>HRR_000042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_COMFORT</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Ingen vintertest vurdert for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>HRR_000043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Eneste tilgjengelige datapunkt (elbil.no, Iconic-trim - samme drivverk, men annet utstyrsnivå) målte 287 km ved konstant 100 km/t i mildvær (5-7°C), ikke reell vinterkulde. Et bekymringsfullt signal, men ikke et bekreftet fall, siden testen verken matcher trim eller forhold.</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_RENAULT4_TEST</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>HRR_000044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Ingen egen vintertest; deler drivverk med Techno, hvor eneste tilgjengelige datapunkt er en usikker proxy (se RENAULT_4_TECHNO).</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>HRR_000045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Ingen egen vintertest; deler drivverk med Techno, hvor eneste tilgjengelige datapunkt er en usikker proxy (se RENAULT_4_TECHNO).</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>HRR_000046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Ingen egen vintertest; deler drivverk med Techno, hvor eneste tilgjengelige datapunkt er en usikker proxy (se RENAULT_4_TECHNO).</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>HRR_000047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_ESSENCE_60</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Ingen uavhengig vintertest funnet for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>HRR_000048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Ingen uavhengig vintertest funnet for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>HRR_000049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_85X</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Ingen uavhengig vintertest funnet for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>HRR_000050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_RS</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Ingen uavhengig vintertest funnet for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>HRR_000051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Ingen vintertest vurdert for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>HRR_000052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Ingen vintertest vurdert for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>HRR_000053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Uavhengig test (elbil.no, matchende Twin Performance/AWD-drivverk) estimerte ca. 338 km reell vinterrekkevidde (~-20°C), som komfortabelt består ~300 km-kravet.</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>SRC_ELBIL_VOLVO_EX30_WINTER</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>HRR_000054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Ingen uavhengig vintertest funnet - sannsynligvis fordi modellen er for ny til det norske markedet.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>HRR_000055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Bekreftet standard via offisiell Tesla-konfigurator.</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_DESIGN</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>HRR_000056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Ikke egen registrert utstyrssjekk for denne konfigurasjonen; anta ikke samme utstyrsnivå som TESLA_MODEL_3_LONG_RANGE_RWD uten bekreftelse.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>HRR_000057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Ikke egen registrert utstyrssjekk for denne konfigurasjonen; anta ikke samme utstyrsnivå som TESLA_MODEL_3_LONG_RANGE_RWD uten bekreftelse.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>HRR_000058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Ikke egen registrert utstyrssjekk for denne konfigurasjonen; anta ikke samme utstyrsnivå som TESLA_MODEL_3_LONG_RANGE_RWD uten bekreftelse.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>HRR_000059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_URBAN</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Evolution-trim har kun fartsholder med fast hastighet, ikke adaptiv cruisekontroll - bekreftet i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>HRR_000060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_COMFORT</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Evolution-trim har kun fartsholder med fast hastighet, ikke adaptiv cruisekontroll - bekreftet i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>HRR_000061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Intelligent cruise control multi target (adaptiv) bekreftet standard i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>HRR_000062</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Intelligent cruise control multi target (adaptiv) bekreftet standard i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>HRR_000063</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Intelligent cruise control multi target (adaptiv) bekreftet standard i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>HRR_000064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Intelligent cruise control multi target (adaptiv) bekreftet standard i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>HRR_000065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_ESSENCE_60</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Prediktiv adaptiv cruisekontroll bekreftet standard i offisiell prisliste.</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>HRR_000066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Prediktiv adaptiv cruisekontroll bekreftet standard i offisiell prisliste.</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>HRR_000067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_85X</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Prediktiv adaptiv cruisekontroll bekreftet standard i offisiell prisliste.</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>HRR_000068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_RS</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Prediktiv adaptiv cruisekontroll bekreftet standard i offisiell prisliste.</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>HRR_000069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Bekreftet tilstede via Motor.no sin test av denne konfigurasjonen (samme kjøreassistentpakke på tvers av rekken, om enn kritisert i vinterforhold).</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>SRC_MOTORNO_EX30_2024</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>HRR_000070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Ikke uavhengig bekreftet for denne spesifikke konfigurasjonen; utledet fra VOLVO_EX30_P8_AWD, som deler samme kjøreassistentpakke på tvers av rekken per Volvos egen produktbeskrivelse.</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>HRR_000071</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Ikke uavhengig bekreftet for denne spesifikke konfigurasjonen; utledet fra VOLVO_EX30_P8_AWD, som deler samme kjøreassistentpakke på tvers av rekken per Volvos egen produktbeskrivelse.</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>HRR_000072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Bekreftet standard i den itemiserte utstyrslisten fra forhandlerens salgstilbud.</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>HRR_000073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Bekreftet standard i Teslas egen brukerhåndbok.</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_OWNERSMANUAL_MODEL3_NO</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>HRR_000074</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_RWD</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Ikke egen registrert utstyrssjekk for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>HRR_000075</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_AWD</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Ikke egen registrert utstyrssjekk for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>HRR_000076</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Ikke egen registrert utstyrssjekk for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>HRR_000077</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_URBAN</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>HRR_000078</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>RENAULT_4_EVOLUTION_COMFORT</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>HRR_000079</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>HRR_000080</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>HRR_000081</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>HRR_000082</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>RENAULT_4_ICONIC_PLEIN_SUD</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i prislistens utstyrssammenligning.</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>HRR_000083</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_ESSENCE_60</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i offisiell prisliste.</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>HRR_000084</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i offisiell prisliste.</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>HRR_000085</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_85X</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i offisiell prisliste.</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>HRR_000086</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_RS</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i offisiell prisliste.</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>HRR_000087</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Ikke uavhengig bekreftet via en presist kildesporet henting - forblir bevisst ukjent fremfor antatt.</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>HRR_000088</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Ikke uavhengig bekreftet via en presist kildesporet henting - forblir bevisst ukjent fremfor antatt.</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>HRR_000089</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P8_AWD</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Ikke uavhengig bekreftet via en presist kildesporet henting - forblir bevisst ukjent fremfor antatt.</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>HRR_000090</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i den itemiserte utstyrslisten fra forhandlerens salgstilbud.</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>SRC_BOS_KIA_EV2_QUOTE</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>Enum_HardRequirementResult</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>Enum_Confidence</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11314,7 +14992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -11368,6 +15046,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>HardRequirementOverride</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -11400,6 +15083,11 @@
           <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002). HARD REQUIREMENT FAILED (M002): Official length is 4720mm, 220mm over the 4500mm maximum. Per docs/02_criteria-and-weighting.md, "Configurations failing a mandatory requirement shall not proceed to weighted evaluation." This was not caught until the length figure was cross-checked against M002 during Garasje (W019) scoring. Kept in the comparison table at the users explicit request so they can personally weigh the 220mm overage, but this configuration is NOT hard-requirement-compliant and all its existing Reviews/Scores/OverallScore should be read with that in mind.</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -11432,6 +15120,11 @@
           <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002). HARD REQUIREMENT FAILED (M002): Official length is 4720mm, 220mm over the 4500mm maximum. Per docs/02_criteria-and-weighting.md, "Configurations failing a mandatory requirement shall not proceed to weighted evaluation." This was not caught until the length figure was cross-checked against M002 during Garasje (W019) scoring. Kept in the comparison table at the users explicit request so they can personally weigh the 220mm overage, but this configuration is NOT hard-requirement-compliant and all its existing Reviews/Scores/OverallScore should be read with that in mind.</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -11470,6 +15163,11 @@
           <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002). M003 (winter highway range): Not verified. Two winter tests were found but both are unreliable matches: a 2022 test used a superseded pre-refresh Model 3 generation with a WLTP figure (614km) that matches no current trim, and a NAF winter 2025 test reports 702km WLTP (matching none of this workbook's four recorded Model 3 configurations) without specifying which trim was tested. Remains genuinely Unknown. Price verified 2026-07-06 via official Tesla Norway configurator (SRC_TESLA_NO_MODEL3_DESIGN): 400539 kr incl. VAT/fees, no optional extras selected (previously unpriced under DATA-001). HARD REQUIREMENT FAILED (M002): Official length is 4720mm, 220mm over the 4500mm maximum. Per docs/02_criteria-and-weighting.md, "Configurations failing a mandatory requirement shall not proceed to weighted evaluation." This was not caught until the length figure was cross-checked against M002 during Garasje (W019) scoring. Kept in the comparison table at the users explicit request so they can personally weigh the 220mm overage, but this configuration is NOT hard-requirement-compliant and all its existing Reviews/Scores/OverallScore should be read with that in mind.</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -11502,6 +15200,11 @@
           <t>Tesla Norway Model 3 page reviewed 2026-07-06: https://www.tesla.com/no_no/model3; official price not exposed in accessible source content. Configuration Status recorded as AVAILABLE: trim is listed on the official Tesla Norway configurator as of the same review date (ADR-004 / IMPL-002). HARD REQUIREMENT FAILED (M002): Official length is 4720mm, 220mm over the 4500mm maximum. Per docs/02_criteria-and-weighting.md, "Configurations failing a mandatory requirement shall not proceed to weighted evaluation." This was not caught until the length figure was cross-checked against M002 during Garasje (W019) scoring. Kept in the comparison table at the users explicit request so they can personally weigh the 220mm overage, but this configuration is NOT hard-requirement-compliant and all its existing Reviews/Scores/OverallScore should be read with that in mind.</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -11540,6 +15243,11 @@
           <t>Renault Norway official price list (Versjon 2, 01-06-2026) reviewed 2026-07-06. Fails Hard Requirement M004 (Adaptive Cruise Control): Evolution trim has only fixed-speed Cruise Control, not adaptive - confirmed in the price list equipment comparison table. Not eligible for weighted scoring.</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11578,6 +15286,11 @@
           <t>Renault Norway official price list (Versjon 2, 01-06-2026) reviewed 2026-07-06. Fails Hard Requirement M004 (Adaptive Cruise Control): Evolution trim has only fixed-speed Cruise Control, not adaptive - confirmed in the price list equipment comparison table. Not eligible for weighted scoring.</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11616,6 +15329,11 @@
           <t>Renault Norway official price list (Versjon 2, 01-06-2026) reviewed 2026-07-06. Meets all checked Hard Requirements (BEV, length 4140mm, Intelligent cruise control multi target = adaptive, standard rearview camera). M003 (winter highway range) remains Unknown - no winter test data reviewed. M003 (winter highway range): No dedicated deep-winter test found for this exact configuration. Closest available data point (elbil.no, Iconic trim - same 52kWh/150hk powertrain as Techno, but a different equipment level) measured 287 km at constant 100km/h highway driving in mild 5-7C conditions - NOT true winter cold. Since colder conditions would be expected to reduce range further, this data point is a concerning signal rather than a confident pass: the hard requirement remains genuinely uncertain, possibly at risk of failing, for this configuration. Flagged for the user's attention rather than resolved either way.</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11654,6 +15372,11 @@
           <t>Renault Norway official price list (Versjon 2, 01-06-2026) reviewed 2026-07-06. Shares Techno equipment level (adaptive cruise control, rearview camera); canvas soltak variant. M003 remains Unknown.</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11692,6 +15415,11 @@
           <t>Renault Norway official price list (Versjon 2, 01-06-2026) reviewed 2026-07-06. Meets all checked Hard Requirements (BEV, length 4140mm, Intelligent cruise control multi target = adaptive, standard rearview camera). M003 remains Unknown.</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11730,6 +15458,11 @@
           <t>Renault Norway official price list (Versjon 2, 01-06-2026) reviewed 2026-07-06. Shares Iconic equipment level (adaptive cruise control, rearview camera); canvas soltak variant. M003 remains Unknown.</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -11768,6 +15501,11 @@
           <t>Skoda Norway official price list (2027-modell, 29.06.2026) reviewed 2026-07-06. Meets all checked Hard Requirements: BEV, length 4488mm (only 12mm under the 4500mm limit - tight margin, flagged), Prediktiv adaptiv cruisekontroll standard, Ryggekamera standard. M003 (winter highway range) remains Unknown.</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -11806,6 +15544,11 @@
           <t>Skoda Norway official price list (2027-modell, 29.06.2026) reviewed 2026-07-06. Reportedly the most popular Elroq variant per Skoda. Meets all checked Hard Requirements (see Essence 60 note; same length/ACC/camera). M003 remains Unknown. M003 (winter highway range): Not verified. NAF's El Prix winter 2026 test included only the Elroq RS variant (different chassis/suspension/power tier), and the results table was rendered as an image, not extractable as text. Searched but found no dedicated winter test for Selection 60 specifically. Remains genuinely Unknown, not assumed.</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -11844,6 +15587,11 @@
           <t>Skoda Norway official price list (2027-modell, 29.06.2026) reviewed 2026-07-06. Meets all checked Hard Requirements (see Essence 60 note). M003 remains Unknown.</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -11882,6 +15630,11 @@
           <t>Skoda Norway official price list (2027-modell, 29.06.2026) reviewed 2026-07-06. Meets all checked Hard Requirements (see Essence 60 note). M003 remains Unknown.</t>
         </is>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -11920,6 +15673,11 @@
           <t>Volvo Norway official specifications page reviewed 2026-07-06. Meets checked Hard Requirements: BEV, length 4233mm (comfortable margin under 4500mm limit), adaptive cruise control confirmed present via Motor.no test of the P8 AWD (same driver-assistance suite across the range, though functionally criticized in winter conditions). Rearview camera standard equipment not independently confirmed via a precisely-sourced fetch - left Unknown rather than assumed. M003 (winter highway range) remains Unknown.</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -11958,6 +15716,11 @@
           <t>Volvo Norway official specifications page reviewed 2026-07-06. Same Hard Requirement notes as P5 (see above).</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -11996,6 +15759,11 @@
           <t>Volvo Norway official specifications page reviewed 2026-07-06. Same Hard Requirement notes as P5. This is the configuration actually tested by Motor.no (Evidence directly applicable, not inferred across trims). M003 (winter highway range): Independent test (elbil.no, matching Twin Performance/dual-motor AWD powertrain) estimated ~75% of the 450km WLTP figure retained in real winter conditions (~-20C), i.e. approximately 338 km. This comfortably passes the ~300km hard requirement.</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -12034,15 +15802,23 @@
           <t>Official Bertel O. Steen (Kia dealer) sales quote reviewed 2026-07-06, valid to 2026-07-12. BasePrice (346417 kr) = base EV2 FWD Long Range (251655 kr) + GT Line package (94762 kr), i.e. the trim as sold. ConfiguredPrice (423340 kr) = this specific quote total, which additionally includes buyer-selected options not part of the base GT Line trim: 4-seat sliding-seat conversion (+3200 kr), 16" Nokian studded winter wheels (+23603 kr), plus delivery (12500 kr), VAT (21430 kr) and registration tax/vrakpant (16190 kr). Colour (Frost Blue - Solid) and interior (Grey/Black) were no-cost selections. No battery capacity, WLTP range, charging power, or vehicle dimensions were stated in the source document - these remain Unknown pending a manufacturer specification sheet. M003 (winter highway range): Not verified. No independent winter test was found for the Kia EV2 - likely because the model is too new to the Norwegian market to have been included in a winter test cycle yet. Remains genuinely Unknown.</t>
         </is>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Enum_Market</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Enum_ConfigurationStatus</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>Validation_Boolean</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add Source.Language and document Type-to-Tier mapping (ADR-012)
ARCH-012 found PublishedDate/RetrievedDate already existed on 09_Sources -
RetrievedDate 100% populated, PublishedDate correctly sparse for
continuously-updated manufacturer pages but under-captured for dated
professional-review articles (the same staleness risk that required manual
detection during Tesla's M003 investigation). Language was genuinely missing:
the data shows a real 38/46/3 NB/EN/OTHER split, not a hypothetical one.
Adds Language + a small enum, backfilled individually for all 87 sources
from their own URL/publisher. Documents the existing Type enum's mapping
onto the Evidence Policy's Tier A/B/C hierarchy in docs/02 instead of adding
a redundant Tier column. Also corrects 09_Sources' Referenced By list, which
was missing 14_HardRequirementResults since ADR-009. FrameworkVersion
1.7 -> 1.8.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -37,6 +37,7 @@
     <definedName name="Validation_Boolean">'README'!$AI$2:$AI$3</definedName>
     <definedName name="Enum_HardRequirementResult">'README'!$AJ$2:$AJ$4</definedName>
     <definedName name="Enum_VersionBumpType">'README'!$AK$2:$AK$4</definedName>
+    <definedName name="Enum_Language">'README'!$AL$2:$AL$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_Criteria'!$A$1:$J$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_Vehicles'!$A$1:$G$5</definedName>
@@ -275,7 +276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK13"/>
+  <dimension ref="A1:AL13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -375,6 +376,11 @@
           <t>Enum_VersionBumpType</t>
         </is>
       </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>Enum_Language</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -384,7 +390,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -455,6 +461,11 @@
       <c r="AK2" t="inlineStr">
         <is>
           <t>SCHEMA</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>NB</t>
         </is>
       </c>
     </row>
@@ -466,7 +477,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -537,6 +548,11 @@
       <c r="AK3" t="inlineStr">
         <is>
           <t>METHODOLOGY</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>EN</t>
         </is>
       </c>
     </row>
@@ -614,6 +630,11 @@
       <c r="AK4" t="inlineStr">
         <is>
           <t>NONE</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>OTHER</t>
         </is>
       </c>
     </row>
@@ -852,7 +873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -906,6 +927,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -943,6 +969,11 @@
           <t>Official Tesla Norway configurator/specification page. Technical values retrieved by switching between the Model 3 (RWD), Premium (Long Range AWD / Long Range RWD) and Performance trim tabs on the live page.</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -980,6 +1011,11 @@
           <t>Test av Tesla Model 3 Long Range firehjulsdrift (AWD). Dekker kupestoy, komfort, styring og sikt.</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1022,6 +1058,11 @@
           <t>Test av Tesla Model 3 Long Range. Dekker NVH/stoydemping, fjaering og infotainment-betjening.</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1064,6 +1105,11 @@
           <t>Rapporterer status og planer for Apple CarPlay-stotte pa Tesla-kjoretoy, inkludert Model 3.</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1101,6 +1147,11 @@
           <t>Official Renault Norway product page. Dimensions, boot volume (evolution default view), ground clearance, driver-assistance feature list, CarPlay/Android Auto support.</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1143,6 +1194,11 @@
           <t>Official Norwegian price list PDF. Per-trim WLTP range, consumption, motor power, torque, DC/AC charging, kerb weight, payload, pricing, and full equipment/feature comparison including adaptive cruise control availability by trim.</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1180,6 +1236,11 @@
           <t>Test av Renault 4 E-Tech 150 Comfort Range (52 kWh, 150 hk). Dekker fjaering/komfort, sikt og infotainment.</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1217,6 +1278,11 @@
           <t>UK professional review. Covers steering, cabin/road noise, ride comfort, and confirms Apple CarPlay/Android Auto support on all models.</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1254,6 +1320,11 @@
           <t>Official Skoda Norway product page. General range/boot/pricing highlights and feature descriptions.</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1296,6 +1367,11 @@
           <t>Official Norwegian price list, 2027 model year, dated 29.06.2026. Per-trim range, consumption, system power, DC charge time, pricing, and full equipment comparison including adaptive cruise control and rearview camera standard on all trims.</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1338,6 +1414,11 @@
           <t>Official global technical data sheet (5.5.2025 revision). Used only for physical dimensions (length, width, height, wheelbase, ground clearance, boot volume) not covered by the Norway 2027 price list. Note: this sheet predates the Norway 2027-model price list by roughly a model year; power/battery/range figures in this sheet do not match the Norway 2027 price list exactly (e.g. Elroq 60: 150kW/59kWh global vs 140kW/58kWh NO 2027) - a documented cross-source discrepancy, likely a running spec revision between model years. Norway price list figures are used for all range/power/battery/charging facts; this sheet is used only for dimensions.</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1375,6 +1456,11 @@
           <t>Test av Skoda Elroq 60 med Motor-pakke. Dekker kupestoy (hjulstoy), fjaering, og betjening/infotainment.</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1412,6 +1498,11 @@
           <t>UK professional review. Covers CarPlay/infotainment, steering, ride comfort and cabin noise.</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1449,6 +1540,11 @@
           <t>UK professional review. Covers outward visibility and driving position.</t>
         </is>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1486,6 +1582,11 @@
           <t>Official Volvo Norway specifications page. Per-configuration (P5, P5 Long Range, P8 AWD) power, torque, range, consumption, battery, charging, weights, plus full vehicle dimensions.</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1523,6 +1624,11 @@
           <t>Test av Volvo EX30 P8 AWD (64 kWh, 428 hk). Dekker kupestoy, fjaering, rattbetjening, infotainment, og forerassistenter pa norske vinterveier.</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1560,6 +1666,11 @@
           <t>UK professional review. Covers CarPlay, steering, ride comfort, cabin noise, and outward visibility.</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1597,6 +1708,11 @@
           <t>Official dealer sales quote (PDF), valid to 2026-07-12. Covers configuration, trim/equipment list, and full pricing breakdown for the specific GT Line configuration. No battery/range/charging/dimension figures included. Customer contact details in the source document deliberately excluded from this citation.</t>
         </is>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1634,6 +1750,11 @@
           <t>Official Kia Norway configurator, saved configuration code A2231F29 (verified directly by fetching the live page 2026-07-06 - matches text supplied by user exactly). Technical data section contains confirmed unit-label errors on Kia's own page template: "Bagasjerom"/"Frunk" labeled kg (should be L, volume), "Forbruk" labeled kWh/km (should be kWh/100km - confirmed by cross-check: 62kWh battery / 15.2kWh-per-100km implies ~408km range, consistent with the stated 453km WLTP figure; taken literally as kWh/km the range would be ~4km, which is physically absurd), "Batterikapasitet" labeled kW (should be kWh, energy not power - same cross-check applies). Numeric values are trusted (official source, tied to a specific saved configuration); unit labels corrected based on physical plausibility and internal arithmetic consistency, not assumed.</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1671,6 +1792,11 @@
           <t>Test av Kia EV2 Standard Range (42.2 kWh, 147 hk), testet i Lisboa. Dekker fjaering/komfort og sikt.</t>
         </is>
       </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1708,6 +1834,11 @@
           <t>UK professional review. Covers CarPlay, steering, ride comfort, cabin noise and outward visibility.</t>
         </is>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1745,6 +1876,11 @@
           <t>UK professional review. Covers infotainment/touchscreen quality.</t>
         </is>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1787,6 +1923,11 @@
           <t>Independent winter test (Tier A: independent winter testing). Tested Twin Performance (dual-motor AWD Ultra) - matches VOLVO_EX30_P8_AWD powertrain. Estimated ~75% of WLTP range retained under real winter conditions (down to approx. -20C) after accounting for a mid-route fast-charge stop.</t>
         </is>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1829,6 +1970,11 @@
           <t>General road test, not a dedicated winter cold-chamber test. Tested Iconic trim (52kWh, same powertrain as Techno, different equipment level) at highway consumption of 1.81 kWh/mil (18.1 kWh/100km) at constant 100km/h in 5-7C conditions - not extreme winter cold. Measured range at this consumption: 287km. Used as a cautious proxy only, explicitly flagged as trim- and condition-mismatched to the Techno configuration and to true deep-winter conditions.</t>
         </is>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1866,6 +2012,11 @@
           <t>Official Tesla Norway configurator. Verified total price for Long Range bakhjulsdrift (Long Range RWD) with no optional extras selected: 369990 kr excl. VAT/fees, 400539 kr incl. VAT and fees.</t>
         </is>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1903,6 +2054,11 @@
           <t>Official Kia UK specifications PDF. GT Line/GT Line S trim: Length 4065mm, Wheelbase 2565mm, Width 1800mm, Height 1585mm. UK market document, not Norway-specific, but physical dimensions are not expected to differ by market for the same generation/trim.</t>
         </is>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1940,6 +2096,11 @@
           <t>Official Tesla owner's manual, camera/parking section. Confirms rear-view camera plus side-pillar camera views, no stitched 360-degree/bird's-eye composite view.</t>
         </is>
       </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1982,6 +2143,11 @@
           <t>Reports Tesla removing 'Basic Autopilot' (TACC+Autosteer bundle) from new North American orders in Jan 2026, later expanded to EU markets (Netherlands May 2026; one-time FSD purchase deadline May 21 2026 per follow-up Electrek coverage). Corroborates the paywall pattern later self-verified on Tesla's own Norwegian configurator (SRC_TESLA_NO_MODEL3_DESIGN).</t>
         </is>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2019,6 +2185,11 @@
           <t>Official Tesla guidance warning that Traffic-Aware Cruise Control/Autopilot should not be used on icy or slippery road surfaces. Generic safety boilerplate, not Norway-specific or comparative to other manufacturers.</t>
         </is>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2056,6 +2227,11 @@
           <t>Anecdotal, mixed user reports on standard Autopilot/TACC behavior on Norwegian winter roads - some describe it as reliable in winter conditions, others report late reactions on icy side roads. Forum anecdote only, not editorial/independent testing.</t>
         </is>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2093,6 +2269,11 @@
           <t>Official Renault Group article confirming Firmware-Over-The-Air (FOTA) update capability via embedded 4G, no workshop visit required. Applies to OpenR Link-equipped models including Renault 4 E-Tech.</t>
         </is>
       </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2135,6 +2316,11 @@
           <t>Independent corroboration of a real, dated shipped OTA update: Google Gemini AI assistant rolled out free to all OpenR Link-equipped models starting mid-June 2026, no workshop visit required.</t>
         </is>
       </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2177,6 +2363,11 @@
           <t>Review of the '60 Select' trim, the closest export-market analog to the Norwegian Selection 60. Confirms Connected Services (incl. OTA updates) is not standard on this trim, praises Travel Assist/ACC quality, and confirms rear-view-only camera as standard with 360-degree Area View reserved for higher trims/packages. Not Norway-specific.</t>
         </is>
       </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2214,6 +2405,11 @@
           <t>Norwegian test of the Skoda Elroq 60. Brief general endorsement of driver-assist systems ('holder orden i sysakene hvis du blir overivrig') - no dedicated winter-specific ACC deep-dive.</t>
         </is>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2251,6 +2447,11 @@
           <t>Reports Volvo pushed its largest-ever OTA update to ~2.5 million vehicles (EX30 included), reworking the UX, with Google Gemini-based conversational AI planned via a further OTA.</t>
         </is>
       </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2288,6 +2489,11 @@
           <t>Reports the EX30 launched with severe software bugs (black screens, keyless-entry failures, reported power loss), serious enough that UK customers exercised consumer-rights returns; Volvo spent roughly a year patching issues via OTA.</t>
         </is>
       </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2325,6 +2531,11 @@
           <t>Confirms 360-degree camera, automatic parking assist, panoramic roof, and powered seats/lumbar are Ultra-trim-exclusive, not included on Plus.</t>
         </is>
       </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2362,6 +2573,11 @@
           <t>Independently corroborates that at the Twin Performance AWD powertrain, Plus trim (468,900 NOK) excludes the 360-degree camera/Park Pilot, which is only added at Ultra trim (~505,900 NOK) for the same powertrain.</t>
         </is>
       </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2404,6 +2620,11 @@
           <t>Official Kia OTA update notice. Applicable models explicitly listed: Carnival (25MY), EV3 (MY25), EV6 PE (MY25), EV6 GT (New Facelift MY25+), EV9 (MY24-MY25), Sorento variants (MY25). EV2, EV4, EV5 are NOT listed as recipients of this update.</t>
         </is>
       </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2446,6 +2667,11 @@
           <t>Press release describing a substantive, feature-adding OTA update to the EV3 (AI voice assistant, YouTube streaming, Wi-Fi hotspot - 18 changes total), demonstrating the shared ccNC platform's OTA capability goes beyond bug fixes.</t>
         </is>
       </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2483,6 +2709,11 @@
           <t>Confirms OTA ('Trådløs programvareoppdateringer') is available on the EV2, without further track-record commentary. Also references a Surround View Monitor ambiguously ('også tilgjengelig') without clearly stating standard vs optional status.</t>
         </is>
       </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2525,6 +2756,11 @@
           <t>Official Euro NCAP assisted-driving assessment of the EV3 (closest platform/software sibling to EV2), rated 'Very Good' overall. Steering Assistance 'Excellent' (35/35): maintains lane position effectively at 80/100/120 km/h. Adaptive Cruise Control 'Adequate' (25.3/40): scores lower on undertake prevention and cut-in situations.</t>
         </is>
       </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2562,6 +2798,11 @@
           <t>EV2-specific Danish test. Direct quote: 'bilen kan selv foretage vognbaneskift på motorvejen, og begge dele fungerer rigtig godt' (the car can change lanes itself on the motorway, and both functions work very well).</t>
         </is>
       </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2599,6 +2840,11 @@
           <t>EV2-specific Danish test. Notes the adaptive cruise/lane-assist system 'holder usædvanligt hårdt i rattet' (holds unusually firmly on the wheel), requiring deliberate steering input to override - an over-intervention complaint, not a performance failure.</t>
         </is>
       </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2636,6 +2882,11 @@
           <t>Official Tesla Norway warranty page. Direct fetch returned HTTP 403; terms corroborated via search-result synthesis (4 års/80 000 km generell nybilgaranti, 8 års batterigaranti med garantert minst 70 % kapasitet, 12 års rustgjennomtæringsgaranti uten kilometergrense). Bør verifiseres direkte ved behov for presisjon.</t>
         </is>
       </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2673,6 +2924,11 @@
           <t>Nyhetsdekning av offisiell registreringsstatistikk fra OFV (Opplysningsrådet for Veitrafikken). Model 3 var Norges mest solgte bilmodell i 2020 og 2021 (over 12 000 solgte i 2021 alene), og over 60 000 eksemplarer er i dag registrert i Norge; OFV-tall for november 2025 viser 2 562 nyregistrerte Model 3 i den ene måneden alene.</t>
         </is>
       </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2710,6 +2966,11 @@
           <t>Dansk Renault-garantiside. Beskriver en paneuropeisk garantiendring fra mai 2025: 5 år/150 000 km generell garanti på alle nye elektriske Renault-modeller, samt 8 år/160 000 km batterigaranti (minst 70 % SOH garantert). Ikke uavhengig bekreftet på en norsk Renault-side; behandlet som MEDIUM-konfidens for det norske markedet.</t>
         </is>
       </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2747,6 +3008,11 @@
           <t>Offisiell Renault Norge-produktside bekrefter at 4 E-Tech Electric kommer tilbake for 2025 som en helelektrisk modell ("tilbake i 2025, 100 % elektrisk"); eksakt norsk lanseringsdato er ikke oppgitt på selve siden. Samlet søkeresultat (ikke uavhengig reverifisert) plasserer markedstilgjengelighet til høsten 2025.</t>
         </is>
       </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2784,6 +3050,11 @@
           <t>Offisiell Skoda Norge-garantiside, hentet direkte. "5 års Norgesgaranti": 5 år/100 000 km generell garanti (biler førstegangsregistrert etter 2011-01-01, importert av Harald A. Møller AS). Alle nye ladbare hybrider og elbiler: 8 år/160 000 km batteripakkegaranti.</t>
         </is>
       </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2821,6 +3092,11 @@
           <t>Bekrefter at Elroq gikk i produksjon januar 2025 med de første kundeleveransene tidlig i 2025, etter å ha blitt vist frem på Paris Motor Show oktober 2024. Er den andre Skoda-modellen på Volkswagen-konsernets MEB-plattform, som deles med Enyaq, ID.3, ID.4/ID.5 og Audi Q4 e-tron.</t>
         </is>
       </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2858,6 +3134,11 @@
           <t>Offisiell Volvo Norge-garantiside. Direkte henting ga HTTP 403; vilkårene er bekreftet via søkeresultat-syntese (5 år/100 000 km generell garanti, opptil 8 år/160 000 km batterigaranti med garantert minst 70 % kapasitet). Bør verifiseres direkte ved behov for presisjon.</t>
         </is>
       </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2895,6 +3176,11 @@
           <t>Offisiell Kia Norge-garantiside, hentet direkte. 7 år/150 000 km generell garanti og batterigaranti for elbiler (kapasitetsgrense 65 % for biler registrert etter oktober 2019), utvidet til 8 år/160 000 km fra modellår 2026. Garantien overføres til neste eier.</t>
         </is>
       </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2932,6 +3218,11 @@
           <t>Offisiell Kia-pressemelding distribuert via NTB. Bekrefter produksjonsstart for alle EV2-batterialternativer 2026-06-25, og en oppfølgende pressemelding bekrefter at salget av EV2 formelt startet 2026-07-02 - få dager før denne vurderingen. GT Line tilbys blant de første variantene i salg.</t>
         </is>
       </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2969,6 +3260,11 @@
           <t>Dekker NAF/Motor sin årlige El Prix-vintertest, der Tesla Model 3 har deltatt hvert år siden 2020 med jevnt sterke resultater (WLTP-oppgitt rekkevidde økt fra 560 til 614 km over generasjoner; faktisk kjørt distanse har variert mellom ca. 521 og 548 km i ulike vintertester, gjennomgående blant de beste i klassen).</t>
         </is>
       </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3006,6 +3302,11 @@
           <t>Dokumenterer tilbakevendende svikt i varmepumpe/varmeelement på Renault Zoe (Renaults forrige generasjons elbil) etter 20 000-30 000 km, som kan redusere rekkevidden i kulde med opptil 40 %. Nyere generasjoner (R110/R135) med aktiv batteritemperaturstyring håndterer dette 'vesentlig bedre' enn de tidligste modellene. Gjelder en annen, eldre Renault-elbilplattform enn den helt nye Renault 4 (AmpR Small), men representerer Renaults dokumenterte merkehistorikk i nordisk kulde over tid.</t>
         </is>
       </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3043,6 +3344,11 @@
           <t>NAF/Motor sin vintertest fra januar 2022 inkluderte VW ID.4 og Skoda Enyaq (samme MEB-plattform som Elroq), samt Tesla Model 3/Model Y og Kia EV6. Konklusjonen for ID.4 var 'rekkevidden holder seg godt i kulde, selv om varmepumpen sliter litt på de kaldeste dagene' - blant flere modeller som kun tapte 11-15 % av WLTP-rekkevidden. Representerer flere års gjentatt, konsistent MEB-plattformytelse i norsk vinterklima, selv om Elroq Selection 60 ikke selv var inkludert i denne konkrete testen.</t>
         </is>
       </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3080,6 +3386,11 @@
           <t>NAF/Motor-vintertester av Kia e-Niro og EV6 viser sterk varmepumpeassistert kuldeytelse ('uvanlig behagelig i kulden'; e-Niro tapte kun rundt 10 % rekkevidde). EV6 gikk fra 481 til 341 km ved rundt -10°C, men rangerte likevel høyt, med varm kupé og upåvirket infotainmentskjerm selv i sterk kulde.</t>
         </is>
       </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3117,6 +3428,11 @@
           <t>En Kia EV2-prototyp (61 kWh Long Range) deltok i NAFs El Prix-vintertest i Norge, februar 2026, i temperaturer mellom -8°C og -31°C: kjørte 310,6 km, kun 24,8 % under WLTP-oppgitt rekkevidde - blant de beste i testfeltet. Hurtiglading 8 %→80 % på under 37 minutter (97 kW effekttopp, 74 kW snitt) selv i ekstrem kulde. Gjelder en produksjonsnær prototyp, ikke en levert kundebil.</t>
         </is>
       </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3154,6 +3470,11 @@
           <t>Bekrefter at Highland-oppdateringen (2024+) erstattet imitasjonstre-dashbordet med mykere plast/gummi, strukturerte flater, veganskinn og aluminium på midtkonsollen. Konkluderer at 'materialene er bedre, og tilpasning/finish er umiskjennelig forbedret' sammenlignet med tidligere generasjoner, samt at kupéen er merkbart roligere (opptil 20 % mindre kupéstøy).</t>
         </is>
       </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3191,6 +3512,11 @@
           <t>Beskriver Tesla Model 3 sin byggekvalitet som uforutsigbar fra bil til bil ('mange eiere rapporterer knirkefrie biler, andre en lang feilliste ved levering'). Knirk fra løse ledningsbunter, panelgap, sprekker fra bakre understell og vindstøy fra dører/glass er vanlige klager. Viser til at Consumer Reports vurderer 2025-modellens generelle pålitelighet under gjennomsnittet, med svakheter i karosseri-maskinvare (vinduer, dører, låser).</t>
         </is>
       </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3228,6 +3554,11 @@
           <t>Edmunds sin langtidstest av en 2024 Model 3 (Highland) konkluderer at de knappbaserte blinklysene er reelt utrygge, ikke bare uvante: 'Det er små knapper med små aktiveringsflater og ingen reell taktil forskjell mellom dem eller panelet de sitter på.' Hele testteamet var samstemte i at de mislikte løsningen etter flere måneders eierskap.</t>
         </is>
       </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3265,6 +3596,11 @@
           <t>Bekrefter at europeiske Model 3-biler (inkludert Highland-generasjonen levert i Norge) opprinnelig hadde samme knappbaserte blinklysløsning uten fysisk spak som i USA, og at en betalt ettermonteringsløsning (660 euro) først ble tilgjengelig i Europa fra rundt oktober 2025 - ikke standard inkludert i leveransen.</t>
         </is>
       </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3302,6 +3638,11 @@
           <t>Brukt som generisk referansepunkt for kriteriet W012 (Ergonomi/førermiljø), som eksplisitt ber om en vurdering mot Kia Rio. Edmunds beskriver Rio sin ergonomi som utmerket ('kontrollene er godt plassert, intuitive, med gammeldagse knapper og brytere'), men interiøret som spartansk med hard plast i flere flater ('plasten er noe hard og billig enkelte steder'). Brukes gjennomgående som lavterskel-referanse for 'et tydelig steg opp,' ikke som en direkte modellsammenligning.</t>
         </is>
       </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3339,6 +3680,11 @@
           <t>Beskriver interiøret som overraskende godt for prisklassen: harde plastdetaljer finnes, men er 'godt gjemt', og kvaliteten er 'svært god.' Stoffinnslag (inkludert quiltet tekstil med gul stikking på høyere nivåer) løfter det opplevde inntrykket - 'kun vesentlig dyrere konkurrenter oppleves mer luksuriøse innvendig.'</t>
         </is>
       </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3376,6 +3722,11 @@
           <t>Dokumenterer tidlige feilrapporter: knirk fra dashbordpaneler innen 10 000 km, fløyte-/summelyd fra klimaanleggets viftemotor rundt 5 000 km, mulig svikt i den motoriserte ladeportluken (~300 euro å reparere), og for tidlig utladning av 12V-hjelpebatteriet på enkelte tidlige 2024-eksemplarer (~150 euro). Bilen er for ny til at omfattende langtidsdata finnes.</t>
         </is>
       </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3413,6 +3764,11 @@
           <t>Langtidstestere rapporterer ingen knirk eller rangling etter over 4000 miles ('ikke et snev av skrapete plast eller irriterende knirk'), med fôrede dørlommer som forhindrer rangling. Ett testeksemplar hadde et elektrisk problem med vindusbryterne; søskenmodellen Enyaq har en rapportert 29 % andel mindre elektriske feil blant rapporterte feil.</t>
         </is>
       </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3450,6 +3806,11 @@
           <t>Beskriver forholdet mellom sete, pedaler og ratt som 'spot on' med en generelt utmerket kjørestilling, samt dedikerte fysiske hurtigknapper for kjøremodus, kjøreassistenter, klimaanlegg og parkeringssensorer under luftventilene - 'alltid betryggende enkle å finne' fremfor skjermmenyer eller haptiske/piano-sort-overflater.</t>
         </is>
       </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3487,6 +3848,11 @@
           <t>Roser kjøreegenskaper og ingeniørkunst, men bemerker at laveste utstyrsnivå har manuelt justerbare seter (ikke elektriske) og mangler enkelte teknologifunksjoner (bl.a. one-pedal-kjøremodus) som noen konkurrenter tilbyr.</t>
         </is>
       </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3524,6 +3890,11 @@
           <t>Ratt og hyppig berørte flater oppleves kvalitetsmessig gode, øvre dashbord (resirkulert plast) har en teksturert, granittlignende følelse, men skrapete plast finnes lenger ned og på dørpaneler. Beskriver et interiøralternativ ('Particle'-trim, laget av knuste PVC-vindusrammer) som en hard, skjør plast - kreativt, men ikke en tradisjonell kvalitetsopplevelse. Vindusbryterne er samlet på midtkonsollen fremfor på hver dør.</t>
         </is>
       </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3561,6 +3932,11 @@
           <t>Rapporterer spredte, ikke-kritiske knirk/rangling, feiljustert bakluke, vindtetningsproblemer og noe ekstra vindstøy - beskrevet som typisk førsteårs-støy. Viser til at Volvo i slutten av 2025 tilbakekalte over 40 000 EX30-biler globalt (69 kWh NMC-batteripakke, bygget 2024-2026) pga. moduler som kan overopphetes ved lading forbi ca. 70 % ladenivå. Mekanisk pålitelighet vurderes som 'god, men fortsatt umoden' - de fleste tidlige problemer er programvarerelaterte.</t>
         </is>
       </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3598,6 +3974,11 @@
           <t>Samler flere anmeldelser: setene og kjørestillingen får gjennomgående ros. Men fraværet av tradisjonelt instrumentpanel/head-up-display (all informasjon på sentralskjermen) trekkes frem som noe man må venne seg til, og flere anmeldelser peker på skjermavhengigheten som bilens klart største svakhet.</t>
         </is>
       </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3635,6 +4016,11 @@
           <t>Dokumenterer at fysiske knapper for grunnleggende funksjoner (sidespeiljustering, temperatur, seteputevarme, bakre tåkelys, hanskerom) er fjernet til fordel for skjermnavigering. Konkluderer at dette er en gjennomgående kritisert designbeslutning på tvers av nesten alle anmeldelser av bilen.</t>
         </is>
       </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3672,6 +4058,11 @@
           <t>Beskriver rikelig med hard plast som likevel oppleves 'godt sammenskrudd' og glatt, ikke grov og billig. GT-Line og GT-Line S får resirkulerte stoffinnlegg på dashbord/dørpaneler for et mer oppgradert preg; myke materialer dekker berøringspunkter som armlener.</t>
         </is>
       </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3709,6 +4100,11 @@
           <t>Fremhever byggekvalitet og tilpasning som en styrke sammenlignet med konkurrentene, uten vesentlige rapporter om knirk. Eneste konkrete innvending: koppholderne på midtkonsollen er upraktisk dimensjonert og rommer ikke vanlige flasker/bokser uten at de rasler rundt.</t>
         </is>
       </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3746,6 +4142,11 @@
           <t>Beskriver en høyere sitteposisjon enn typiske små elbiler, god utsikt takket være oppreiste dørstolper og høye vinduer, og et helelektrisk justerbart førersete med korsryggstøtte på GT-Line-utgaven som stemmer overens med ratt/pedaler.</t>
         </is>
       </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3783,6 +4184,11 @@
           <t>Oppsummerer pålitelighetsdata for Kias nylige elbilportefølje: EV6 (2022-2026 årsmodeller) har en gjennomsnittlig pålitelighetsscore på 75/100 (JD Power/Consumer Reports-baserte kilder), med tidlige modeller som hadde elektriske/drivverk-problemer, men betydelig forbedring fra 2025-årsmodellen. EV9 (større, mer kompleks 3-seters SUV) scorer lavere, 67/100, under gjennomsnittet for nye biler. EV2 er nærmere EV6/Niro EV i segment og kompleksitet enn EV9.</t>
         </is>
       </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3820,6 +4226,11 @@
           <t>Offisiell norsk brukerhåndbok, avsnitt om barnesikringsutstyr/ISOFIX. Bekrefter ISOFIX/i-Size-forankring i begge ytre baksetene, ingen ISOFIX-forankring i forsetet, og at beltebaserte barneseter kan monteres i alle passasjerseter.</t>
         </is>
       </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3857,6 +4268,11 @@
           <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Bekrefter 594 L bagasjerom bak + 88 L frunk (682 L kombinert, samsvarer med Teslas eget totaltall), flatt bakgulv uten sentertunnel, 60/40-delt nedfellbar rygglene, samt at sedan-bagasjeromsåpningen er mindre fleksibel enn en femdørs/stasjonsvogn og at baksetets kne-høye sittestilling oppleves noe ubehagelig på lengre turer.</t>
         </is>
       </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3894,6 +4310,11 @@
           <t>Norsk markedsartikkel som gjengir Renaults offisielle spesifikasjoner for Renault 4 E-Tech: bagasjerom på 420 liter (1405 liter med nedfelt baksete), 40/60-delt nedfellbar baksete, hands-free bakluke, lav terskel og bred åpning, samt 23,3 liter oppbevaringsplass i kupeen.</t>
         </is>
       </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3931,6 +4352,11 @@
           <t>Britisk profesjonell anmeldelse/spesifikasjonsside (ikke Norge-spesifikk). Bekrefter ISOFIX-forankring i begge ytre baksetene (tre ISOFIX-kompatible posisjoner totalt), 60/40-delt rygglene uten gjennomlastingsluke, samt at fotplassen bak er trang fordi batteriet stikker inn i fotrommet - ingen fotplass under forsetene. Noterer også at det mangler et to-nivås bagasjeromsgulv, som skaper et trinn ved nedfelte seter.</t>
         </is>
       </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3968,6 +4394,11 @@
           <t>Norsk markedsartikkel som gjengir Skodas offisielle spesifikasjoner for Elroq: bagasjerom på 470 liter (1580 liter med nedfelte seter), kabeloppbevaring under hattehyllen, og samme akselavstand som den større Enyaq til tross for 160 mm kortere karosseri, som gir svært god benplass i baksetet.</t>
         </is>
       </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4005,6 +4436,11 @@
           <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Bekrefter ISOFIX-forankring i begge ytre baksetene og i forsetet (tre punkter totalt), et flatt baksete som gir plass til en voksen midt bak, en hattehylle som kan plasseres i to høyder for å dele opp bagasjerommet, samt Simply Clever-detaljer (isskrape i bakluken, paraplyholder i førerdøren, hjørnehyller mot forskyvning av last).</t>
         </is>
       </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4042,6 +4478,11 @@
           <t>Offisiell norsk Volvo-støtteside. Direkte henting ga HTTP 403; innhold bekreftet via søkeresultat-syntese. Oppgir bagasjerom på 318 liter, utvidbart til opptil 1000 liter med nedfelte bakseter (40/60-delt), inkludert et eget rom på 61 liter under lastegulvet.</t>
         </is>
       </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4079,6 +4520,11 @@
           <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Oppgir 318 liter bagasjerom / 904 liter med nedfelte seter (60/40-delt) - noe lavere enn Volvos eget nedfelt-tall, trolig grunnet ulik målemetode. Beskriver baksetet som trangt for fot- og knehøyde ved en over gjennomsnittlig høy fører, bemerker at et stort barnesete kan være vanskelig å montere bak, og gir bagasjerom/praktisk bruk 3,0 av 5.</t>
         </is>
       </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4116,6 +4562,11 @@
           <t>Offisiell norsk Volvo-støtteside. Beskriver baksetet mer positivt enn uavhengige anmeldere: tilstrekkelig benplass til å strekke bena under forsetene, svært god hodeplass takket være panoramatak, komfortable seter med god korsryggstøtte, og plass til to barneseter eller to langbeinte voksne bak.</t>
         </is>
       </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4153,6 +4604,11 @@
           <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Bekrefter 362 liter bagasjerom pluss 15 liter frunk foran, en flyttbar falskbunn under lastegulvet, 60/40-delt rygglene med minimal terskel/trinn ved nedfelling, helt flatt gulv uten sentertunnel, bedre hodeplass enn Renault 4 og mer knebplass enn Jeep Avenger Electric - men trangt for tre voksne ved siden av hverandre bak.</t>
         </is>
       </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4190,12 +4646,20 @@
           <t>Britisk profesjonell anmeldelse (ikke Norge-spesifikk). Oppgir 362 liter bagasjerom (mot 420 liter i Renault 4), "fairly generous" hodeplass bak, og "just enough" knebplass for en 183 cm passasjer, med trang midtsete. Bekrefter at en 4-seters variant med skyvbar bakbenk finnes i enkelte europeiske markeder (ikke bekreftet for Storbritannia), beskrevet som "nyttig".</t>
         </is>
       </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Enum_SourceType</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>Enum_Language</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8275,7 +8739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9193,6 +9657,48 @@
       <c r="H22" t="inlineStr">
         <is>
           <t>NONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DEC_ADR_012</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Added 09_Sources.Language and documented Type-to-Tier mapping (ADR-012)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ARCH-012 found PublishedDate/RetrievedDate already existed (RetrievedDate 100% populated, PublishedDate correctly sparse for manufacturer pages but under-captured for professional reviews); Language did not exist and the data showed a real 31/56 no-domain/other split.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Backfilled Language for all 87 existing Sources from each row's own URL/Publisher - no new research performed. Documented the existing Type enum's mapping onto the Evidence Policy's Tier A/B/C hierarchy in docs/02 instead of adding a redundant Tier column.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>SCHEMA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix ASCII-substituted Norwegian diacritics in Reviews, Evidence and Sources
39 cells across 07_Reviews.Summary (24), 08_Evidence.Observation (9), and
09_Sources.Notes (6) had å/æ/ø typed as plain a/ae/oe, predating this
project's diacritics rule. Pure spelling correction - no wording, meaning,
Score, Confidence, or ID changed; URLs left untouched. Closes out the
architecture review's remaining loose end (previously tracked as a spawned
background task, now superseded).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -1055,7 +1055,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Test av Tesla Model 3 Long Range. Dekker NVH/stoydemping, fjaering og infotainment-betjening.</t>
+          <t>Test av Tesla Model 3 Long Range. Dekker NVH/støydemping, fjæring og infotainment-betjening.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Rapporterer status og planer for Apple CarPlay-stotte pa Tesla-kjoretoy, inkludert Model 3.</t>
+          <t>Rapporterer status og planer for Apple CarPlay-støtte på Tesla-kjøretøy, inkludert Model 3.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Test av Renault 4 E-Tech 150 Comfort Range (52 kWh, 150 hk). Dekker fjaering/komfort, sikt og infotainment.</t>
+          <t>Test av Renault 4 E-Tech 150 Comfort Range (52 kWh, 150 hk). Dekker fjæring/komfort, sikt og infotainment.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Test av Skoda Elroq 60 med Motor-pakke. Dekker kupestoy (hjulstoy), fjaering, og betjening/infotainment.</t>
+          <t>Test av Skoda Elroq 60 med Motor-pakke. Dekker kupestøy (hjulstøy), fjæring, og betjening/infotainment.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Test av Volvo EX30 P8 AWD (64 kWh, 428 hk). Dekker kupestoy, fjaering, rattbetjening, infotainment, og forerassistenter pa norske vinterveier.</t>
+          <t>Test av Volvo EX30 P8 AWD (64 kWh, 428 hk). Dekker kupestøy, fjæring, rattbetjening, infotainment, og førerassistenter på norske vinterveier.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Test av Kia EV2 Standard Range (42.2 kWh, 147 hk), testet i Lisboa. Dekker fjaering/komfort og sikt.</t>
+          <t>Test av Kia EV2 Standard Range (42.2 kWh, 147 hk), testet i Lisboa. Dekker fjæring/komfort og sikt.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -8739,7 +8739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9699,6 +9699,48 @@
       <c r="H23" t="inlineStr">
         <is>
           <t>SCHEMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DEC_DIACRITICS_001</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Corrected ASCII-substituted Norwegian diacritics across 07_Reviews, 08_Evidence and 09_Sources</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>33 Review/Evidence rows and 6 Source Notes rows had ASCII substitutes for Norwegian aa/ae/oe (e.g. plain a instead of å, ae instead of æ, oe instead of ø) predating the project's diacritics rule. Pure spelling correction - no wording, meaning, Score, Confidence, or ID changed.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>24 07_Reviews.Summary rows, 9 08_Evidence.Observation rows, 6 09_Sources.Notes rows corrected. URLs (containing 'no' as part of domain/path substrings) deliberately left untouched - they are real addresses, not prose.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>NONE</t>
         </is>
       </c>
     </row>
@@ -25953,7 +25995,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>To uavhengige profesjonelle tester (Motor.no, Cars.com) bekrefter betydelig redusert kupestoy i den oppgraderte Model 3-plattformen sammenlignet med tidligere arsmodeller; dekkstoy fremheves som blant de beste i klassen. Testet pa Long Range AWD/Long Range, men deler karosseri og lydisolasjon med Long Range bakhjulsdrift. [Kriterium W001]</t>
+          <t>To uavhengige profesjonelle tester (Motor.no, Cars.com) bekrefter betydelig redusert kupestøy i den oppgraderte Model 3-plattformen sammenlignet med tidligere årsmodeller; dekkstøy fremheves som blant de beste i klassen. Testet på Long Range AWD/Long Range, men deler karosseri og lydisolasjon med Long Range bakhjulsdrift. [Kriterium W001]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -25993,7 +26035,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Motor.no gir 8/10 for komfort og beskriver fjaeringen som behagelig ved hoyere hastighet; Cars.com bekrefter at det ikke oppstar bra stot takket vaere frekvensavhengige dempere. Testet pa AWD/Long Range-varianter; RWD-spesifikk fjaeringskarakter er ikke uavhengig bekreftet. [Kriterium W002]</t>
+          <t>Motor.no gir 8/10 for komfort og beskriver fjæringen som behagelig ved høyere hastighet; Cars.com bekrefter at det ikke oppstår brå støt takket være frekvensavhengige dempere. Testet på AWD/Long Range-varianter; RWD-spesifikk fjæringskarakter er ikke uavhengig bekreftet. [Kriterium W002]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -26033,7 +26075,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Motor.no rapporterer suveren sikt fremover, men darlig sikt bakover - sistnevnte er en reell praktisk ulempe ved manovrering. Kun en uavhengig kilde funnet. [Kriterium W003]</t>
+          <t>Motor.no rapporterer suveren sikt fremover, men dårlig sikt bakover - sistnevnte er en reell praktisk ulempe ved manøvrering. Kun en uavhengig kilde funnet. [Kriterium W003]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -26153,7 +26195,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MacRumors bekrefter at Apple CarPlay per undersokelsestidspunkt (juli 2026) fortsatt ikke stottes pa noen Tesla-modell, inkludert Model 3. Tesla har varslet tradlos CarPlay "i lopet av kommende maneder" (kunngjort november 2025), men uten bekreftet lanseringsdato. [Kriterium W007]</t>
+          <t>MacRumors bekrefter at Apple CarPlay per undersøkelsestidspunkt (juli 2026) fortsatt ikke støttes på noen Tesla-modell, inkludert Model 3. Tesla har varslet trådløs CarPlay "i løpet av kommende måneder" (kunngjort november 2025), men uten bekreftet lanseringsdato. [Kriterium W007]</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -26273,7 +26315,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Motoriserende funn: Motor.no rapporterer at bilen "tramper urolig rundt pa ujevn vei" med ubehagelig humpete kjoring pa harde skjoter, mens RAC Drive pa samme drivlinje (150 Comfort Range) rapporterer at fjaeringen "smothers potholes and speed bumps quietly." De to profesjonelle kildene motsier hverandre direkte om komfort - dokumentert som uenighet, ikke lost ved a velge en foretrukket verdi (jf. rammeverkets prinsipp om a dokumentere uenighet mellom autoritative kilder). [Kriterium W002]</t>
+          <t>Motoriserende funn: Motor.no rapporterer at bilen "tramper urolig rundt på ujevn vei" med ubehagelig humpete kjøring på harde skjøter, mens RAC Drive på samme drivlinje (150 Comfort Range) rapporterer at fjæringen "smothers potholes and speed bumps quietly." De to profesjonelle kildene motsier hverandre direkte om komfort - dokumentert som uenighet, ikke løst ved å velge en foretrukket verdi (jf. rammeverkets prinsipp om å dokumentere uenighet mellom autoritative kilder). [Kriterium W002]</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -26313,7 +26355,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Motor.no rapporterer at en 180cm passasjer sa vidt far plass bak en like hoy forer i baksetet, og at pedalplassering er trang - en reell praktisk ulempe. Samtidig gir hoyere sittestilling bedre oversikt over omgivelsene. Blandet funn fra en uavhengig kilde. [Kriterium W003]</t>
+          <t>Motor.no rapporterer at en 180cm passasjer så vidt får plass bak en like høy fører i baksetet, og at pedalplassering er trang - en reell praktisk ulempe. Samtidig gir høyere sittestilling bedre oversikt over omgivelsene. Blandet funn fra en uavhengig kilde. [Kriterium W003]</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -26433,7 +26475,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Apple CarPlay er standard pa alle versjoner av Renault 4, bekreftet bade av offisiell Renault-spesifikasjon og uavhengig av RAC Drive ("comes on all models"). Motsatt funn av Tesla Model 3 Long Range RWD, som mangler CarPlay-stotte. [Kriterium W007]</t>
+          <t>Apple CarPlay er standard på alle versjoner av Renault 4, bekreftet både av offisiell Renault-spesifikasjon og uavhengig av RAC Drive ("comes on all models"). Motsatt funn av Tesla Model 3 Long Range RWD, som mangler CarPlay-støtte. [Kriterium W007]</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -26473,7 +26515,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Offisiell prisliste viser 100 kW DC-hurtiglading (15-80% pa ca. 30 minutter) og 15,5 kWh/100km forbruk for Techno (52 kWh Comfort Range) - solid ladeeffekt for segmentet, godt over minimumsbehovet gitt lav estimert arlig kjorelengde. [Kriterium W020]</t>
+          <t>Offisiell prisliste viser 100 kW DC-hurtiglading (15-80% på ca. 30 minutter) og 15,5 kWh/100km forbruk for Techno (52 kWh Comfort Range) - solid ladeeffekt for segmentet, godt over minimumsbehovet gitt lav estimert årlig kjørelengde. [Kriterium W020]</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -26513,7 +26555,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Motor.no rapporterer at hjulstoy er "en familiesvakhet for bilene pa MEB-plattformen" og at Elroq hadde mest hjulstoy av fem sammenlignede biler. What Car? rapporterer motsatt at Elroq var "fractionally quieter" enn konkurrentene (EV3, S5, Scenic) ved 70mph. Direkte motstridende funn fra to profesjonelle kilder - dokumentert som uenighet. [Kriterium W001]</t>
+          <t>Motor.no rapporterer at hjulstøy er "en familiesvakhet for bilene på MEB-plattformen" og at Elroq hadde mest hjulstøy av fem sammenlignede biler. What Car? rapporterer motsatt at Elroq var "fractionally quieter" enn konkurrentene (EV3, S5, Scenic) ved 70mph. Direkte motstridende funn fra to profesjonelle kilder - dokumentert som uenighet. [Kriterium W001]</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -26553,7 +26595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Motor.no beskriver fjaeringen som hastighetsavhengig (stiv i lav fart, fast og fin i hoy fart) - noytralt til svakt positivt funn. What Car? er klart positiv: fjaeringen "absorbs imperfections in the road surface extremely well and delivers a controlled ride at all speeds." [Kriterium W002]</t>
+          <t>Motor.no beskriver fjæringen som hastighetsavhengig (stiv i lav fart, fast og fin i høy fart) - nøytralt til svakt positivt funn. What Car? er klart positiv: fjæringen "absorbs imperfections in the road surface extremely well and delivers a controlled ride at all speeds." [Kriterium W002]</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -26713,7 +26755,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Apple CarPlay er standard pa alle versjoner av Skoda Elroq, bekreftet bade av What Car? og offisiell Skoda-spesifikasjon (SmartLink). Samme positive funn som Renault 4; motsatt funn av Tesla Model 3 Long Range RWD. [Kriterium W007]</t>
+          <t>Apple CarPlay er standard på alle versjoner av Skoda Elroq, bekreftet både av What Car? og offisiell Skoda-spesifikasjon (SmartLink). Samme positive funn som Renault 4; motsatt funn av Tesla Model 3 Long Range RWD. [Kriterium W007]</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -26753,7 +26795,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Offisiell prisliste viser 105 kW DC-hurtiglading (10-80% pa ca. 26 minutter) og 15,3 kWh/100km forbruk for Selection 60 - solid ladeeffekt for segmentet. [Kriterium W020]</t>
+          <t>Offisiell prisliste viser 105 kW DC-hurtiglading (10-80% på ca. 26 minutter) og 15,3 kWh/100km forbruk for Selection 60 - solid ladeeffekt for segmentet. [Kriterium W020]</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -26793,7 +26835,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Motor.no rapporterer lite hjulstoy pa piggfrie vinterdekk; What Car? beskriver bilen som "fairly hushed" ved hoy fart med kun litt vind-/veistoy. To uavhengige kilder er enige. [Kriterium W001]</t>
+          <t>Motor.no rapporterer lite hjulstøy på piggfrie vinterdekk; What Car? beskriver bilen som "fairly hushed" ved høy fart med kun litt vind-/veistøy. To uavhengige kilder er enige. [Kriterium W001]</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -26833,7 +26875,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Motor.no beskriver fjaeringen som svaert stiv over skarpe ujevnheter, men behagelig i fart. What Car? vurderer balansen mellom komfort og kjoreegenskaper som "almost spot-on." Begge kilder peker i samme retning (godt, med en viss stivhet over skarpe support). [Kriterium W002]</t>
+          <t>Motor.no beskriver fjæringen som svært stiv over skarpe ujevnheter, men behagelig i fart. What Car? vurderer balansen mellom komfort og kjøreegenskaper som "almost spot-on." Begge kilder peker i samme retning (godt, med en viss stivhet over skarpe support). [Kriterium W002]</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -26993,7 +27035,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>What Car? bekrefter at "Wireless Android Auto and Apple CarPlay are also included" pa Volvo EX30. Samme positive funn som Renault 4 og Skoda Elroq; motsatt funn av Tesla Model 3 Long Range RWD. [Kriterium W007]</t>
+          <t>What Car? bekrefter at "Wireless Android Auto and Apple CarPlay are also included" på Volvo EX30. Samme positive funn som Renault 4 og Skoda Elroq; motsatt funn av Tesla Model 3 Long Range RWD. [Kriterium W007]</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -27033,7 +27075,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Offisiell spesifikasjon viser 175 kW DC-hurtiglading (10-80% pa ca. 27 minutter) og 17,5 kWh/100km forbruk for P8 AWD.</t>
+          <t>Offisiell spesifikasjon viser 175 kW DC-hurtiglading (10-80% på ca. 27 minutter) og 17,5 kWh/100km forbruk for P8 AWD.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -27073,7 +27115,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>What Car? rapporterer lite motorstoy, lite dekkstoy pa motorvei og lite fjaeringsstoy i by. Kun en uavhengig kilde funnet. [Kriterium W001]</t>
+          <t>What Car? rapporterer lite motorstøy, lite dekkstøy på motorvei og lite fjæringsstøy i by. Kun en uavhengig kilde funnet. [Kriterium W001]</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -27113,7 +27155,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Motor.no rapporterer at bilen rister over brostein og oppleves spretten i hoyere hastighet pa Standard Range-varianten, med dempere beskrevet som stive og "ikke spesielt sofistikerte." What Car? rapporterer motsatt at fjaeringen er relativt myk og glatter ut humper, om enn med krengning i svinger. Direkte motstridende funn - dokumentert som uenighet, ikke lost. [Kriterium W002]</t>
+          <t>Motor.no rapporterer at bilen rister over brostein og oppleves spretten i høyere hastighet på Standard Range-varianten, med dempere beskrevet som stive og "ikke spesielt sofistikerte." What Car? rapporterer motsatt at fjæringen er relativt myk og glatter ut humper, om enn med krengning i svinger. Direkte motstridende funn - dokumentert som uenighet, ikke løst. [Kriterium W002]</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -27313,7 +27355,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Offisiell konfigurator viser 11 kW AC-lading og 15,2 kWh/100km forbruk for denne konfigurasjonen. DC-hurtigladeeffekt var ikke oppgitt pa kildesiden, noe som begrenser vurderingen av reell ladeegenskap sammenlignet med de andre bilene. [Kriterium W020]</t>
+          <t>Offisiell konfigurator viser 11 kW AC-lading og 15,2 kWh/100km forbruk for denne konfigurasjonen. DC-hurtigladeeffekt var ikke oppgitt på kildesiden, noe som begrenser vurderingen av reell ladeegenskap sammenlignet med de andre bilene. [Kriterium W020]</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -27473,7 +27515,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Dyrest av de fem (468 900 kr) og samtidig minst effektiv (17,5 kWh/100km, hoyest forbruk i utvalget) uten tilsvarende mer rekkevidde. Merprisen gar hovedsakelig til firehjulsdrift og ytelse (0-100 pa 3,6 sek), som rammeverket eksplisitt ekskluderer som en meningsfull faktor for langsiktig eierskap. Svakest verdi for pengene av de fem. [Kriterium W017]</t>
+          <t>Dyrest av de fem (468 900 kr) og samtidig minst effektiv (17,5 kWh/100km, høyest forbruk i utvalget) uten tilsvarende mer rekkevidde. Merprisen går hovedsakelig til firehjulsdrift og ytelse (0-100 på 3,6 sek), som rammeverket eksplisitt ekskluderer som en meningsfull faktor for langsiktig eierskap. Svakest verdi for pengene av de fem. [Kriterium W017]</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -27513,7 +27555,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Grunnprisen for selve GT Line-trimmen (346 417 kr) er faktisk lavest av alle fem, for nest-best rekkevidde (453 km) og det mest omfattende standardutstyret registrert i dette datasettet. Totalprisen i det spesifikke tilbudet (423 340 kr) reflekterer kjoperens egne tilvalg (4-seter, vinterhjul) og er ikke representativt for trimmens egen verdi. Vurdert pa grunnprisen: sterk verdi for pengene. [Kriterium W017]</t>
+          <t>Grunnprisen for selve GT Line-trimmen (346 417 kr) er faktisk lavest av alle fem, for nest-best rekkevidde (453 km) og det mest omfattende standardutstyret registrert i dette datasettet. Totalprisen i det spesifikke tilbudet (423 340 kr) reflekterer kjøperens egne tilvalg (4-seter, vinterhjul) og er ikke representativt for trimmens egen verdi. Vurdert på grunnprisen: sterk verdi for pengene. [Kriterium W017]</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -27713,7 +27755,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Lengde 4065mm gir 435mm margin under 4500mm-grensen - storst margin av alle fem, og eneste konfigurasjon med over 400mm margin. [Kriterium W019]</t>
+          <t>Lengde 4065mm gir 435mm margin under 4500mm-grensen - størst margin av alle fem, og eneste konfigurasjon med over 400mm margin. [Kriterium W019]</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -27953,7 +27995,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>elbil.no sin norske test gir en positiv, direkte vurdering av adaptiv cruise control - 'fungerer overraskende greit pa motorvei.' Kort omtale fremfor en dyptgaende vinterspesifikk test, men et reelt norsk testverdikt. [Kriterium W008]</t>
+          <t>elbil.no sin norske test gir en positiv, direkte vurdering av adaptiv cruise control - 'fungerer overraskende greit på motorvei.' Kort omtale fremfor en dyptgående vinterspesifikk test, men et reelt norsk testverdikt. [Kriterium W008]</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -27993,7 +28035,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Techno-trimmet far kun ryggekamera og parkeringssensorer foran - 360-graders kamera og automatisk parkering er reservert Iconic-varianten (+20 000 kr). Fungerende grunnutstyr, men mangler den spesifikke 360-verdien kriteriet fremhever. [Kriterium W009]</t>
+          <t>Techno-trimmet får kun ryggekamera og parkeringssensorer foran - 360-graders kamera og automatisk parkering er reservert Iconic-varianten (+20 000 kr). Fungerende grunnutstyr, men mangler den spesifikke 360-verdien kriteriet fremhever. [Kriterium W009]</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -30299,7 +30341,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ride comfort/suspension: Motor.no: "Bilen tramper urolig rundt pa ujevn vei, og harde skjoter gir ubehagelig humpete kjoring" - large 18" standard wheels place high demands on the suspension for a relaxed ride (tested: 150 Comfort Range).</t>
+          <t>Ride comfort/suspension: Motor.no: "Bilen tramper urolig rundt på ujevn vei, og harde skjøter gir ubehagelig humpete kjøring" - large 18" standard wheels place high demands on the suspension for a relaxed ride (tested: 150 Comfort Range).</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -30515,7 +30557,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Cabin/road noise: Motor.no: "hjulstoyen - en familiesvakhet for bilene pa MEB-plattformen - som odelegger her"; Elroq had the most wheel noise of five compared cars (tested: Elroq 60 with Motor-pakke).</t>
+          <t>Cabin/road noise: Motor.no: "hjulstøyen - en familiesvakhet for bilene på MEB-plattformen - som ødelegger her"; Elroq had the most wheel noise of five compared cars (tested: Elroq 60 with Motor-pakke).</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -30569,7 +30611,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Ride comfort/suspension: Motor.no: "Fjaeringen er stiv i lavere fart, fast og fin i hoyere fart" (tested: Elroq 60 with Motor-pakke).</t>
+          <t>Ride comfort/suspension: Motor.no: "Fjæringen er stiv i lavere fart, fast og fin i høyere fart" (tested: Elroq 60 with Motor-pakke).</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -30677,7 +30719,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Infotainment/software quality: Motor.no: "Betjeningen - ikke minst den pa rattet - er kanskje best av alle," praising a "fin miks av analoge og digitale funksjoner." What Car?: "responds quickly enough and is much easier to operate than... Mini Countryman Electric," though "EV3 and Scenic are even better."</t>
+          <t>Infotainment/software quality: Motor.no: "Betjeningen - ikke minst den på rattet - er kanskje best av alle," praising a "fin miks av analoge og digitale funksjoner." What Car?: "responds quickly enough and is much easier to operate than... Mini Countryman Electric," though "EV3 and Scenic are even better."</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -30785,7 +30827,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Cabin/road noise: Motor.no: "Lite hjulstoy pa piggfrie vinterdekk" (minimal tire noise on studless winter tires) (tested: P8 AWD).</t>
+          <t>Cabin/road noise: Motor.no: "Lite hjulstøy på piggfrie vinterdekk" (minimal tire noise on studless winter tires) (tested: P8 AWD).</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -30947,7 +30989,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Infotainment/software quality: Motor.no: Google-based system "fungerer bra" (works well), though driver-assistance features were "lunefull pa norske vinterveier" (temperamental on Norwegian winter roads) - adjusting adaptive cruise speed/interval "viste seg i praksis umulig" (proved practically impossible). What Car?: the Google-based system is "fundamentally excellent," responsive, most functions easy to find.</t>
+          <t>Infotainment/software quality: Motor.no: Google-based system "fungerer bra" (works well), though driver-assistance features were "lunefull på norske vinterveier" (temperamental on Norwegian winter roads) - adjusting adaptive cruise speed/interval "viste seg i praksis umulig" (proved practically impossible). What Car?: the Google-based system is "fundamentally excellent," responsive, most functions easy to find.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -31082,7 +31124,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Ride comfort/suspension: Motor.no: "Det rister godt over brostein, og humper og dumper i litt hoyere hastigheter gir en vel spretten folelse" (shakes noticeably over cobblestones, bouncy over bumps at higher speed); dampers described as stiff and "not particularly sophisticated" (tested: Standard Range, 42.2 kWh).</t>
+          <t>Ride comfort/suspension: Motor.no: "Det rister godt over brostein, og humper og dumper i litt høyere hastigheter gir en vel spretten følelse" (shakes noticeably over cobblestones, bouncy over bumps at higher speed); dampers described as stiff and "not particularly sophisticated" (tested: Standard Range, 42.2 kWh).</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -31730,7 +31772,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Forerassistenter kvalitet: elbil.no sin norske test bekrefter adaptiv cruise control er standard pa Techno (og Iconic), og at den fungerer 'overraskende greit pa motorvei'. Kort omtale, ikke en dyptgaende vintertest.</t>
+          <t>Førerassistenter kvalitet: elbil.no sin norske test bekrefter adaptiv cruise control er standard på Techno (og Iconic), og at den fungerer 'overraskende greit på motorvei'. Kort omtale, ikke en dyptgående vintertest.</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -31757,7 +31799,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Kamera/parkering: elbil.no bekrefter at 360-graders kamera og automatisk parkering kun finnes pa Iconic-varianten (+20 000 kr over Techno). Techno far ryggekamera og parkeringssensorer foran, men ingen 360-visning.</t>
+          <t>Kamera/parkering: elbil.no bekrefter at 360-graders kamera og automatisk parkering kun finnes på Iconic-varianten (+20 000 kr over Techno). Techno får ryggekamera og parkeringssensorer foran, men ingen 360-visning.</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">

</xml_diff>

<commit_message>
Add BYD Atto 3 as sixth vehicle - Design scored end-to-end
Vehicle, both real Norwegian trims (Comfort/Design), Technical, Equipment
and HardRequirementResults added for both configs (M001/M002/M004/M005
PASS, M003 winter range genuinely Unknown - an unconfirmed search-summary
figure was rejected rather than assumed). Design taken through the full
20-criterion weighted pipeline per the user's choice, backed by real
sources (Bil24, Formel E, BYD's warranty PDF, an owner-problems
compilation, a CarPlay-update article) - OverallScore ~69.2/100 at 100%
coverage. Two genuine findings documented rather than resolved: an
infotainment-quality source disagreement, and a DC-charging figure
conflict between BYD's spec and NAF's measurement.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -873,7 +873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4649,6 +4649,347 @@
       <c r="I88" t="inlineStr">
         <is>
           <t>EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Atto3 | Opplev din neste BYD idag</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>BYD Norge</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://byd.no/modeller/atto3</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Offisiell BYD Norge modellside for Atto 3 (Comfort/Design-nivå, 60 kWh/420 km WLTP). Ikke å forveksle med det separat markedsførte EVO 4x4 (byd.no/modeller/evo-4x4).</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>DATABASE</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>BYD ATTO 3 (MY23-24) (2022-2025) price and specifications</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>EV Database</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://ev-database.org/car/1782/BYD-ATTO-3</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Tredjeparts spesifikasjonsdatabase; brukt for lengde/bredde/høyde/motoreffekt/dreiemoment/toppfart som ikke er oppgitt på byd.no.</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>SRC_NAF_BILGUIDEN_ATTO3</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>BYD Atto 3 - pris, rekkevidde og tester</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>NAF</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>https://www.naf.no/bilguiden/bilmodell/byd-atto-3</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>NAFs egen testside viser kun sommertest 2023-resultater (ladetest, egenvekt); ingen vintertest-rekkevidde er publisert her, til tross for at et søkemotor-sammendrag hevdet et 311 km-tall som ikke lot seg bekrefte ved direkte henting av siden.</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Vi har testet BYD Atto 3</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Bil24</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>https://bil24.no/vi-har-testet-byd-atto-3</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Norsk redaksjonell test, 350 km kjørt. Testbil er Comfort-basert (pris ~423 000 kr inkl. vinterhjul/metallic/ladekabel), men deler karosseri/fjæring/infotainment/kamerasystem med Design - kun skjermstørrelse, bakluke og ambientbelysning skiller nivåene.</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>SRC_FORMELE_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>BYD Atto 3 Design - biltest</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Formel E (Danmark)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>https://formele.dk/index.php/el-biler/biltest-provekorsler/byd-test/383-byd-atto-3-design-biltest</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Dansk test spesifikt på Design-utstyrsnivå - direkte anvendelig på den norske Design-konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>SRC_EVPARTS4X4_ATTO3</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>COMMUNITY</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>BYD Atto 3 Common Problems, Fixes &amp; Reliability (2026 update)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>EVparts4x4</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://evparts4x4.com/blogs/news/byd-atto-3-common-problems-2026-update</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Sammenstilling av eierrapporterte problemer, ikke en profesjonell redaksjonell test - vektet lavere/supplerende, ikke som eneste kilde for W008.</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>SRC_CAREXPERT_ATTO3_CARPLAY</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>BYD Atto 3, Seal, Dolphin gain wireless Apple CarPlay</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>CarExpert</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://www.carexpert.com.au/car-news/byd-atto-3-seal-dolphin-gain-wireless-apple-carplay</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>2024-07-02</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Bekrefter trådløs CarPlay ankom via OTA-oppdatering (V1.8.0, 2. juli 2024) - før dette kun kablet CarPlay.</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>SRC_BYD_WARRANTY_NO</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Håndbok for begrenset garanti</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>BYD</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>https://www.byd.com/material/byd-site/eu/support/service/warranty/20251021/BYDH%C3%A5ndbok%20for%20begrenset%20garanti-NO.pdf</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Offisiell norsk garantihåndbok: 6 år/150 000 km generell, 8 år/250 000 km batteri (SOH&gt;=70%), 12 år rust, 8 år/150 000 km drivmotor.</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>NB</t>
         </is>
       </c>
     </row>
@@ -4672,7 +5013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8727,6 +9068,806 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>SCORE_000102</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>W001</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>REV_000101</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F102">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D102,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G102">
+        <f>ROUND(F102*INDEX('01_Criteria'!$F:$F,MATCH(C102,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000101 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>SCORE_000103</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>W002</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>REV_000102</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F103">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D103,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G103">
+        <f>ROUND(F103*INDEX('01_Criteria'!$F:$F,MATCH(C103,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000102 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>SCORE_000104</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>W003</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>REV_000103</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F104">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D104,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G104">
+        <f>ROUND(F104*INDEX('01_Criteria'!$F:$F,MATCH(C104,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000103 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>SCORE_000105</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>W004</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>REV_000104</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F105">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D105,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G105">
+        <f>ROUND(F105*INDEX('01_Criteria'!$F:$F,MATCH(C105,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000104 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>SCORE_000106</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>W005</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>REV_000105</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F106">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D106,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G106">
+        <f>ROUND(F106*INDEX('01_Criteria'!$F:$F,MATCH(C106,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000105 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>SCORE_000107</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>W006</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>REV_000106</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F107">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D107,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G107">
+        <f>ROUND(F107*INDEX('01_Criteria'!$F:$F,MATCH(C107,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000106 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>SCORE_000108</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>W007</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>REV_000107</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F108">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D108,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G108">
+        <f>ROUND(F108*INDEX('01_Criteria'!$F:$F,MATCH(C108,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000107 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>SCORE_000109</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>W008</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>REV_000108</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F109">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D109,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G109">
+        <f>ROUND(F109*INDEX('01_Criteria'!$F:$F,MATCH(C109,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Review score 2/5 (normalized RawScore = 40.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000108 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>SCORE_000110</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>W009</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>REV_000109</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F110">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D110,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G110">
+        <f>ROUND(F110*INDEX('01_Criteria'!$F:$F,MATCH(C110,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Review score 5/5 (normalized RawScore = 100.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000109 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>SCORE_000111</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>W010</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>REV_000110</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F111">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D111,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G111">
+        <f>ROUND(F111*INDEX('01_Criteria'!$F:$F,MATCH(C111,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000110 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>SCORE_000112</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>W011</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>REV_000111</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F112">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D112,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G112">
+        <f>ROUND(F112*INDEX('01_Criteria'!$F:$F,MATCH(C112,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000111 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>SCORE_000113</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>W012</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>REV_000112</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F113">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D113,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G113">
+        <f>ROUND(F113*INDEX('01_Criteria'!$F:$F,MATCH(C113,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000112 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>SCORE_000114</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>W013</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>REV_000113</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F114">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D114,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G114">
+        <f>ROUND(F114*INDEX('01_Criteria'!$F:$F,MATCH(C114,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000113 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>SCORE_000115</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>W014</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>REV_000114</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F115">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D115,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G115">
+        <f>ROUND(F115*INDEX('01_Criteria'!$F:$F,MATCH(C115,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000114 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>SCORE_000116</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>W015</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>REV_000115</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F116">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D116,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G116">
+        <f>ROUND(F116*INDEX('01_Criteria'!$F:$F,MATCH(C116,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Review score 5/5 (normalized RawScore = 100.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000115 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>SCORE_000117</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>W016</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>REV_000116</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F117">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D117,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G117">
+        <f>ROUND(F117*INDEX('01_Criteria'!$F:$F,MATCH(C117,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000116 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>SCORE_000118</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>W017</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>REV_000117</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F118">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D118,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G118">
+        <f>ROUND(F118*INDEX('01_Criteria'!$F:$F,MATCH(C118,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000117 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>SCORE_000119</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>W018</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>REV_000118</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F119">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D119,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G119">
+        <f>ROUND(F119*INDEX('01_Criteria'!$F:$F,MATCH(C119,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000118 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>SCORE_000120</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>W019</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>REV_000119</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F120">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D120,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G120">
+        <f>ROUND(F120*INDEX('01_Criteria'!$F:$F,MATCH(C120,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000119 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>SCORE_000121</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>W020</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>REV_000120</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F121">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D121,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G121">
+        <f>ROUND(F121*INDEX('01_Criteria'!$F:$F,MATCH(C121,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Review score 2/5 (normalized RawScore = 40.0/100 on a documented 1-5 scale, since the framework does not prescribe a numeric scale). Traceable to REV_000120 -&gt; supporting Evidence -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8739,7 +9880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9739,6 +10880,90 @@
         </is>
       </c>
       <c r="H24" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DEC_DATA_009</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Added sixth Vehicle (BYD Atto 3) - Vehicle, Configurations, Technical, Equipment and HardRequirementResults</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>First vehicle onboarded since the P1-P6 architecture review closed (FrameworkVersion 1.8) - first real test of 13_TechnicalFieldDefinitions/14_HardRequirementResults/Source.Language being used from day one instead of retrofitted. User confirmed via direct question that «BYD Atto 3» means the standard Atto 3 (FWD, 60 kWh), not the separately marketed BYD EVO 4x4 (AWD, 74.8 kWh, 443hk) - BYD Norge's own site treats these as two distinct model pages, not trims of one car.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Added both real Norwegian trims (Comfort 365920kr, Design 389920kr) as Configurations; Technical facts recorded once at Vehicle level since both trims share the same battery/dimensions/powertrain per byd.no. All 5 Hard Requirements resolved for both configs: M001/M002/M004/M005 PASS, M003 UNKNOWN (a search-engine-summarized 311km NAF winter-test figure could not be confirmed via direct fetch of NAF's own page, which only shows summer 2023 test data - left genuinely unresolved rather than assumed). DC fast-charging shows a genuine source disagreement (BYD states 80kW, NAF measured 90kW peak) - both recorded via Qualifier rather than picking one. No Evidence/Review/Score/OverallScore added yet - which trim to take through the full 20-criterion weighted scoring pipeline is still to be decided.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DEC_DATA_010</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Added BYD Atto 3 Design Evidence/Review/Score - now 6th vehicle in the full comparison, all 20 weighted criteria</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Completed the full weighted-scoring pipeline for BYD_ATTO3_DESIGN (chosen over Comfort per user's explicit choice - Design is closer in equipment tier to the other 5 vehicles' chosen configurations). All 5 Hard Requirements already resolved (DEC_DATA_009): M001/M002/M004/M005 PASS, M003 UNKNOWN.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>5 real sources used (Bil24 and Formel E professional tests, BYD's own warranty PDF, an owner-reported-problems compilation, and a dedicated CarPlay-update news article), 20 Evidence rows, 20 Reviews, 20 Scores. Two genuine findings documented rather than resolved: (1) infotainment quality source disagreement (Formel E praises the Design screen; Bil24 finds menu logic inconsistent), (2) a real, multi-source-confirmed ADAS quality weakness (jerky lane-keep, phantom collision warnings) scored low (W008=2/5) despite the underlying hardware being present and passing M004. Bil24's own reviewer was personally ambivalent about price/value, reflected honestly in W017 rather than inflated. No FrameworkVersion bump - pure data addition, same precedent as DEC_DATA_003/004/006/008.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
@@ -9761,7 +10986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9998,6 +11223,43 @@
       </c>
       <c r="H6">
         <f>IF(E6&lt;100,"Partial evaluation - "&amp;F6&amp;" of "&amp;G6&amp;" WEIGHTED+Active criteria scored ("&amp;E6&amp;"% of total weight).","Complete evaluation - all WEIGHTED+Active criteria scored.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OVSC_000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="D7">
+        <f>SUMIFS('10_Scoring'!$G$2:$G$1000,'10_Scoring'!$B$2:$B$1000,B7,'10_Scoring'!$E$2:$E$1000,C7)</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>ROUND(SUMPRODUCT(('10_Scoring'!$B$2:$B$1000=B7)*('10_Scoring'!$E$2:$E$1000=C7)*IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH('10_Scoring'!$C$2:$C$1000,'01_Criteria'!$A$2:$A$1000,0)),0))/SUMIFS('01_Criteria'!$F$2:$F$1000,'01_Criteria'!$E$2:$E$1000,"WEIGHTED",'01_Criteria'!$H$2:$H$1000,"TRUE")*100,2)</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>COUNTIFS('10_Scoring'!$B$2:$B$1000,B7,'10_Scoring'!$E$2:$E$1000,C7)</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>COUNTIFS('01_Criteria'!$E$2:$E$1000,"WEIGHTED",'01_Criteria'!$H$2:$H$1000,"TRUE")</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>IF(E7&lt;100,"Partial evaluation - "&amp;F7&amp;" of "&amp;G7&amp;" WEIGHTED+Active criteria scored ("&amp;E7&amp;"% of total weight).","Complete evaluation - all WEIGHTED+Active criteria scored.")</f>
         <v/>
       </c>
     </row>
@@ -10427,7 +11689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14024,6 +15286,406 @@
       <c r="H91" t="inlineStr">
         <is>
           <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>HRR_000091</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_COMFORT</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>HRR_000092</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_COMFORT</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4455mm er innenfor 4500mm-grensen med 45mm margin - en reell, men moderat margin.</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>HRR_000093</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_COMFORT</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Ingen bekreftet uavhengig vintertest funnet. Et søkemotor-sammendrag hevdet 311 km i NAFs vintertest, men dette tallet kunne ikke bekreftes ved direkte henting av NAFs egen Atto 3-side, som kun viser sommertest 2023-resultater. Forblir genuint ukjent, ikke antatt.</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>HRR_000094</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_COMFORT</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Adaptiv cruisekontroll bekreftet standard på offisiell BYD Norge-side (ikke brutt ned per utstyrsnivå, men listet som generell modellfunksjon).</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>HRR_000095</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_COMFORT</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Ryggekamera/360-graders kamera bekreftet standard på offisiell BYD Norge-side (ikke brutt ned per utstyrsnivå, men listet som generell modellfunksjon).</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>HRR_000096</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Kun helelektriske biler inkluderes i denne sammenligningen; alle vurderte konfigurasjoner er BEV.</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>HRR_000097</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4455mm er innenfor 4500mm-grensen med 45mm margin - en reell, men moderat margin.</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>HRR_000098</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Ingen bekreftet uavhengig vintertest funnet. Et søkemotor-sammendrag hevdet 311 km i NAFs vintertest, men dette tallet kunne ikke bekreftes ved direkte henting av NAFs egen Atto 3-side, som kun viser sommertest 2023-resultater. Forblir genuint ukjent, ikke antatt.</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>HRR_000099</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Adaptiv cruisekontroll bekreftet standard på offisiell BYD Norge-side (ikke brutt ned per utstyrsnivå, men listet som generell modellfunksjon).</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>HRR_000100</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Ryggekamera/360-graders kamera bekreftet standard på offisiell BYD Norge-side (ikke brutt ned per utstyrsnivå, men listet som generell modellfunksjon).</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>1.8</t>
         </is>
       </c>
     </row>
@@ -15499,7 +17161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15730,6 +17392,43 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>Volvo Norway official specifications page reviewed 2026-07-06: https://www.volvocars.com/no/cars/ex30-electric/specifications/. Model year and platform not specified in workbook-supported source fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BYD</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Atto 3</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>BYD Norge offisiell modellside sett 2026-07-07: https://byd.no/modeller/atto3. To utstyrsnivåer (Comfort, Design), ett batteri/drivverk (60 kWh, forhjulsdrift). Modellår og plattform ikke spesifisert i kildegrunnlaget. Skilt fra det separat markedsførte BYD EVO 4x4 (byd.no/modeller/evo-4x4), som ikke er del av denne sammenligningen.</t>
         </is>
       </c>
     </row>
@@ -15750,7 +17449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -16561,6 +18260,92 @@
         </is>
       </c>
       <c r="I19" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_COMFORT</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Comfort</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>365920</v>
+      </c>
+      <c r="G20" t="n">
+        <v>365920</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>BYD Norge offisiell prisliste sett 2026-07-07: https://byd.no/modeller/atto3. Møter alle sjekkede Hard Requirements - se 14_HardRequirementResults. M003 forblir Ukjent.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>389920</v>
+      </c>
+      <c r="G21" t="n">
+        <v>389920</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>BYD Norge offisiell prisliste sett 2026-07-07: https://byd.no/modeller/atto3. Deler ACC/ryggekamera/360-kamera med Comfort (kilden bryter ikke ned utstyr per nivå); Design-spesifikke tillegg er elektrisk bakluke, større skjerm (15,6"), flerfarget ambientbelysning. M003 forblir Ukjent.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -16589,7 +18374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K146"/>
+  <dimension ref="A1:K160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -23238,6 +25023,656 @@
       <c r="J146" t="inlineStr">
         <is>
           <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>TECH_000146</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>TF_LENGTH</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>4455</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>TECH_000147</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>TF_WIDTH</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>1875</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Excluding mirrors</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>TECH_000148</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>TF_WIDTH</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>2050</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Mirrors unfolded</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>TECH_000149</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>TF_HEIGHT</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>1615</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>TECH_000150</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>TF_KERB_WEIGHT</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>1750</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>SRC_NAF_BILGUIDEN_ATTO3</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>TECH_000151</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>TF_BOOT_VOLUME</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>440</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>TECH_000152</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>TF_BATTERY_NET</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>60.48</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>KWH</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>TECH_000153</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>TF_AC_MAX_CHARGING</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>11</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>TECH_000154</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>TF_DC_MAX_CHARGING</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>80</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Manufacturer-stated</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>TECH_000155</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>TF_DC_MAX_CHARGING</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>90</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>SRC_NAF_BILGUIDEN_ATTO3</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>NAF-measured peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>TECH_000156</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>TF_WLTP_RANGE</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>420</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>TECH_000157</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>TF_MOTOR_POWER</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>150</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>TECH_000158</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>TF_TORQUE</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>310</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>TECH_000159</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>TF_TOP_SPEED</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>160</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>KMH</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>1.8</t>
         </is>
       </c>
     </row>
@@ -23261,7 +25696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -25285,6 +27720,198 @@
       <c r="F63" t="inlineStr">
         <is>
           <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>EQ_000063</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_COMFORT</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>EQ_000064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_COMFORT</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>EQ_000065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_COMFORT</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>EQ_360</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>EQ_000066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>EQ_000067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>EQ_000068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>EQ_360</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -25908,7 +28535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -29966,6 +32593,806 @@
       <c r="I101" t="inlineStr">
         <is>
           <t>1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>REV_000101</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>3</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bil24 rapporterer komfortabelt støynivå opp til 80 km/t, men merkbart mer støy ved 100 km/t - nettopp den motorveifarten dette kriteriet vektlegger tungt. Testet på Comfort, men deler karosseri/lydisolasjon med Design. Kun én uavhengig kilde funnet. [Kriterium W001]</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>EV_000128</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>REV_000102</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>4</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>To uavhengige kilder (Bil24 på Comfort, Formel E på Design) er samstemte om en komfortabel, mykt avstemt fjæring. Bil24 fremhever komfortable seter over lengre kjøreturer, men med begrenset justeringsmulighet. [Kriterium W002]</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>EV_000129,EV_000130</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>REV_000103</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>4</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Bil24 fremhever 360-graders kamerasystemet som klart og tydelig med gode tilpasningsmuligheter, noe som gir god oversikt ved manøvrering og parkering. Generell fremrutesikt ikke eksplisitt vurdert i den ene kilden funnet. [Kriterium W003]</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>EV_000131</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>REV_000104</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>3</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Formel E (Design-testbil) beskriver kjøringen som 'stabil og ganske underholdende', med velavstemt fjæringsgeometri - men vurderingen er generell og ikke en detaljert styrefølelse-analyse. Kun én tynn kilde funnet, ingen motstridende eller bekreftende data. [Kriterium W004]</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>EV_000130</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>REV_000105</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>3</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Genuin kildemotsigelse: Formel E (Design) beskriver den 15,6 tommers skjermen som stor og svært tydelig, mens Bil24 finner infotainmentet stort sett brukervennlig men med ulogiske strukturer (f.eks. DAB-radio gjemt i en egen 'app'). Dokumentert som reell uenighet, ikke forsøkt løst. [Kriterium W005]</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>EV_000135,EV_000134</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>REV_000106</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>4</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Bil24 fremhever OTA-oppdateringsmuligheten som en tydelig fordel, som også gjør bilen attraktiv for tredjeparts appleverandører over tid. Kun én kilde, men entydig positiv og teknisk bekreftet (samme OTA-kanal brukt til å legge til trådløs CarPlay, se W007). [Kriterium W006]</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>EV_000136</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>REV_000107</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>3</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>CarPlay var kun kablet ved lansering; trådløs CarPlay ble lagt til via en bekreftet OTA-oppdatering (V1.8.0, 2026-forgjenger-dato 2024-07-02). Fungerer altså i dag, men den forsinkede/ettermonterte trådløsheten er en reell historisk begrensning verdt å notere. Android Auto var trådløst fra start. [Kriterium W007]</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>EV_000137</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>REV_000108</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>2</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>To uavhengige kilder peker samme vei: Bil24 (profesjonell test) beskriver adaptiv cruisekontroll som unødig hjelpsom med nedbremsing i svinger; en samling eierrapporter (EVparts4x4) dokumenterer falske frontkollisjonsvarsler i klar trafikk og en filholdsassistent med 'jerky' styreinngrep. Fungerer, men kvaliteten er en reell, dokumentert svakhet. [Kriterium W008]</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>EV_000132,EV_000133</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>REV_000109</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>5</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Bil24 gir eksplisitt positiv omtale av 360-graders kamerasystemet: klar og tydelig visning fra flere vinkler med gode tilpasningsmuligheter. Ingen negative funn om kamerakvalitet i noen av kildene gjennomgått. [Kriterium W009]</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>EV_000131</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>REV_000110</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Opplevd kvalitet</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>4</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Formel E (Design) beskriver interiøret som 'well-built, well-composed and modern' med detaljer som vegansk lær på rattet; Bil24 (Comfort) beskriver et overraskende 'lekent' interiør i form og farge. Ingen hardplast-kritikk funnet i noen kilde - solid for prisklassen. [Kriterium W010]</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>EV_000138,EV_000139</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>REV_000111</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Opplevd kvalitet</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>4</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Formel E vurderer Design-testbilen som 'well-built, well-composed' uten å nevne knirk eller løse paneler. Kun én kilde med eksplisitt byggekvalitetsvurdering, og ingen motstridende funn om knirk/skranglete inntrykk i de øvrige kildene. [Kriterium W011]</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>EV_000138</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>REV_000112</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Opplevd kvalitet</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>3</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Bil24 gir en detaljert, blandet vurdering: setet oppleves 'meget komfortabel' over en 350 km tur, men mangler lengde- og helningsjustering; hodehøyde er begrenset for høye passasjerer under panoramataket, og armlenet er relativt stort. Reelle, konkrete innvendinger, ikke bare generell positivitet. [Kriterium W012]</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>EV_000129,EV_000140</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>REV_000113</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Opplevd kvalitet</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>3</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Bil24 beskriver fysiske detaljer som polariserende: bakdørhåndtak i 'gitarstreng'-design er nytenkende men potensielt uheldig med barn i baksetet, girspaken oppleves som 'artig', men enkelte menystrukturer er ikke intuitive og rattvarme mangler helt. [Kriterium W013]</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>EV_000141</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>REV_000114</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>4</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>BYD er verdens største EV-produsent etter volum og har vært etablert som bilprodusent siden 1995 - ikke en ny, uprøvd aktør. Atto 3 har dessuten vært til salgs i Norge siden minst 2023 med flere uavhengige testrunder over tid, altså reell modellspesifikk historikk fremfor kun merke-fallback (se [[feedback-langtidseierskap-brand-fallback-confidence]]-prinsippet, som her ikke engang er nødvendig å ty til). [Kriterium W014]</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>EV_000145</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>REV_000115</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>5</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Offisiell garantihåndbok bekrefter 6 år/150 000 km generell garanti, 8 år/250 000 km batterigaranti (SOH&gt;=70%), 12 år rustgaranti og 8 år/150 000 km drivmotorgaranti - et objektivt sterkt garantipakke sammenlignet med de øvrige 5 bilene i denne sammenligningen. [Kriterium W015]</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>EV_000142</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>REV_000116</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>3</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Flere års dokumentert tilstedeværelse i det norske markedet (NAF-test datert 2023, samt nyere tester fra Bil24/Formel E) viser reell nordisk modenhet sammenlignet med f.eks. Kia EV2, som ble vurdert som for ny for vintertestsykluser. Trekkes likevel ned av at ingen kilde har dokumentert en faktisk vintertest av rekkevidde (se M003, forblir Ukjent). [Kriterium W016]</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>EV_000145</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>REV_000117</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Økonomi</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>3</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Design til 389 920 kr ligger midt i feltet av de 6 bilene (billigere enn Tesla, Kia og Volvo; dyrere enn Renault og Skoda) for en pakke med 5-stjerners NCAP, sterk garanti og OTA-økosystem, men svakere DC-lading og dokumenterte ADAS-kvirker. Bil24s egen tester er selv usikker på om dette er god verdi for en forhjulsdrevet 5-seter ('Det er kanskje det?') - en ærlig, ikke overdrevet, vurdering. [Kriterium W017]</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>EV_000144</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>REV_000118</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Praktisk bruk</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>4</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>440 liter bagasjerom med flatt gulv, 60/40 delt bakseterygg og to romslige sidekott gir god fleksibilitet for voksne passasjerer og bagasje. Eneste dokumenterte praktiske begrensning er redusert hodehøyde for høye passasjerer under panoramataket - ingen barnesetefokusert vurdering (jf. [[user-no-children-household]]). [Kriterium W018]</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>EV_000143,EV_000140</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>REV_000119</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Garasje</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>3</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4455mm gir 45mm margin til 4500mm-grensen - en reell, men moderat margin: trangere enn Kia EV2s 435mm, men romsligere enn Skoda Elroqs 12mm. Se 14_HardRequirementResults (M002) for samme grunnlag. [Kriterium W019]</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>EV_000146</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>REV_000120</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Rekkevidde/lading</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>2</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>DC-lading på 80kW (produsentoppgitt) til 90kW (NAF-målt) og AC på 11kW ligger under nivået til mange 2026-konkurrenter som ofte tilbyr 150-220kW DC. Kriteriet er lavt vektet, og svakheten trekker score noe ned, men ikke drastisk. [Kriterium W020]</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>EV_000147</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>1.8</t>
         </is>
       </c>
     </row>
@@ -29986,7 +33413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H128"/>
+  <dimension ref="A1:H148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -33460,6 +36887,546 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>EV_000128</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Kupéstøy: komfortable fjæringer og hyggelig støynivå opp til 80 km/t, men merkbart mer støy ved 100 km/t (motorveifart). Testet på Comfort-spesifikasjon, som deler karosseri og lydisolasjon med Design.</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>EV_000129</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Fjæring/seter: komfortabel over en 350 km kjøretur; førersete beskrevet som 'meget komfortabel', men mangler lengdejustering og setehelningsjustering. Armlene relativt stort. Testet på Comfort-spesifikasjon.</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>EV_000130</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Fjæring/styring (Design-testbil): avansert multilink bakaksel, fast men komfortabel fjæring; beskrevet som 'stabil og ganske underholdende å kjøre', velavstemt fjæringsgeometri kombinert med forhjulsdrift.</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>SRC_FORMELE_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>EV_000131</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>360-graders kamera: klar og tydelig visning foran, bak og ovenfra, med flere tilpasningsmuligheter for visningsvinkel. Testet på Comfort-spesifikasjon, men kamerasystemet er delt med Design.</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>EV_000132</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Adaptiv cruisekontroll beskrevet som 'noe hjelpsom med nedbremsing i svinger, kanskje litt mer enn undertegnede setter pris på'. Mange assistentfunksjoner kan deaktiveres.</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>EV_000133</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Eierrapporter: falske frontkollisjonsvarsler i klar trafikk ('beeping or flashing with no obstacle'), overivrige parkeringssensorer, og filholdsassistent beskrevet som gir 'overly aggressive or jerky steering input'.</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>SRC_EVPARTS4X4_ATTO3</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>EV_000134</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Infotainment oppleves i hovedsak brukervennlig, men med enkelte ulogiske strukturer (DAB-radio krever egen 'app' i stedet for å ligge i hovedradiomenyen). Spotify-integrasjon tilgjengelig.</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>EV_000135</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>15,6 tommers skjerm (Design) beskrevet som stor og svært tydelig, kan roteres 90 grader.</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>SRC_FORMELE_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>EV_000136</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>OTA-oppdateringsmulighet fremhevet som en tydelig fordel - gjør bilen attraktiv for tredjeparts appleverandører.</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>EV_000137</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Apple CarPlay var kun kablet ved lansering; trådløs CarPlay ble lagt til via en OTA-oppdatering (V1.8.0) 2. juli 2024. Android Auto har vært tilgjengelig trådløst fra start.</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>SRC_CAREXPERT_ATTO3_CARPLAY</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>EV_000138</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Design-testbil beskrevet som 'well-built, well-composed and modern' med et 'appealing design'; ratt i vegansk lær.</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>SRC_FORMELE_ATTO3_DESIGN</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>EV_000139</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Interiøret beskrives som overraskende lekent, 'både i former og i farge' - ikke et tradisjonelt/nøytralt SUV-interiør.</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>EV_000140</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Førermiljø: setet mangler lengde- og helningsjustering (risiko for enkelte kroppsstørrelser), stort armlene, og begrenset hodehøyde for høye passasjerer under panoramataket. Seterygg med to varmenivåer.</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>EV_000141</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Bakdørhåndtak i 'gitarstreng'-design beskrevet som artig, men potensielt problematisk med barn i baksetet. Girspaken beskrevet som 'artig'. Enkelte menystrukturer ikke intuitive. Ingen rattvarme.</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>EV_000142</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Offisiell garanti: 6 år/150 000 km generell garanti, 8 år/250 000 km batterigaranti (SOH&gt;=70%), 12 år rustgaranti, 8 år/150 000 km drivmotorgaranti.</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>SRC_BYD_WARRANTY_NO</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>EV_000143</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>440 liter bagasjerom, 60/40 delt bakseterygg med trekkstropper for nedfelling, to romslige sidekott, flatt gulv fremhevet som en praktisk fordel.</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>EV_000144</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Reviewer stiller åpent spørsmål ved verdien for en forhjulsdrevet 5-seters SUV til ~380-423 000 kr avhengig av utstyrsnivå/opsjoner: 'Det er kanskje det?' - ambivalent, ikke en sterk anbefaling.</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>SRC_BIL24_ATTO3</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>EV_000145</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Atto 3 har vært til salgs i Norge siden minst 2023 (jf. datert NAF-test av Comfort 2023) med flere uavhengige testrunder over tid (elbil.no, bil24.no, formele.dk, NAF) - reell modellspesifikk historikk, ikke kun merke-fallback.</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>SRC_NAF_BILGUIDEN_ATTO3</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>EV_000146</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4455mm gir 45mm margin til 4500mm-grensen - en reell, men moderat margin (trangere enn Kia EV2s 435mm, romsligere enn Skoda Elroqs 12mm).</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>SRC_EVDATABASE_ATTO3</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>EV_000147</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>DC-lading 80kW (produsentoppgitt) / 90kW (NAF-målt) og AC 11kW - under nivået til mange 2026-konkurrenter (ofte 150-220kW DC), men lavt vektet kriterium.</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Formalize vehicle-onboarding conventions and add dry-run tooling (ADR-013)
Onboarding BYD Atto 3 surfaced five conventions the last six sessions
followed only as undocumented, memorized practice: Confidence defaults,
ID-prefix zero-padding, and "one flagship Configuration per Vehicle gets
scored" (confirmed 6/6 vehicles). Writes these down in workbook-schema.md,
adds a sourcing-verification rule to docs/02 after a web-search summary
was found to misstate a source's actual content, and adds a committed
onboarding checklist plus a read-only scripts/ helper (first code in this
repo) to sanity-check OverallScore/CoveragePercent without LibreOffice.
Forward-looking only - no existing vehicle data audited or changed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -9880,7 +9880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -10964,6 +10964,48 @@
         </is>
       </c>
       <c r="H26" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DEC_ADR_013</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Formalized Confidence defaults, ID-prefix conventions, and flagship-Configuration scope; added a sourcing-verification rule; added an onboarding checklist template and read-only dry-run/ID-helper scripts (ADR-013)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Onboarding BYD Atto 3 as the sixth vehicle surfaced five conventions followed only as undocumented, memorized practice - Confidence defaults (98%/85%/72%/49% MEDIUM across 04_Technical/05_Equipment/07_Reviews/14_HardRequirementResults), ID-prefix zero-padding, and "one flagship Configuration per Vehicle gets scored" (confirmed 6/6 Vehicles) had never been written down; a web-search AI summary was also found to confidently misstate a source's actual content (BYD/NAF winter-range claim), caught only by direct verification.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>No workbook column added. scripts/onboarding_helpers.py and framework/templates/vehicle-onboarding-checklist.md added as new, non-workbook repository artifacts. Forward-looking only - no existing Vehicle, Configuration, or record was audited or modified for convention conformance.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>

</xml_diff>

<commit_message>
Update EV_Decision_Framework.xlsx and enhance winter range evaluation criteria
Modified the EV_Decision_Framework.xlsx file. In the criteria-and-weighting documentation, added guidance for evaluating winter range when no independent test exists, allowing for an estimate based on WLTP_RANGE at a low confidence level. This change aims to improve the clarity and usability of the evaluation process.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -59,7 +59,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Aptos"/>
       <family val="2"/>
@@ -101,8 +101,12 @@
       <name val="Aptos"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +117,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -143,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -155,6 +169,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -774,7 +796,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -10177,7 +10199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11515,6 +11537,48 @@
       <c r="H32" t="inlineStr">
         <is>
           <t>NONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>DEC_ADR_014</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Introduced a WLTP-based estimation method for M003 (winter motorway range) when no independent winter test exists, and resolved it for all six flagship Configurations (ADR-014)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>M003 had been UNKNOWN for all six flagships since DEC_M003_VERIFY - only two real winter test data points exist workbook-wide (Volvo P8 AWD, mismatched-trim Renault). User confirmed the underlying need tolerates one charging stop (not a strict zero-stop 300km requirement) but chose to fix the immediate data gap with a conservative WLTP x 0.70 estimate (below both real observed ratios of 72-75%) rather than wait indefinitely for real winter test data on 2026-model-year cars.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>6 HardRequirementResults rows updated in place (IDs unchanged): Tesla/Skoda/Volvo/Kia now PASS at LOW confidence; Renault and BYD now FAIL at LOW confidence. Per user's explicit direction, Renault and BYD are kept scored via HardRequirementOverride=TRUE, same treatment as Tesla's existing M002 FAIL override - not excluded from the comparison. 6 new 04_Technical TF_WINTER_HIGHWAY_RANGE_ESTIMATE rows added (TECH_000160-000165), Qualifier-disambiguated from the 2 existing real-test-based rows (Volvo P8 AWD, Renault Techno) which were left untouched. 15_Dashboard Decision Summary gained a Hard Requirement Reason column. Whether M003's own binary PASS/FAIL shape should be redefined to reflect a real 1-stop tolerance instead of a flat 300km/no-stop gate is a separate, larger question - deliberately out of scope here, see ADR-014 Alternatives Considered.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>METHODOLOGY</t>
         </is>
       </c>
     </row>
@@ -13723,22 +13787,22 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>To vintertester funnet, men begge er upålitelige treff: en 2022-test brukte en utgått pre-facelift-generasjon, og en NAF-vintertest 2025 rapporterer 702km WLTP som ikke matcher noen av de fire registrerte Model 3-konfigurasjonene. Forblir reelt ukjent.</t>
+          <t>Estimert vintervegkjørelengde = 70% av WLTP (ADR-014): 691 km (19-tommers hjul, konservativt valgt fremfor 750 km/18-tommers) x 0.70 = 483.7 km, god margin over ~300 km-kravet. Faktiske vintertester funnet tidligere ble forkastet som upålitelige (utdatert generasjon; NAF-tall matcher ingen registrert konfigurasjon) - forblir en LOW-konfidens estimering, ikke en måling.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -13945,7 +14009,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -13955,7 +14019,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Eneste tilgjengelige datapunkt (elbil.no, Iconic-trim - samme drivverk, men annet utstyrsnivå) målte 287 km ved konstant 100 km/t i mildvær (5-7°C), ikke reell vinterkulde. Et bekymringsfullt signal, men ikke et bekreftet fall, siden testen verken matcher trim eller forhold.</t>
+          <t>Estimert vintervegkjørelengde = 70% av WLTP (ADR-014): 398 km x 0.70 = 278.6 km, under ~300 km-kravet med 21.4 km. Bekreftes av det eksisterende reelle datapunktet (elbil.no, Iconic-trim, 287 km) - begge tall peker under 300 km selv om testen ikke matcher trim/forhold nøyaktig.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -13965,7 +14029,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -14135,7 +14199,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -14145,12 +14209,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Ingen uavhengig vintertest funnet for denne konfigurasjonen.</t>
+          <t>Ingen uavhengig vintertest funnet. Estimert vintervegkjørelengde = 70% av WLTP (ADR-014): 448 km x 0.70 = 313.6 km, bestått med kun 13.6 km margin - tett, men bestått under denne metodikken.</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -14283,7 +14347,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -14293,12 +14357,12 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Ingen vintertest vurdert for denne konfigurasjonen.</t>
+          <t>Ingen vintertest vurdert for denne spesifikke konfigurasjonen. Estimert vintervegkjørelengde = 70% av WLTP (ADR-014): 475 km x 0.70 = 332.5 km, bestått med 32.5 km margin. Bekreftes av det reelle testresultatet for søsterkonfigurasjonen P8 AWD (338 km, samme plattform) som ligger tett opptil.</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -14362,7 +14426,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -14372,12 +14436,12 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Ingen uavhengig vintertest funnet - sannsynligvis fordi modellen er for ny til det norske markedet.</t>
+          <t>Ingen uavhengig vintertest funnet - trolig fordi modellen er for ny for det norske markedet. Estimert vintervegkjørelengde = 70% av WLTP (ADR-014): 453 km x 0.70 = 317.1 km, bestått med 17.1 km margin.</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -16135,7 +16199,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -16145,12 +16209,12 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Ingen bekreftet uavhengig vintertest funnet. Et søkemotor-sammendrag hevdet 311 km i NAFs vintertest, men dette tallet kunne ikke bekreftes ved direkte henting av NAFs egen Atto 3-side, som kun viser sommertest 2023-resultater. Forblir genuint ukjent, ikke antatt.</t>
+          <t>Ingen bekreftet uavhengig vintertest funnet (tidligere søkemotor-sammendrag om 311 km kunne ikke bekreftes mot NAFs egen side). Estimert vintervegkjørelengde = 70% av WLTP (ADR-014): 420 km x 0.70 = 294.0 km, marginalt under ~300 km-kravet med 6.0 km - svært tett, i praksis på grensen.</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -16257,7 +16321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:R115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -16271,9 +16335,13 @@
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="32" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="3" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="14" max="14"/>
+    <col width="3" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="55" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16363,8 +16431,13 @@
           <t>FailCriterion</t>
         </is>
       </c>
-    </row>
-    <row r="6">
+      <c r="R5" s="10" t="inlineStr">
+        <is>
+          <t>Hard Requirement Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="6">
         <f>IF($H6="","",RANK($D6,$D$6:$D$25,0))</f>
         <v/>
@@ -16419,8 +16492,12 @@
         <f>IF($L6="","",IF($L6&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H6)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="7">
+      <c r="R6" s="11">
+        <f>IF($N6="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H6)*('14_HardRequirementResults'!$C$2:$C$1000=$N6),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
       <c r="A7" s="6">
         <f>IF($H7="","",RANK($D7,$D$6:$D$25,0))</f>
         <v/>
@@ -16475,8 +16552,12 @@
         <f>IF($L7="","",IF($L7&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H7)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="8">
+      <c r="R7" s="11">
+        <f>IF($N7="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H7)*('14_HardRequirementResults'!$C$2:$C$1000=$N7),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
       <c r="A8" s="6">
         <f>IF($H8="","",RANK($D8,$D$6:$D$25,0))</f>
         <v/>
@@ -16531,8 +16612,12 @@
         <f>IF($L8="","",IF($L8&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H8)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="9">
+      <c r="R8" s="11">
+        <f>IF($N8="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H8)*('14_HardRequirementResults'!$C$2:$C$1000=$N8),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="6">
         <f>IF($H9="","",RANK($D9,$D$6:$D$25,0))</f>
         <v/>
@@ -16587,8 +16672,12 @@
         <f>IF($L9="","",IF($L9&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H9)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="10">
+      <c r="R9" s="11">
+        <f>IF($N9="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H9)*('14_HardRequirementResults'!$C$2:$C$1000=$N9),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
       <c r="A10" s="6">
         <f>IF($H10="","",RANK($D10,$D$6:$D$25,0))</f>
         <v/>
@@ -16643,8 +16732,12 @@
         <f>IF($L10="","",IF($L10&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H10)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="11">
+      <c r="R10" s="11">
+        <f>IF($N10="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H10)*('14_HardRequirementResults'!$C$2:$C$1000=$N10),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
       <c r="A11" s="6">
         <f>IF($H11="","",RANK($D11,$D$6:$D$25,0))</f>
         <v/>
@@ -16699,8 +16792,12 @@
         <f>IF($L11="","",IF($L11&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H11)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="12">
+      <c r="R11" s="11">
+        <f>IF($N11="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H11)*('14_HardRequirementResults'!$C$2:$C$1000=$N11),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
       <c r="A12" s="6">
         <f>IF($H12="","",RANK($D12,$D$6:$D$25,0))</f>
         <v/>
@@ -16751,8 +16848,12 @@
         <f>IF($L12="","",IF($L12&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H12)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="13">
+      <c r="R12" s="11">
+        <f>IF($N12="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H12)*('14_HardRequirementResults'!$C$2:$C$1000=$N12),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
       <c r="A13" s="6">
         <f>IF($H13="","",RANK($D13,$D$6:$D$25,0))</f>
         <v/>
@@ -16803,8 +16904,12 @@
         <f>IF($L13="","",IF($L13&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H13)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="14">
+      <c r="R13" s="11">
+        <f>IF($N13="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H13)*('14_HardRequirementResults'!$C$2:$C$1000=$N13),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="6">
         <f>IF($H14="","",RANK($D14,$D$6:$D$25,0))</f>
         <v/>
@@ -16855,8 +16960,12 @@
         <f>IF($L14="","",IF($L14&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H14)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="15">
+      <c r="R14" s="11">
+        <f>IF($N14="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H14)*('14_HardRequirementResults'!$C$2:$C$1000=$N14),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
       <c r="A15" s="6">
         <f>IF($H15="","",RANK($D15,$D$6:$D$25,0))</f>
         <v/>
@@ -16907,8 +17016,12 @@
         <f>IF($L15="","",IF($L15&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H15)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="16">
+      <c r="R15" s="11">
+        <f>IF($N15="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H15)*('14_HardRequirementResults'!$C$2:$C$1000=$N15),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
       <c r="A16" s="6">
         <f>IF($H16="","",RANK($D16,$D$6:$D$25,0))</f>
         <v/>
@@ -16959,8 +17072,12 @@
         <f>IF($L16="","",IF($L16&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H16)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="17">
+      <c r="R16" s="11">
+        <f>IF($N16="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H16)*('14_HardRequirementResults'!$C$2:$C$1000=$N16),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
       <c r="A17" s="6">
         <f>IF($H17="","",RANK($D17,$D$6:$D$25,0))</f>
         <v/>
@@ -17011,8 +17128,12 @@
         <f>IF($L17="","",IF($L17&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H17)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="18">
+      <c r="R17" s="11">
+        <f>IF($N17="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H17)*('14_HardRequirementResults'!$C$2:$C$1000=$N17),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
       <c r="A18" s="6">
         <f>IF($H18="","",RANK($D18,$D$6:$D$25,0))</f>
         <v/>
@@ -17063,8 +17184,12 @@
         <f>IF($L18="","",IF($L18&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H18)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="19">
+      <c r="R18" s="11">
+        <f>IF($N18="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H18)*('14_HardRequirementResults'!$C$2:$C$1000=$N18),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
       <c r="A19" s="6">
         <f>IF($H19="","",RANK($D19,$D$6:$D$25,0))</f>
         <v/>
@@ -17115,8 +17240,12 @@
         <f>IF($L19="","",IF($L19&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H19)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="20">
+      <c r="R19" s="11">
+        <f>IF($N19="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H19)*('14_HardRequirementResults'!$C$2:$C$1000=$N19),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
       <c r="A20" s="6">
         <f>IF($H20="","",RANK($D20,$D$6:$D$25,0))</f>
         <v/>
@@ -17167,8 +17296,12 @@
         <f>IF($L20="","",IF($L20&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H20)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="21">
+      <c r="R20" s="11">
+        <f>IF($N20="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H20)*('14_HardRequirementResults'!$C$2:$C$1000=$N20),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
       <c r="A21" s="6">
         <f>IF($H21="","",RANK($D21,$D$6:$D$25,0))</f>
         <v/>
@@ -17219,8 +17352,12 @@
         <f>IF($L21="","",IF($L21&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H21)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="22">
+      <c r="R21" s="11">
+        <f>IF($N21="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H21)*('14_HardRequirementResults'!$C$2:$C$1000=$N21),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
       <c r="A22" s="6">
         <f>IF($H22="","",RANK($D22,$D$6:$D$25,0))</f>
         <v/>
@@ -17271,8 +17408,12 @@
         <f>IF($L22="","",IF($L22&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H22)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="23">
+      <c r="R22" s="11">
+        <f>IF($N22="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H22)*('14_HardRequirementResults'!$C$2:$C$1000=$N22),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="45" customHeight="1">
       <c r="A23" s="6">
         <f>IF($H23="","",RANK($D23,$D$6:$D$25,0))</f>
         <v/>
@@ -17323,8 +17464,12 @@
         <f>IF($L23="","",IF($L23&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H23)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="24">
+      <c r="R23" s="11">
+        <f>IF($N23="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H23)*('14_HardRequirementResults'!$C$2:$C$1000=$N23),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="45" customHeight="1">
       <c r="A24" s="6">
         <f>IF($H24="","",RANK($D24,$D$6:$D$25,0))</f>
         <v/>
@@ -17375,8 +17520,12 @@
         <f>IF($L24="","",IF($L24&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H24)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
-    </row>
-    <row r="25">
+      <c r="R24" s="11">
+        <f>IF($N24="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H24)*('14_HardRequirementResults'!$C$2:$C$1000=$N24),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1">
       <c r="A25" s="6">
         <f>IF($H25="","",RANK($D25,$D$6:$D$25,0))</f>
         <v/>
@@ -17427,6 +17576,10 @@
         <f>IF($L25="","",IF($L25&gt;0,IFERROR(INDEX('14_HardRequirementResults'!$C$2:$C$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H25)*('14_HardRequirementResults'!$D$2:$D$1000="FAIL"),0),0)),""),""))</f>
         <v/>
       </c>
+      <c r="R25" s="11">
+        <f>IF($N25="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$H25)*('14_HardRequirementResults'!$C$2:$C$1000=$N25),0),0)),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -19004,12 +19157,1647 @@
         <v/>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>4. Configuration Comparator</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Select two ConfigurationIDs below to compare every scored Criterion side-by-side, including Confidence and the underlying Review text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
+          <t>Configuration A</t>
+        </is>
+      </c>
+      <c r="B77" s="9" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t>Configuration B</t>
+        </is>
+      </c>
+      <c r="B78" s="9" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t>Configuration A</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>Configuration B</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>Vehicle / Trim</t>
+        </is>
+      </c>
+      <c r="B81">
+        <f>IF($B$77="","",IFERROR(INDEX('02_Vehicles'!$B$2:$B$1000,MATCH(INDEX('03_Configurations'!$B$2:$B$1000,MATCH($B$77,'03_Configurations'!$A$2:$A$1000,0)),'02_Vehicles'!$A$2:$A$1000,0))&amp;" "&amp;INDEX('02_Vehicles'!$C$2:$C$1000,MATCH(INDEX('03_Configurations'!$B$2:$B$1000,MATCH($B$77,'03_Configurations'!$A$2:$A$1000,0)),'02_Vehicles'!$A$2:$A$1000,0))&amp;" ("&amp;INDEX('03_Configurations'!$E$2:$E$1000,MATCH($B$77,'03_Configurations'!$A$2:$A$1000,0))&amp;")",""))</f>
+        <v/>
+      </c>
+      <c r="C81">
+        <f>IF($B$78="","",IFERROR(INDEX('02_Vehicles'!$B$2:$B$1000,MATCH(INDEX('03_Configurations'!$B$2:$B$1000,MATCH($B$78,'03_Configurations'!$A$2:$A$1000,0)),'02_Vehicles'!$A$2:$A$1000,0))&amp;" "&amp;INDEX('02_Vehicles'!$C$2:$C$1000,MATCH(INDEX('03_Configurations'!$B$2:$B$1000,MATCH($B$78,'03_Configurations'!$A$2:$A$1000,0)),'02_Vehicles'!$A$2:$A$1000,0))&amp;" ("&amp;INDEX('03_Configurations'!$E$2:$E$1000,MATCH($B$78,'03_Configurations'!$A$2:$A$1000,0))&amp;")",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>ConfiguredPrice</t>
+        </is>
+      </c>
+      <c r="B82">
+        <f>IF($B$77="","",IFERROR(INDEX('03_Configurations'!$G$2:$G$1000,MATCH($B$77,'03_Configurations'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C82">
+        <f>IF($B$78="","",IFERROR(INDEX('03_Configurations'!$G$2:$G$1000,MATCH($B$78,'03_Configurations'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>OverallScore</t>
+        </is>
+      </c>
+      <c r="B83">
+        <f>IF($B$77="","",IFERROR(INDEX('12_OverallScores'!$D$2:$D$1000,MATCH($B$77,'12_OverallScores'!$B$2:$B$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C83">
+        <f>IF($B$78="","",IFERROR(INDEX('12_OverallScores'!$D$2:$D$1000,MATCH($B$78,'12_OverallScores'!$B$2:$B$1000,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="inlineStr">
+        <is>
+          <t>CoveragePercent</t>
+        </is>
+      </c>
+      <c r="B84">
+        <f>IF($B$77="","",IFERROR(INDEX('12_OverallScores'!$E$2:$E$1000,MATCH($B$77,'12_OverallScores'!$B$2:$B$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C84">
+        <f>IF($B$78="","",IFERROR(INDEX('12_OverallScores'!$E$2:$E$1000,MATCH($B$78,'12_OverallScores'!$B$2:$B$1000,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>Hard Requirement Status</t>
+        </is>
+      </c>
+      <c r="B85">
+        <f>IF($B$77="","",IF(COUNTIFS('14_HardRequirementResults'!$B$2:$B$1000,$B$77,'14_HardRequirementResults'!$D$2:$D$1000,"FAIL")&gt;0,IF(IFERROR(INDEX('03_Configurations'!$I$2:$I$1000,MATCH($B$77,'03_Configurations'!$A$2:$A$1000,0)),"FALSE")="TRUE","FAIL - kept, overridden","FAIL - excluded"),IF(COUNTIFS('14_HardRequirementResults'!$B$2:$B$1000,$B$77,'14_HardRequirementResults'!$D$2:$D$1000,"UNKNOWN")&gt;0,"UNKNOWN","PASS")))</f>
+        <v/>
+      </c>
+      <c r="C85">
+        <f>IF($B$78="","",IF(COUNTIFS('14_HardRequirementResults'!$B$2:$B$1000,$B$78,'14_HardRequirementResults'!$D$2:$D$1000,"FAIL")&gt;0,IF(IFERROR(INDEX('03_Configurations'!$I$2:$I$1000,MATCH($B$78,'03_Configurations'!$A$2:$A$1000,0)),"FALSE")="TRUE","FAIL - kept, overridden","FAIL - excluded"),IF(COUNTIFS('14_HardRequirementResults'!$B$2:$B$1000,$B$78,'14_HardRequirementResults'!$D$2:$D$1000,"UNKNOWN")&gt;0,"UNKNOWN","PASS")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="inlineStr">
+        <is>
+          <t>CriterionID</t>
+        </is>
+      </c>
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C87" s="10" t="inlineStr">
+        <is>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="D87" s="10" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="E87" s="10" t="inlineStr">
+        <is>
+          <t>A: Score (1-5)</t>
+        </is>
+      </c>
+      <c r="F87" s="10" t="inlineStr">
+        <is>
+          <t>A: Confidence</t>
+        </is>
+      </c>
+      <c r="G87" s="10" t="inlineStr">
+        <is>
+          <t>A: WeightedScore</t>
+        </is>
+      </c>
+      <c r="H87" s="10" t="inlineStr">
+        <is>
+          <t>B: Score (1-5)</t>
+        </is>
+      </c>
+      <c r="I87" s="10" t="inlineStr">
+        <is>
+          <t>B: Confidence</t>
+        </is>
+      </c>
+      <c r="J87" s="10" t="inlineStr">
+        <is>
+          <t>B: WeightedScore</t>
+        </is>
+      </c>
+      <c r="K87" s="10" t="inlineStr">
+        <is>
+          <t>Δ WeightedScore (B-A)</t>
+        </is>
+      </c>
+      <c r="M87" s="10" t="inlineStr">
+        <is>
+          <t>A: Review Summary</t>
+        </is>
+      </c>
+      <c r="N87" s="10" t="inlineStr">
+        <is>
+          <t>B: Review Summary</t>
+        </is>
+      </c>
+      <c r="P87" s="10" t="inlineStr">
+        <is>
+          <t>A: ReviewID (helper)</t>
+        </is>
+      </c>
+      <c r="Q87" s="10" t="inlineStr">
+        <is>
+          <t>B: ReviewID (helper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="60" customHeight="1">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>W001</t>
+        </is>
+      </c>
+      <c r="B88">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A88,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C88">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A88,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D88">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A88,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E88">
+        <f>IF($P88="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P88,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F88">
+        <f>IF($P88="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P88,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G88">
+        <f>IF($P88="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P88,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H88">
+        <f>IF($Q88="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q88,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I88">
+        <f>IF($Q88="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q88,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J88">
+        <f>IF($Q88="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q88,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K88">
+        <f>IF(OR($G88="",$J88=""),"",$J88-$G88)</f>
+        <v/>
+      </c>
+      <c r="M88" s="11">
+        <f>IF($P88="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P88,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N88" s="11">
+        <f>IF($Q88="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q88,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P88">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A88),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q88">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A88),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" ht="60" customHeight="1">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>W002</t>
+        </is>
+      </c>
+      <c r="B89">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A89,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C89">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A89,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D89">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A89,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E89">
+        <f>IF($P89="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P89,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F89">
+        <f>IF($P89="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P89,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G89">
+        <f>IF($P89="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P89,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H89">
+        <f>IF($Q89="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q89,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I89">
+        <f>IF($Q89="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q89,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J89">
+        <f>IF($Q89="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q89,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K89">
+        <f>IF(OR($G89="",$J89=""),"",$J89-$G89)</f>
+        <v/>
+      </c>
+      <c r="M89" s="11">
+        <f>IF($P89="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P89,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N89" s="11">
+        <f>IF($Q89="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q89,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P89">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A89),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q89">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A89),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" ht="60" customHeight="1">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>W003</t>
+        </is>
+      </c>
+      <c r="B90">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A90,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C90">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A90,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D90">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A90,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E90">
+        <f>IF($P90="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P90,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F90">
+        <f>IF($P90="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P90,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G90">
+        <f>IF($P90="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P90,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H90">
+        <f>IF($Q90="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q90,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I90">
+        <f>IF($Q90="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q90,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J90">
+        <f>IF($Q90="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q90,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K90">
+        <f>IF(OR($G90="",$J90=""),"",$J90-$G90)</f>
+        <v/>
+      </c>
+      <c r="M90" s="11">
+        <f>IF($P90="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P90,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N90" s="11">
+        <f>IF($Q90="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q90,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P90">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A90),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q90">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A90),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91" ht="60" customHeight="1">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>W004</t>
+        </is>
+      </c>
+      <c r="B91">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A91,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C91">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A91,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D91">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A91,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E91">
+        <f>IF($P91="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P91,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F91">
+        <f>IF($P91="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P91,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G91">
+        <f>IF($P91="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P91,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H91">
+        <f>IF($Q91="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q91,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I91">
+        <f>IF($Q91="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q91,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J91">
+        <f>IF($Q91="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q91,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K91">
+        <f>IF(OR($G91="",$J91=""),"",$J91-$G91)</f>
+        <v/>
+      </c>
+      <c r="M91" s="11">
+        <f>IF($P91="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P91,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N91" s="11">
+        <f>IF($Q91="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q91,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P91">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A91),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q91">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A91),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92" ht="60" customHeight="1">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>W005</t>
+        </is>
+      </c>
+      <c r="B92">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A92,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C92">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A92,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D92">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A92,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E92">
+        <f>IF($P92="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P92,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F92">
+        <f>IF($P92="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P92,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G92">
+        <f>IF($P92="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P92,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H92">
+        <f>IF($Q92="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q92,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I92">
+        <f>IF($Q92="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q92,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J92">
+        <f>IF($Q92="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q92,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K92">
+        <f>IF(OR($G92="",$J92=""),"",$J92-$G92)</f>
+        <v/>
+      </c>
+      <c r="M92" s="11">
+        <f>IF($P92="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P92,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N92" s="11">
+        <f>IF($Q92="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q92,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P92">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A92),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q92">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A92),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93" ht="60" customHeight="1">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>W006</t>
+        </is>
+      </c>
+      <c r="B93">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A93,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C93">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A93,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D93">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A93,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E93">
+        <f>IF($P93="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P93,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F93">
+        <f>IF($P93="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P93,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G93">
+        <f>IF($P93="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P93,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H93">
+        <f>IF($Q93="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q93,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I93">
+        <f>IF($Q93="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q93,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J93">
+        <f>IF($Q93="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q93,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K93">
+        <f>IF(OR($G93="",$J93=""),"",$J93-$G93)</f>
+        <v/>
+      </c>
+      <c r="M93" s="11">
+        <f>IF($P93="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P93,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N93" s="11">
+        <f>IF($Q93="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q93,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P93">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A93),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q93">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A93),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94" ht="60" customHeight="1">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>W007</t>
+        </is>
+      </c>
+      <c r="B94">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A94,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C94">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A94,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D94">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A94,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E94">
+        <f>IF($P94="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P94,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F94">
+        <f>IF($P94="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P94,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G94">
+        <f>IF($P94="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P94,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H94">
+        <f>IF($Q94="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q94,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I94">
+        <f>IF($Q94="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q94,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J94">
+        <f>IF($Q94="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q94,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K94">
+        <f>IF(OR($G94="",$J94=""),"",$J94-$G94)</f>
+        <v/>
+      </c>
+      <c r="M94" s="11">
+        <f>IF($P94="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P94,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N94" s="11">
+        <f>IF($Q94="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q94,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P94">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A94),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q94">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A94),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95" ht="60" customHeight="1">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>W008</t>
+        </is>
+      </c>
+      <c r="B95">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A95,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C95">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A95,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D95">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A95,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E95">
+        <f>IF($P95="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P95,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F95">
+        <f>IF($P95="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P95,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G95">
+        <f>IF($P95="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P95,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H95">
+        <f>IF($Q95="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q95,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I95">
+        <f>IF($Q95="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q95,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J95">
+        <f>IF($Q95="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q95,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K95">
+        <f>IF(OR($G95="",$J95=""),"",$J95-$G95)</f>
+        <v/>
+      </c>
+      <c r="M95" s="11">
+        <f>IF($P95="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P95,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N95" s="11">
+        <f>IF($Q95="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q95,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P95">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A95),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q95">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A95),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96" ht="60" customHeight="1">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>W009</t>
+        </is>
+      </c>
+      <c r="B96">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A96,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C96">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A96,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D96">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A96,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E96">
+        <f>IF($P96="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P96,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F96">
+        <f>IF($P96="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P96,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G96">
+        <f>IF($P96="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P96,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H96">
+        <f>IF($Q96="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q96,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I96">
+        <f>IF($Q96="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q96,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J96">
+        <f>IF($Q96="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q96,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K96">
+        <f>IF(OR($G96="",$J96=""),"",$J96-$G96)</f>
+        <v/>
+      </c>
+      <c r="M96" s="11">
+        <f>IF($P96="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P96,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N96" s="11">
+        <f>IF($Q96="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q96,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P96">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A96),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q96">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A96),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97" ht="60" customHeight="1">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>W010</t>
+        </is>
+      </c>
+      <c r="B97">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A97,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C97">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A97,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D97">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A97,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E97">
+        <f>IF($P97="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P97,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F97">
+        <f>IF($P97="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P97,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G97">
+        <f>IF($P97="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P97,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H97">
+        <f>IF($Q97="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q97,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I97">
+        <f>IF($Q97="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q97,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J97">
+        <f>IF($Q97="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q97,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K97">
+        <f>IF(OR($G97="",$J97=""),"",$J97-$G97)</f>
+        <v/>
+      </c>
+      <c r="M97" s="11">
+        <f>IF($P97="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P97,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N97" s="11">
+        <f>IF($Q97="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q97,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P97">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A97),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q97">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A97),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98" ht="60" customHeight="1">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>W011</t>
+        </is>
+      </c>
+      <c r="B98">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A98,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C98">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A98,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D98">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A98,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E98">
+        <f>IF($P98="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P98,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F98">
+        <f>IF($P98="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P98,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G98">
+        <f>IF($P98="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P98,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H98">
+        <f>IF($Q98="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q98,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I98">
+        <f>IF($Q98="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q98,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J98">
+        <f>IF($Q98="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q98,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K98">
+        <f>IF(OR($G98="",$J98=""),"",$J98-$G98)</f>
+        <v/>
+      </c>
+      <c r="M98" s="11">
+        <f>IF($P98="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P98,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N98" s="11">
+        <f>IF($Q98="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q98,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P98">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A98),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q98">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A98),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99" ht="60" customHeight="1">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>W012</t>
+        </is>
+      </c>
+      <c r="B99">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A99,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C99">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A99,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D99">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A99,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E99">
+        <f>IF($P99="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P99,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F99">
+        <f>IF($P99="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P99,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G99">
+        <f>IF($P99="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P99,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H99">
+        <f>IF($Q99="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q99,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I99">
+        <f>IF($Q99="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q99,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J99">
+        <f>IF($Q99="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q99,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K99">
+        <f>IF(OR($G99="",$J99=""),"",$J99-$G99)</f>
+        <v/>
+      </c>
+      <c r="M99" s="11">
+        <f>IF($P99="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P99,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N99" s="11">
+        <f>IF($Q99="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q99,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P99">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A99),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q99">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A99),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100" ht="60" customHeight="1">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>W013</t>
+        </is>
+      </c>
+      <c r="B100">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A100,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C100">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A100,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D100">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A100,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E100">
+        <f>IF($P100="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P100,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F100">
+        <f>IF($P100="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P100,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G100">
+        <f>IF($P100="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P100,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H100">
+        <f>IF($Q100="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q100,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I100">
+        <f>IF($Q100="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q100,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J100">
+        <f>IF($Q100="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q100,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K100">
+        <f>IF(OR($G100="",$J100=""),"",$J100-$G100)</f>
+        <v/>
+      </c>
+      <c r="M100" s="11">
+        <f>IF($P100="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P100,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N100" s="11">
+        <f>IF($Q100="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q100,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P100">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A100),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q100">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A100),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101" ht="60" customHeight="1">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>W014</t>
+        </is>
+      </c>
+      <c r="B101">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A101,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C101">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A101,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D101">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A101,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E101">
+        <f>IF($P101="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P101,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F101">
+        <f>IF($P101="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P101,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G101">
+        <f>IF($P101="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P101,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H101">
+        <f>IF($Q101="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q101,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I101">
+        <f>IF($Q101="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q101,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J101">
+        <f>IF($Q101="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q101,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K101">
+        <f>IF(OR($G101="",$J101=""),"",$J101-$G101)</f>
+        <v/>
+      </c>
+      <c r="M101" s="11">
+        <f>IF($P101="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P101,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N101" s="11">
+        <f>IF($Q101="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q101,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P101">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A101),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q101">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A101),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102" ht="60" customHeight="1">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>W015</t>
+        </is>
+      </c>
+      <c r="B102">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A102,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C102">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A102,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D102">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A102,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E102">
+        <f>IF($P102="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P102,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F102">
+        <f>IF($P102="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P102,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G102">
+        <f>IF($P102="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P102,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H102">
+        <f>IF($Q102="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q102,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I102">
+        <f>IF($Q102="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q102,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J102">
+        <f>IF($Q102="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q102,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K102">
+        <f>IF(OR($G102="",$J102=""),"",$J102-$G102)</f>
+        <v/>
+      </c>
+      <c r="M102" s="11">
+        <f>IF($P102="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P102,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N102" s="11">
+        <f>IF($Q102="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q102,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P102">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A102),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q102">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A102),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103" ht="60" customHeight="1">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>W016</t>
+        </is>
+      </c>
+      <c r="B103">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A103,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C103">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A103,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D103">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A103,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E103">
+        <f>IF($P103="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P103,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F103">
+        <f>IF($P103="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P103,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G103">
+        <f>IF($P103="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P103,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H103">
+        <f>IF($Q103="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q103,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I103">
+        <f>IF($Q103="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q103,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J103">
+        <f>IF($Q103="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q103,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K103">
+        <f>IF(OR($G103="",$J103=""),"",$J103-$G103)</f>
+        <v/>
+      </c>
+      <c r="M103" s="11">
+        <f>IF($P103="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P103,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N103" s="11">
+        <f>IF($Q103="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q103,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P103">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A103),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q103">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A103),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104" ht="60" customHeight="1">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>W017</t>
+        </is>
+      </c>
+      <c r="B104">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A104,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C104">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A104,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D104">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A104,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E104">
+        <f>IF($P104="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P104,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F104">
+        <f>IF($P104="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P104,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G104">
+        <f>IF($P104="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P104,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H104">
+        <f>IF($Q104="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q104,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I104">
+        <f>IF($Q104="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q104,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J104">
+        <f>IF($Q104="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q104,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K104">
+        <f>IF(OR($G104="",$J104=""),"",$J104-$G104)</f>
+        <v/>
+      </c>
+      <c r="M104" s="11">
+        <f>IF($P104="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P104,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N104" s="11">
+        <f>IF($Q104="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q104,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P104">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A104),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q104">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A104),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105" ht="60" customHeight="1">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>W018</t>
+        </is>
+      </c>
+      <c r="B105">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A105,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C105">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A105,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D105">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A105,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E105">
+        <f>IF($P105="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P105,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F105">
+        <f>IF($P105="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P105,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G105">
+        <f>IF($P105="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P105,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H105">
+        <f>IF($Q105="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q105,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I105">
+        <f>IF($Q105="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q105,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J105">
+        <f>IF($Q105="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q105,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K105">
+        <f>IF(OR($G105="",$J105=""),"",$J105-$G105)</f>
+        <v/>
+      </c>
+      <c r="M105" s="11">
+        <f>IF($P105="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P105,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N105" s="11">
+        <f>IF($Q105="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q105,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P105">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A105),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q105">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A105),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106" ht="60" customHeight="1">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>W019</t>
+        </is>
+      </c>
+      <c r="B106">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A106,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C106">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A106,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D106">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A106,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E106">
+        <f>IF($P106="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P106,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F106">
+        <f>IF($P106="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P106,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G106">
+        <f>IF($P106="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P106,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H106">
+        <f>IF($Q106="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q106,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I106">
+        <f>IF($Q106="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q106,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J106">
+        <f>IF($Q106="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q106,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K106">
+        <f>IF(OR($G106="",$J106=""),"",$J106-$G106)</f>
+        <v/>
+      </c>
+      <c r="M106" s="11">
+        <f>IF($P106="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P106,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N106" s="11">
+        <f>IF($Q106="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q106,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P106">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A106),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q106">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A106),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107" ht="60" customHeight="1">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>W020</t>
+        </is>
+      </c>
+      <c r="B107">
+        <f>IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH($A107,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C107">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A107,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D107">
+        <f>IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH($A107,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E107">
+        <f>IF($P107="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($P107,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F107">
+        <f>IF($P107="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($P107,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="G107">
+        <f>IF($P107="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($P107,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H107">
+        <f>IF($Q107="","",IFERROR(INDEX('07_Reviews'!$E$2:$E$1000,MATCH($Q107,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="I107">
+        <f>IF($Q107="","",IFERROR(INDEX('07_Reviews'!$F$2:$F$1000,MATCH($Q107,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="J107">
+        <f>IF($Q107="","",IFERROR(INDEX('10_Scoring'!$G$2:$G$1000,MATCH($Q107,'10_Scoring'!$D$2:$D$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="K107">
+        <f>IF(OR($G107="",$J107=""),"",$J107-$G107)</f>
+        <v/>
+      </c>
+      <c r="M107" s="11">
+        <f>IF($P107="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($P107,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="N107" s="11">
+        <f>IF($Q107="","",IFERROR(INDEX('07_Reviews'!$G$2:$G$1000,MATCH($Q107,'07_Reviews'!$A$2:$A$1000,0)),""))</f>
+        <v/>
+      </c>
+      <c r="P107">
+        <f>IF($B$77="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$77)*('10_Scoring'!$C$2:$C$1000=$A107),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="Q107">
+        <f>IF($B$78="","",IFERROR(INDEX('10_Scoring'!$D$2:$D$1000,MATCH(1,INDEX(('10_Scoring'!$B$2:$B$1000=$B$78)*('10_Scoring'!$C$2:$C$1000=$A107),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>Hard Requirement Comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="10" t="inlineStr">
+        <is>
+          <t>CriterionID</t>
+        </is>
+      </c>
+      <c r="B110" s="10" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="C110" s="10" t="inlineStr">
+        <is>
+          <t>A: Result</t>
+        </is>
+      </c>
+      <c r="D110" s="10" t="inlineStr">
+        <is>
+          <t>A: Reason</t>
+        </is>
+      </c>
+      <c r="E110" s="10" t="inlineStr">
+        <is>
+          <t>B: Result</t>
+        </is>
+      </c>
+      <c r="F110" s="10" t="inlineStr">
+        <is>
+          <t>B: Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="B111">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A111,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C111">
+        <f>IF($B$77="","",IFERROR(INDEX('14_HardRequirementResults'!$D$2:$D$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$77)*('14_HardRequirementResults'!$C$2:$C$1000=$A111),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="D111" s="11">
+        <f>IF($B$77="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$77)*('14_HardRequirementResults'!$C$2:$C$1000=$A111),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="E111">
+        <f>IF($B$78="","",IFERROR(INDEX('14_HardRequirementResults'!$D$2:$D$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$78)*('14_HardRequirementResults'!$C$2:$C$1000=$A111),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="F111" s="11">
+        <f>IF($B$78="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$78)*('14_HardRequirementResults'!$C$2:$C$1000=$A111),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="B112">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A112,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C112">
+        <f>IF($B$77="","",IFERROR(INDEX('14_HardRequirementResults'!$D$2:$D$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$77)*('14_HardRequirementResults'!$C$2:$C$1000=$A112),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="D112" s="11">
+        <f>IF($B$77="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$77)*('14_HardRequirementResults'!$C$2:$C$1000=$A112),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="E112">
+        <f>IF($B$78="","",IFERROR(INDEX('14_HardRequirementResults'!$D$2:$D$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$78)*('14_HardRequirementResults'!$C$2:$C$1000=$A112),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="F112" s="11">
+        <f>IF($B$78="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$78)*('14_HardRequirementResults'!$C$2:$C$1000=$A112),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="B113">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A113,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C113">
+        <f>IF($B$77="","",IFERROR(INDEX('14_HardRequirementResults'!$D$2:$D$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$77)*('14_HardRequirementResults'!$C$2:$C$1000=$A113),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="D113" s="11">
+        <f>IF($B$77="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$77)*('14_HardRequirementResults'!$C$2:$C$1000=$A113),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="E113">
+        <f>IF($B$78="","",IFERROR(INDEX('14_HardRequirementResults'!$D$2:$D$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$78)*('14_HardRequirementResults'!$C$2:$C$1000=$A113),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="F113" s="11">
+        <f>IF($B$78="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$78)*('14_HardRequirementResults'!$C$2:$C$1000=$A113),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="B114">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A114,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C114">
+        <f>IF($B$77="","",IFERROR(INDEX('14_HardRequirementResults'!$D$2:$D$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$77)*('14_HardRequirementResults'!$C$2:$C$1000=$A114),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="D114" s="11">
+        <f>IF($B$77="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$77)*('14_HardRequirementResults'!$C$2:$C$1000=$A114),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="E114">
+        <f>IF($B$78="","",IFERROR(INDEX('14_HardRequirementResults'!$D$2:$D$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$78)*('14_HardRequirementResults'!$C$2:$C$1000=$A114),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="F114" s="11">
+        <f>IF($B$78="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$78)*('14_HardRequirementResults'!$C$2:$C$1000=$A114),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="B115">
+        <f>IFERROR(INDEX('01_Criteria'!$C$2:$C$1000,MATCH($A115,'01_Criteria'!$A$2:$A$1000,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C115">
+        <f>IF($B$77="","",IFERROR(INDEX('14_HardRequirementResults'!$D$2:$D$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$77)*('14_HardRequirementResults'!$C$2:$C$1000=$A115),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="D115" s="11">
+        <f>IF($B$77="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$77)*('14_HardRequirementResults'!$C$2:$C$1000=$A115),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="E115">
+        <f>IF($B$78="","",IFERROR(INDEX('14_HardRequirementResults'!$D$2:$D$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$78)*('14_HardRequirementResults'!$C$2:$C$1000=$A115),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="F115" s="11">
+        <f>IF($B$78="","",IFERROR(INDEX('14_HardRequirementResults'!$F$2:$F$1000,MATCH(1,INDEX(('14_HardRequirementResults'!$B$2:$B$1000=$B$78)*('14_HardRequirementResults'!$C$2:$C$1000=$A115),0),0)),""))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="A27:N27"/>
+    <mergeCell ref="A74:Q74"/>
     <mergeCell ref="A4:N4"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A51:N51"/>
+    <mergeCell ref="A75:Q75"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B53:F72">
@@ -19024,6 +20812,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="B77 B78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>='03_Configurations'!$A$2:$A$21</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -21052,12 +22845,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Renault Norway official price list (Versjon 2, 01-06-2026) reviewed 2026-07-06. Meets all checked Hard Requirements (BEV, length 4140mm, Intelligent cruise control multi target = adaptive, standard rearview camera). M003 (winter highway range) remains Unknown - no winter test data reviewed. M003 (winter highway range): No dedicated deep-winter test found for this exact configuration. Closest available data point (elbil.no, Iconic trim - same 52kWh/150hk powertrain as Techno, but a different equipment level) measured 287 km at constant 100km/h highway driving in mild 5-7C conditions - NOT true winter cold. Since colder conditions would be expected to reduce range further, this data point is a concerning signal rather than a confident pass: the hard requirement remains genuinely uncertain, possibly at risk of failing, for this configuration. Flagged for the user's attention rather than resolved either way.</t>
+          <t>Renault Norway official price list (Versjon 2, 01-06-2026) reviewed 2026-07-06. Meets all checked Hard Requirements (BEV, length 4140mm, Intelligent cruise control multi target = adaptive, standard rearview camera). M003 (winter highway range) remains Unknown - no winter test data reviewed. M003 (winter highway range): No dedicated deep-winter test found for this exact configuration. Closest available data point (elbil.no, Iconic trim - same 52kWh/150hk powertrain as Techno, but a different equipment level) measured 287 km at constant 100km/h highway driving in mild 5-7C conditions - NOT true winter cold. Since colder conditions would be expected to reduce range further, this data point is a concerning signal rather than a confident pass: the hard requirement remains genuinely uncertain, possibly at risk of failing, for this configuration. Flagged for the user's attention rather than resolved either way. See 14_HardRequirementResults (M003) and DecisionLog DEC_ADR_014 for the Hard Requirement failure and override rationale.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -21611,12 +23404,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>BYD Norge offisiell prisliste sett 2026-07-07: https://byd.no/modeller/atto3. Deler ACC/ryggekamera/360-kamera med Comfort (kilden bryter ikke ned utstyr per nivå); Design-spesifikke tillegg er elektrisk bakluke, større skjerm (15,6"), flerfarget ambientbelysning. M003 forblir Ukjent.</t>
+          <t>BYD Norge offisiell prisliste sett 2026-07-07: https://byd.no/modeller/atto3. Deler ACC/ryggekamera/360-kamera med Comfort (kilden bryter ikke ned utstyr per nivå); Design-spesifikke tillegg er elektrisk bakluke, større skjerm (15,6"), flerfarget ambientbelysning. M003 forblir Ukjent. See 14_HardRequirementResults (M003) and DecisionLog DEC_ADR_014 for the Hard Requirement failure and override rationale.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -21643,7 +23436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K160"/>
+  <dimension ref="A1:K166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -28942,6 +30735,306 @@
       <c r="J160" t="inlineStr">
         <is>
           <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>TECH_000160</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>TESLA_MODEL_3_LONG_RANGE_RWD</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>TF_WINTER_HIGHWAY_RANGE_ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>483.7</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>SRC_TESLA_NO_MODEL3_CONFIGURATOR</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Estimated (70% of WLTP, ADR-014)</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>TECH_000161</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>RENAULT_4_TECHNO</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>TF_WINTER_HIGHWAY_RANGE_ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>278.6</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>SRC_RENAULT_NO_R4_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>Estimated (70% of WLTP, ADR-014)</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>TECH_000162</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>SKODA_ELROQ_SELECTION_60</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>TF_WINTER_HIGHWAY_RANGE_ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>313.6</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_NO_ELROQ_PRICELIST</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Estimated (70% of WLTP, ADR-014)</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>TECH_000163</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>TF_WINTER_HIGHWAY_RANGE_ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>332.5</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>SRC_VOLVO_NO_EX30_SPECS</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Estimated (70% of WLTP, ADR-014)</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>TECH_000164</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>KIA_EV2_FWD_LONG_RANGE_GT_LINE</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>TF_WINTER_HIGHWAY_RANGE_ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>317.1</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>SRC_KIA_NETTBUTIKK_EV2</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Estimated (70% of WLTP, ADR-014)</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>TECH_000165</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>BYD_ATTO3</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>TF_WINTER_HIGHWAY_RANGE_ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>294</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>SRC_BYD_NO_ATTO3</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>Estimated (70% of WLTP, ADR-014)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update EV_Decision_Framework.xlsx with new data revisions
The EV_Decision_Framework.xlsx file has been updated, reflecting changes in the data structure. This update includes adjustments to the evaluation criteria, enhancing the overall framework's accuracy and usability. No specific details on the changes are provided, but the binary file indicates a significant modification.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -1192,7 +1192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2879,7 +2879,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.frydenbo.no/</t>
+          <t>https://www.frydenbo-bil.no/aktuelt/slik-velger-du-riktig-utstyrsniva-for-din-volvo-ex30</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Independently corroborates that at the Twin Performance AWD powertrain, Plus trim (468,900 NOK) excludes the 360-degree camera/Park Pilot, which is only added at Ultra trim (~505,900 NOK) for the same powertrain.</t>
+          <t>Independently corroborates that at the Twin Performance AWD powertrain, Plus trim (468,900 NOK) excludes the 360-degree camera/Park Pilot, which is only added at Ultra trim (~505,900 NOK) for the same powertrain. Same article also confirms Adaptive Cruise Control and a reversing camera are standard from Core level upward across the EX30 range.</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -5309,6 +5309,216 @@
       <c r="I96" t="inlineStr">
         <is>
           <t>NB</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>SRC_FRYDENBO_EX30_UTSTYRSNIVA_GUIDE</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Slik velger du riktig utstyrsnivå for din Volvo EX30</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Frydenbø Bil (Volvo-forhandler, Norge)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://www.frydenbo-bil.no/aktuelt/slik-velger-du-riktig-utstyrsniva-for-din-volvo-ex30</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Bekrefter at Adaptiv Cruise Kontroll og ryggekamera er standard fra og med Core-utstyrsnivå (laveste nivå) på EX30; 360-graders kamera forblir forbeholdt Ultra.</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>SRC_FRYDENBO_EX30_CAMPAIGN_PRICING</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Kampanje på Volvo EX30 (modell/utstyrsnivå/pris-oversikt)</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Frydenbø Bil (Volvo-forhandler, Norge)</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>https://www.frydenbo-bil.no/kampanje/nybil/volvo/ex30</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Bekrefter at Single Motor Extended Range (476 km rekkevidde, matcher denne konfigurasjonens registrerte WLTP) selges som Plus-utstyrsnivå i det norske markedet - ikke Core eller Ultra. Første uavhengige bekreftelse av hvilket utstyrsnivå P5 Long Range faktisk tilsvarer (se REV_000057s tidligere åpne usikkerhet).</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>SRC_NAF_BILGUIDEN_VOLVO_EX30</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Volvo EX30 - pris, rekkevidde og tester</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>NAF (Norges Automobil-Forbund)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>https://www.naf.no/bilguiden/bilmodell/volvo-ex30</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Oppgir bagasjeromskapasitet (318 liter bak, 7 liter foran/frunk) og maksimal DC-ladeeffekt (153 kW). Ikke trimnivå-spesifikk.</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>SRC_AUTOMOLI_VOLVO_EX30_SPECS</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Tekniske data Volvo EX30</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Automoli</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>https://www.automoli.com/no/vehicles/volvo/ex30/ex30-9517/</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Oppgir bakkeklaring (165mm, oppgitt å gjelde alle tre motorvarianter) og alternative bagasjeromstall (min 234L / maks 904L). Eneste funnet kilde for bakkeklaring - ikke uavhengig krysssjekket.</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>SRC_ZECAR_VOLVO_EX30_CHARGING</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Volvo EX30 Single Motor Extended Charging Guide</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Zecar</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>https://zecar.com/ev-charging-guides/volvo/ex30/2024/single-motor-extended</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Oppgir 11 kW AC/onboard-lading for Single Motor Extended Range (P5 Long Range). 22kW er kun tilgjengelig som opsjon på Twin Performance (AWD), ikke relevant for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>EN</t>
         </is>
       </c>
     </row>
@@ -10199,7 +10409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11579,6 +11789,48 @@
       <c r="H33" t="inlineStr">
         <is>
           <t>METHODOLOGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DEC_DATA_011</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Researched Volvo EX30 P5 Long Range: resolved M004/M005 from Unknown/borrowed, populated Equipment, added Boot Volume/Ground Clearance/AC Charging Technical facts, upgraded W009 Review confidence</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Volvo P5 Long Range had the thinnest data footprint of the six flagships: M005 (rearview camera) was UNKNOWN, M004 (ACC) was PASS but LOW-confidence borrowed from the P8 AWD sibling configuration, 05_Equipment had only 1 row (CarPlay), and REV_000057 (W009) carried an explicit open question - which equipment tier (Plus/Ultra) P5 Long Range is actually sold at was never independently confirmed, only assumed identical to P8 AWD.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Official volvocars.com pages returned HTTP 403 for direct fetch throughout this research (manufacturer site blocks automated fetching) - all facts sourced from accessible secondary sources instead (Frydenbo, a Volvo Norway dealer; NAF; Automoli; Zecar), each fetched and read directly per the ADR-013 sourcing rule (a search summary alone was never used to confirm content). Key finding: Frydenbo's own EX30 campaign pricing page confirms Single Motor Extended Range (476km, matching this Configuration's own WLTP figure) is sold as Plus trim in the Norwegian market - resolving REV_000057's previously open question. HRR_000071 (M004) and HRR_000088 (M005) both now PASS at MEDIUM confidence (was LOW/UNKNOWN). 4 new 05_Equipment rows (EQ_000069-072). 3 new 04_Technical rows (TECH_000166-168): Boot Volume 318L (MEDIUM, NAF), Ground Clearance 165mm (LOW, single-source Automoli, not independently cross-checked), AC charging 11kW (MEDIUM, Zecar). REV_000057 confidence upgraded LOW-&gt;MEDIUM, EvidenceID extended to include the new trim-confirming EV_000150. Score (2/5, no 360 camera) unchanged - the underlying conclusion was already correct, only the confidence behind it improves. Separately noted but NOT resolved: Frydenbo's campaign page states 468,900 kr (regular) for this exact Plus/Single-Motor-Extended-Range combination, which does not match this Configuration's recorded 437,900 kr price (see 03_Configurations) - a real discrepancy worth checking, out of scope for this research pass, flagged for the user rather than silently corrected (same precedent as the Kia price fix). RESOLVED 2026-07-08: user confirmed 437 900 kr is the correct base price for this Plus-trim configuration - the 468 900 kr figure on Frydenbo campaign page very likely includes a bundled winter-tire package (mandatory in Norway, commonly bundled by dealers), not a genuine price discrepancy like the earlier Kia case. No price change made.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>NONE</t>
         </is>
       </c>
     </row>
@@ -15120,17 +15372,17 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Ikke uavhengig bekreftet for denne spesifikke konfigurasjonen; utledet fra VOLVO_EX30_P8_AWD, som deler samme kjøreassistentpakke på tvers av rekken per Volvos egen produktbeskrivelse.</t>
+          <t>Bekreftet standard fra og med Core-utstyrsnivå per Frydenbøs egen utstyrsnivå-veiledning. Denne konfigurasjonen (Single Motor Extended Range) er uavhengig bekreftet solgt som Plus-nivå i det norske markedet (Frydenbøs kampanjeside, 476 km rekkevidde matcher registrert WLTP) - Plus ligger over Core, så ACC er inkludert uavhengig av tidligere usikkerhet knyttet til P8 AWD-utledningen.</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -15804,22 +16056,22 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Ikke uavhengig bekreftet via en presist kildesporet henting - forblir bevisst ukjent fremfor antatt.</t>
+          <t>Ryggekamera bekreftet standard fra og med Core-utstyrsnivå per Frydenbøs egen utstyrsnivå-veiledning. Denne konfigurasjonen uavhengig bekreftet som Plus-nivå i det norske markedet (se M004-begrunnelse) - ryggekamera dermed inkludert.</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -23232,7 +23484,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Volvo Norway official specifications page reviewed 2026-07-06. Flagship Configuration for this Vehicle as of 2026-07-07 (switched from P8 AWD to more closely match the other five vehicles trim level) - see 11_DecisionLog DEC_DASHBOARD_004 and the driving-dynamics caveats on 07_Reviews W008/W009/W016. Same Hard Requirement notes as P5 (see above); M003 remains Unknown (see 14_HardRequirementResults) since the only winter-range data point (elbil.no, ~338km) was measured on P8 AWD, a different drivetrain.</t>
+          <t>Volvo Norway official specifications page reviewed 2026-07-06. Flagship Configuration for this Vehicle as of 2026-07-07 (switched from P8 AWD to more closely match the other five vehicles trim level) - see 11_DecisionLog DEC_DASHBOARD_004 and the driving-dynamics caveats on 07_Reviews W008/W016. M003 resolved via ADR-014 WLTP-based estimate (see 14_HardRequirementResults, DEC_ADR_014). 437 900 kr confirmed by user as the correct base price for this Plus-trim configuration; a higher 468 900 kr figure found on a dealer campaign page during DEC_DATA_011 research is very likely a winter-tire-inclusive package price (winter tires are mandatory in Norway and commonly bundled by dealers), not a base-price discrepancy.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -23436,7 +23688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K166"/>
+  <dimension ref="A1:K169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -31035,6 +31287,141 @@
       <c r="K166" t="inlineStr">
         <is>
           <t>Estimated (70% of WLTP, ADR-014)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>TECH_000166</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>TF_BOOT_VOLUME</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>318</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>SRC_NAF_BILGUIDEN_VOLVO_EX30</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>TECH_000167</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>TF_GROUND_CLEARANCE</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>165</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>SRC_AUTOMOLI_VOLVO_EX30_SPECS</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>TECH_000168</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>TF_AC_MAX_CHARGING</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>11</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>SRC_ZECAR_VOLVO_EX30_CHARGING</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -31058,7 +31445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -33272,6 +33659,134 @@
         </is>
       </c>
       <c r="F69" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>EQ_000069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>SRC_FRYDENBO_EX30_UTSTYRSNIVA_GUIDE</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>EQ_000070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>SRC_FRYDENBO_EX30_UTSTYRSNIVA_GUIDE</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>EQ_000071</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>EQ_360</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>SRC_FRYDENBO_EX30_UTSTYRSNIVA_GUIDE</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>EQ_000072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>EQ_LANE_CENTER</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>SRC_FRYDENBO_EX30_UTSTYRSNIVA_GUIDE</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -36219,22 +36734,22 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>elbil.no og Frydenbøs trimnivå-sammenligning bekrefter at 360-graders kamera er forbeholdt Ultra-utstyrsnivå, ikke inkludert på Plus - men denne sammenligningen ble gjort for Twin Performance AWD (P8 AWD) spesifikt, same drivlinje til 468 900 kr. Hvilket utstyrsnivå (Plus/Ultra) P5 Long Range faktisk selges med er ikke uavhengig bekreftet - forblir bevisst ukjent for denne konfigurasjonen fremfor antatt identisk med P8 AWD. [Kriterium W009]</t>
+          <t>elbil.no og Frydenbøs trimnivå-sammenligning bekrefter at 360-graders kamera er forbeholdt Ultra-utstyrsnivå, ikke inkludert på Plus. Hvilket utstyrsnivå P5 Long Range selges med er nå uavhengig bekreftet: Frydenbøs egen kampanjeside viser Single Motor Extended Range (476 km, matcher denne konfigurasjonens WLTP) selges som Plus - samme nivå den tidligere P8 AWD-baserte sammenligningen gjaldt. 360-kamera fortsatt ikke inkludert på denne konfigurasjonen. [Kriterium W009]</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>EV_000073</t>
+          <t>EV_000073,EV_000150</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -38775,7 +39290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H150"/>
+  <dimension ref="A1:H152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -42843,6 +43358,60 @@
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>EV_000150</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Frydenbøs egen EX30-kampanjeside bekrefter at Single Motor Extended Range (476 km rekkevidde - matcher denne konfigurasjonens registrerte WLTP-tall) selges som Plus-utstyrsnivå i det norske markedet (468 900 kr veiledende), ikke Core eller Ultra. Løser for første gang hvilket utstyrsnivå denne konfigurasjonen faktisk tilsvarer.</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>SRC_FRYDENBO_EX30_CAMPAIGN_PRICING</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>EV_000151</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>VOLVO_EX30_P5_LONG_RANGE</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Frydenbøs utstyrsnivå-veiledning bekrefter at Adaptiv Cruise Kontroll og ryggekamera er standard fra og med Core-nivå (laveste nivå) på EX30 - dermed inkludert på Plus (se EV_000150 for bekreftelse av at denne konfigurasjonen er Plus-nivå). 360-graders kamera forblir forbeholdt Ultra, ikke inkludert her.</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>SRC_FRYDENBO_EX30_UTSTYRSNIVA_GUIDE</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Update onboarding_helpers.py to include new flagship configuration and adjust documentation
The onboarding_helpers.py script has been modified to add "SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION" to the list of flagship configurations, increasing the total from 6 to 7. The accompanying documentation has been updated to reflect this change, ensuring clarity in the configuration treatment process.
</commit_message>
<xml_diff>
--- a/data/EV_Decision_Framework.xlsx
+++ b/data/EV_Decision_Framework.xlsx
@@ -419,6 +419,25 @@
             </numRef>
           </val>
         </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'15_Dashboard'!$A$35</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <val>
+            <numRef>
+              <f>'15_Dashboard'!$B$35:$I$35</f>
+            </numRef>
+          </val>
+        </ser>
         <gapWidth val="150"/>
         <overlap val="-10"/>
         <axId val="10"/>
@@ -1192,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5517,6 +5536,300 @@
         </is>
       </c>
       <c r="I101" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Nye Skoda Epiq - Sulland</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Sulland (Skoda-forhandler, Norge)</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>https://www.sulland.no/nybil/skoda/epiq</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Norsk forhandlerside. Bekrefter dimensjoner (4170x1800x1580mm), bagasjerom (475L), maks tilhengervekt (1200kg), batteri netto (52 kWt), motoreffekt (211 hk), WLTP-rekkevidde (435 km Selection / 440 km Essence), forbruk (13,7 kWt/100km), DC-lading (10-80% på 24 min), pris for begge Launch Edition-variantene.</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>SRC_AUTORIA_SKODA_EPIQ_PRIS</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Skoda Epiq - Pris - Kampanje - Leasing</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Autoria.no</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>https://www.autoria.no/kampanjer/epiq-pris</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Norsk utstyrsliste for Epiq 55 Launch Edition: bekrefter adaptiv cruise kontroll, ryggekamera, parkeringssensorer foran og bak, og Lane Assist som standardutstyr. Apple CarPlay ikke nevnt på denne listen til tross for at internasjonale kilder oppgir det som standard - se W007-Reviewen for drøfting.</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>SRC_AUTODATA_SKODA_EPIQ55</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Skoda Epiq 55 55 kWh (211 Hp) Electric - technical specs</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Auto-data.net</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>https://www.auto-data.net/en/skoda-epiq-55-55-kwh-211hp-electric-56719</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Oppgir egenvekt (1469 kg), toppfart (160 km/t), dreiemoment (290 Nm), 0-100 km/t (7,4 sek).</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>SRC_ARENAEV_SKODA_EPIQ_CHARGING</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Skoda details the Epiq's power, batteries, range, and performance</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>ArenaEV</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>https://www.arenaev.com/skoda_details_the_epiqs_power_batteries_range_and_performance-news-5585.php</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Oppgir 11 kW AC / 133 kW DC-lading for Epiq 55. Andre kilder oppgir avvikende DC-tall (105-125 kW) - reell kildeuenighet, sannsynligvis fordi spesifikasjonene ikke er fullt stabilisert for denne ennå ikke lanserte modellen. Laveste konfidens gitt spredningen i tallene.</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_STORYBOARD_EPIQ_PRESSKIT</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Skoda Epiq press kit - the new all-electric entry model</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Skoda Auto (Storyboard)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>https://www.skoda-storyboard.com/en/press-kits/skoda-epiq-press-kit/skoda-epiq-the-new-all-electric-entry-model-combining-accessibilitycompact-dimensions-and-everyday-practicality/</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Internasjonalt pressemateriale. Bekrefter frunk-volum (25 liter) og luftmotstandstall (Cw 0,275). Ikke markedsspesifikt, men fysiske mål antas like på tvers av markeder.</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_SKODA_EPIQ_REVIEW</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Skoda Epiq review</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>What Car?</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>https://www.whatcar.com/skoda/epiq/estate/review/n29034</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Forhåndsvurdering basert på prototypkjøring - ikke ferdig produksjonsbil, ikke spesifisert utstyrsnivå. Dekker kjørekomfort, synlighet, styring, kupéstøy, seteplass, materialkvalitet og betjening.</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>SRC_ELECTRIFYING_SKODA_EPIQ_REVIEW</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL_REVIEW</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Skoda Epiq Review &amp; Buying Guide</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Electrifying.com</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>https://www.electrifying.com/long-term-reviews/skoda-reviews/epiq/review</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Forhåndsvurdering basert på ca. 1 times prototypkjøring i Porto (anmelder Vicky Parrott) - ikke ferdig produksjonsbil. Dekker kjørekomfort, styring, materialkvalitet, infotainment og seteplass.</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
@@ -5542,7 +5855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -10397,6 +10710,686 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>SCORE_000122</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>W001</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>REV_000121</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F122">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D122,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G122">
+        <f>ROUND(F122*INDEX('01_Criteria'!$F:$F,MATCH(C122,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale). Traceable to REV_000121 -&gt; supporting Evidence EV_000152 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>SCORE_000123</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>W002</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>REV_000122</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F123">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D123,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G123">
+        <f>ROUND(F123*INDEX('01_Criteria'!$F:$F,MATCH(C123,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale). Traceable to REV_000122 -&gt; supporting Evidence EV_000153 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>SCORE_000124</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>W003</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>REV_000123</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F124">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D124,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G124">
+        <f>ROUND(F124*INDEX('01_Criteria'!$F:$F,MATCH(C124,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale). Traceable to REV_000123 -&gt; supporting Evidence EV_000154 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>SCORE_000125</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>W004</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>REV_000124</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F125">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D125,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G125">
+        <f>ROUND(F125*INDEX('01_Criteria'!$F:$F,MATCH(C125,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale). Traceable to REV_000124 -&gt; supporting Evidence EV_000155 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>SCORE_000126</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>W005</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>REV_000125</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F126">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D126,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G126">
+        <f>ROUND(F126*INDEX('01_Criteria'!$F:$F,MATCH(C126,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale). Traceable to REV_000125 -&gt; supporting Evidence EV_000156 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>SCORE_000127</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>W007</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>REV_000126</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F127">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D127,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G127">
+        <f>ROUND(F127*INDEX('01_Criteria'!$F:$F,MATCH(C127,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale). Traceable to REV_000126 -&gt; supporting Evidence EV_000157 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>SCORE_000128</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>W009</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>REV_000127</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F128">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D128,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G128">
+        <f>ROUND(F128*INDEX('01_Criteria'!$F:$F,MATCH(C128,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale). Traceable to REV_000127 -&gt; supporting Evidence EV_000158 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>SCORE_000129</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>W010</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>REV_000128</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F129">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D129,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G129">
+        <f>ROUND(F129*INDEX('01_Criteria'!$F:$F,MATCH(C129,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale). Traceable to REV_000128 -&gt; supporting Evidence EV_000159 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>SCORE_000130</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>W012</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>REV_000129</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F130">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D130,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G130">
+        <f>ROUND(F130*INDEX('01_Criteria'!$F:$F,MATCH(C130,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale). Traceable to REV_000129 -&gt; supporting Evidence EV_000160 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>SCORE_000131</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>W013</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>REV_000130</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F131">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D131,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G131">
+        <f>ROUND(F131*INDEX('01_Criteria'!$F:$F,MATCH(C131,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale). Traceable to REV_000130 -&gt; supporting Evidence EV_000161 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>SCORE_000132</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>W014</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>REV_000131</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F132">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D132,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G132">
+        <f>ROUND(F132*INDEX('01_Criteria'!$F:$F,MATCH(C132,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale). Traceable to REV_000131 -&gt; supporting Evidence EV_000162 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>SCORE_000133</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>W015</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>REV_000132</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F133">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D133,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G133">
+        <f>ROUND(F133*INDEX('01_Criteria'!$F:$F,MATCH(C133,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale). Traceable to REV_000132 -&gt; supporting Evidence EV_000163 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>SCORE_000134</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>W016</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>REV_000133</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F134">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D134,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G134">
+        <f>ROUND(F134*INDEX('01_Criteria'!$F:$F,MATCH(C134,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale). Traceable to REV_000133 -&gt; supporting Evidence EV_000164 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>SCORE_000135</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>W017</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>REV_000134</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F135">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D135,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G135">
+        <f>ROUND(F135*INDEX('01_Criteria'!$F:$F,MATCH(C135,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale). Traceable to REV_000134 -&gt; supporting Evidence EV_000165 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>SCORE_000136</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>W018</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>REV_000135</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F136">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D136,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G136">
+        <f>ROUND(F136*INDEX('01_Criteria'!$F:$F,MATCH(C136,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale). Traceable to REV_000135 -&gt; supporting Evidence EV_000166 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>SCORE_000137</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>W019</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>REV_000136</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F137">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D137,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G137">
+        <f>ROUND(F137*INDEX('01_Criteria'!$F:$F,MATCH(C137,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Review score 4/5 (normalized RawScore = 80.0/100 on a documented 1-5 scale). Traceable to REV_000136 -&gt; supporting Evidence EV_000167 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>SCORE_000138</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>W020</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>REV_000137</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F138">
+        <f>ROUND(INDEX('07_Reviews'!$E:$E,MATCH(D138,'07_Reviews'!$A:$A,0))/5*100,2)</f>
+        <v/>
+      </c>
+      <c r="G138">
+        <f>ROUND(F138*INDEX('01_Criteria'!$F:$F,MATCH(C138,'01_Criteria'!$A:$A,0))/100,2)</f>
+        <v/>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Review score 3/5 (normalized RawScore = 60.0/100 on a documented 1-5 scale). Traceable to REV_000137 -&gt; supporting Evidence EV_000168 -&gt; cited Source.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10409,7 +11402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11829,6 +12822,48 @@
         </is>
       </c>
       <c r="H34" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>DEC_DATA_012</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Added seventh Vehicle (Skoda Epiq) - Selection 55 Launch Edition scored end-to-end, Essence 55 Launch Edition as sibling</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>User requested a car to challenge Skoda Elroq (2nd place) and chose Epiq, a brand-new pre-release Skoda model launching Q4 2026 in Norway, explicitly anticipating fewer real-world tests than the other six vehicles (same caveat as Kia EV2 at onboarding time).</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Confirmed naming directly with a Norwegian dealer (Sulland): "Epiq Selection 55 Launch Edition" (359 900 kr) is a real, currently-orderable Norwegian SKU, distinct from the separate, more expensive "First Edition" special edition found during research - avoided conflating the two. Skoda has no skoda.no manufacturer site; sourced instead from Sulland and Autoria.no (Norwegian dealers/resellers), auto-data.net, ArenaEV, Skoda's international press kit, and two prototype-drive previews (What Car?, Electrifying.com) - both explicitly not full production-car road tests. All 5 Hard Requirements resolved for both Configurations (M001/M002/M004/M005 PASS for Selection at MEDIUM-HIGH confidence; M004/M005 left UNKNOWN for Essence since no direct Norwegian source confirms its equipment beyond interior/wheel packages). M003 (winter range) resolved via the ADR-014 WLTP x 0.70 estimate for both configs (Selection: 304.5km, a 4.5km margin - very tight; Essence: 308km). Scored 17 of 20 weighted Criteria for the flagship (Selection) - W006 (OTA/future-proofing), W008 (real-world ADAS quality beyond confirmed presence), and W011 (long-term build quality/rattles) deliberately left unscored, no genuine evidence existed for any of the three from a ~1-hour prototype preview drive. Resulting CoveragePercent is 86% (vs 100% for all six existing flagships) - the lowest in the comparison, honestly reflecting the pre-release data gap rather than forcing full coverage. OverallScore: 59.2 - 7th of 7, below every existing vehicle including Elroq, not the stronger competitor the user was hoping to add. W014/W016 (manufacturer risk / Nordic maturity) scored more conservatively than Elroq's equivalent criteria specifically because Epiq sits on MEB+, a brand-new platform shared only with the also-unreleased VW ID.2 - unlike Elroq's mature, multi-year MEB inheritance. W015 (warranty) reused Skoda/Moller's existing brand-wide warranty policy already documented for Elroq, at the same HIGH confidence. 15_Dashboard (Decision Summary row 12, Category Breakdown row 35 + chart series, Coverage Grid row 59) and scripts/onboarding_helpers.py FLAGSHIP_CONFIGURATION_IDS updated to include the new flagship.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
@@ -11851,7 +12886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12125,6 +13160,39 @@
       </c>
       <c r="H7">
         <f>IF(E7&lt;100,"Partial evaluation - "&amp;F7&amp;" of "&amp;G7&amp;" WEIGHTED+Active criteria scored ("&amp;E7&amp;"% of total weight).","Complete evaluation - all WEIGHTED+Active criteria scored.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OVSC_000007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="D8">
+        <f>SUMIFS('10_Scoring'!$G$2:$G$1000,'10_Scoring'!$B$2:$B$1000,B8,'10_Scoring'!$E$2:$E$1000,C8)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>ROUND(SUMPRODUCT(('10_Scoring'!$B$2:$B$1000=B8)*('10_Scoring'!$E$2:$E$1000=C8)*IFERROR(INDEX('01_Criteria'!$F$2:$F$1000,MATCH('10_Scoring'!$C$2:$C$1000,'01_Criteria'!$A$2:$A$1000,0)),0))/SUMIFS('01_Criteria'!$F$2:$F$1000,'01_Criteria'!$E$2:$E$1000,"WEIGHTED",'01_Criteria'!$H$2:$H$1000,"TRUE")*100,2)</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>COUNTIFS('10_Scoring'!$B$2:$B$1000,B8,'10_Scoring'!$E$2:$E$1000,C8)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>COUNTIFS('01_Criteria'!$E$2:$E$1000,"WEIGHTED",'01_Criteria'!$H$2:$H$1000,"TRUE")</f>
         <v/>
       </c>
     </row>
@@ -12554,7 +13622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16551,6 +17619,386 @@
       <c r="H101" t="inlineStr">
         <is>
           <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>HRR_000101</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Skoda Epiq er en helelektrisk modell (BEV); ingen forbrenningsmotor- eller hybridvariant eksisterer.</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>HRR_000102</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4170mm (Sulland) er godt innenfor 4500mm-grensen, med 330mm margin.</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>HRR_000103</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Ingen uavhengig vintertest eksisterer for denne ennå ikke leverte modellen. Estimert vintervegkjørelengde = 70% av WLTP (ADR-014): 435 km x 0.70 = 304.5 km, bestått med kun 4.5 km margin - svært tett, i praksis på grensen.</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>HRR_000104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Adaptiv cruise kontroll bekreftet standard i norsk utstyrsliste (Autoria.no) for Epiq 55 Launch Edition.</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>SRC_AUTORIA_SKODA_EPIQ_PRIS</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>HRR_000105</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Ryggekamera bekreftet standard i norsk utstyrsliste (Autoria.no) for Epiq 55 Launch Edition.</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>SRC_AUTORIA_SKODA_EPIQ_PRIS</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>HRR_000106</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_ESSENCE_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Skoda Epiq er en helelektrisk modell (BEV); ingen forbrenningsmotor- eller hybridvariant eksisterer.</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>HRR_000107</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_ESSENCE_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4170mm (Sulland, delt mellom alle Epiq-varianter) er godt innenfor 4500mm-grensen, med 330mm margin.</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>HRR_000108</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_ESSENCE_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Ingen uavhengig vintertest eksisterer for denne ennå ikke leverte modellen. Estimert vintervegkjørelengde = 70% av WLTP (ADR-014): 440 km x 0.70 = 308.0 km, bestått med 8 km margin.</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>HRR_000109</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_ESSENCE_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Ikke bekreftet for denne spesifikke (grunnivå) konfigurasjonen - Sullands egen prisliste nevner kun interior- og felgpakke for Essence, ingen fullstendig utstyrsliste ble funnet ved direkte henting. Internasjonale kilder hevder adaptiv cruise kontroll er standard selv på laveste nivå, men dette er ikke bekreftet mot en norsk kilde direkte - forblir bevisst ukjent fremfor antatt.</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>HRR_000110</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_ESSENCE_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Ikke bekreftet for denne konfigurasjonen. Enkelte kilder antyder ryggekamera er en Selection-nivå-tilføyelse, ikke inkludert på Essence, men dette er heller ikke uavhengig bekreftet mot en norsk kilde direkte - forblir bevisst ukjent fremfor antatt.</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -17075,7 +18523,11 @@
         <v/>
       </c>
       <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
       <c r="I12" s="6">
         <f>IFERROR(INDEX('02_Vehicles'!$B$2:$B$1000,MATCH(INDEX('03_Configurations'!$B$2:$B$1000,MATCH($H12,'03_Configurations'!$A$2:$A$1000,0)),'02_Vehicles'!$A$2:$A$1000,0)),"")</f>
         <v/>
@@ -18187,7 +19639,11 @@
         <f>IF($J35="","",IFERROR(SUMPRODUCT(('10_Scoring'!$B$2:$B$1000=$J35)*('10_Scoring'!$E$2:$E$1000=INDEX('12_OverallScores'!$C$2:$C$1000,MATCH($J35,'12_OverallScores'!$B$2:$B$1000,0)))*(IFERROR(INDEX('01_Criteria'!$B$2:$B$1000,MATCH('10_Scoring'!$C$2:$C$1000,'01_Criteria'!$A$2:$A$1000,0)),"")=I$28)*'10_Scoring'!$G$2:$G$1000),0))</f>
         <v/>
       </c>
-      <c r="J35" s="6" t="n"/>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6">
@@ -18987,7 +20443,11 @@
         <v/>
       </c>
       <c r="G59" s="6" t="n"/>
-      <c r="H59" s="6" t="n"/>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
       <c r="I59" s="6">
         <f>IFERROR(INDEX('03_Configurations'!$B$2:$B$1000,MATCH($H59,'03_Configurations'!$A$2:$A$1000,0)),"")</f>
         <v/>
@@ -22475,7 +23935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -22743,6 +24203,41 @@
       <c r="G7" t="inlineStr">
         <is>
           <t>BYD Norge offisiell modellside sett 2026-07-07: https://byd.no/modeller/atto3. To utstyrsnivåer (Comfort, Design), ett batteri/drivverk (60 kWh, forhjulsdrift). Modellår og plattform ikke spesifisert i kildegrunnlaget. Skilt fra det separat markedsførte BYD EVO 4x4 (byd.no/modeller/evo-4x4), som ikke er del av denne sammenligningen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Škoda</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Epiq</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MEB+</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>UPCOMING</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Ny modell, ikke levert i Norge ennå - bestilling åpnet hos norske forhandlere (Sulland m.fl.), første kundebiler ventet 4. kvartal 2026. Ingen uavhengig norsk vintertest eller full produksjonsbil-anmeldelse eksisterer ennå - se 07_Reviews for kildegrunnlag (forhandlersider + internasjonale prototyp-forhåndsvurderinger).</t>
         </is>
       </c>
     </row>
@@ -22763,7 +24258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -23662,6 +25157,92 @@
       <c r="I21" t="inlineStr">
         <is>
           <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Selection 55 Launch Edition (FWD, 52 kWh)</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>359900</v>
+      </c>
+      <c r="G22" t="n">
+        <v>359900</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Sulland (norsk Skoda-forhandler) og Autoria.no bekrefter Epiq Selection 55 Launch Edition til 359 900 kr, bestillbar nå, levering ventet 4. kvartal 2026. Flaggskip-konfigurasjon for denne kjøretøymodellen (ADR-013) - eneste konfigurasjon med full Evidence/Review/Score-behandling. Se 11_DecisionLog DEC_DATA_012.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_ESSENCE_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Essence 55 Launch Edition (FWD, 52 kWh)</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>339900</v>
+      </c>
+      <c r="G23" t="n">
+        <v>339900</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Sulland bekrefter Epiq Essence 55 Launch Edition til 339 900 kr. Søsterkonfigurasjon - kun Technical/Equipment/HardRequirementResults, ikke tatt gjennom full scoring (ADR-013 flaggskip-omfang). Se 11_DecisionLog DEC_DATA_012.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -23688,7 +25269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K169"/>
+  <dimension ref="A1:K187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -31422,6 +33003,826 @@
       <c r="J169" t="inlineStr">
         <is>
           <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>TECH_000169</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>TF_LENGTH</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>4170</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>TECH_000170</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>TF_WIDTH</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>TECH_000171</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>TF_HEIGHT</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>1580</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>TECH_000172</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>TF_BOOT_VOLUME</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>475</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>TECH_000173</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>TF_FRUNK_VOLUME</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>25</v>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>SRC_SKODA_STORYBOARD_EPIQ_PRESSKIT</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>TECH_000174</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>TF_MAX_TRAILER_WEIGHT</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>TECH_000175</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>TF_BATTERY_NET</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>52</v>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>KWH</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>TECH_000176</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>TF_MOTOR_POWER</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>155</v>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>TECH_000177</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>TF_TORQUE</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>290</v>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>SRC_AUTODATA_SKODA_EPIQ55</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>TECH_000178</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>TF_TOP_SPEED</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>160</v>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>KMH</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>SRC_AUTODATA_SKODA_EPIQ55</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>TECH_000179</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>TF_KERB_WEIGHT</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>1469</v>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>SRC_AUTODATA_SKODA_EPIQ55</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>TECH_000180</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>TF_AC_MAX_CHARGING</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>11</v>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>SRC_ARENAEV_SKODA_EPIQ_CHARGING</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>TECH_000181</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>TF_DC_MAX_CHARGING</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>133</v>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>SRC_ARENAEV_SKODA_EPIQ_CHARGING</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>TECH_000182</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>TF_WLTP_RANGE</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>435</v>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>TECH_000183</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>TF_WLTP_CONSUMPTION</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>KWH_100KM</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>TECH_000184</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_ESSENCE_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>TF_WLTP_RANGE</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>440</v>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>TECH_000185</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>TF_WINTER_HIGHWAY_RANGE_ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>304.5</v>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>Estimated (70% of WLTP, ADR-014)</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>TECH_000186</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_ESSENCE_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>TF_WINTER_HIGHWAY_RANGE_ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>308</v>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>Estimated (70% of WLTP, ADR-014)</t>
         </is>
       </c>
     </row>
@@ -31445,7 +33846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -33787,6 +36188,102 @@
         </is>
       </c>
       <c r="F73" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>EQ_000073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>EQ_ACC</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>SRC_AUTORIA_SKODA_EPIQ_PRIS</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>EQ_000074</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>EQ_REAR_CAMERA</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>SRC_AUTORIA_SKODA_EPIQ_PRIS</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>EQ_000075</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>EQ_LANE_CENTER</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>SRC_AUTORIA_SKODA_EPIQ_PRIS</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -34412,7 +36909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I121"/>
+  <dimension ref="A1:I138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -39270,6 +41767,686 @@
       <c r="I121" t="inlineStr">
         <is>
           <t>1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>REV_000121</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>3</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>To uavhengige prototyp-forhåndsvurderinger er uenige om kupéstøy ved motorveifart: What Car? beskriver bilen som stillegående med lite veistøy, mens Electrifying.com bemerker merkbar fjærings- og dekkstøy til tross for et generelt rolig og forfinet inntrykk. Ingen av testene gjelder ferdig produksjonsbil eller norsk vinterkjøring. [Kriterium W001]</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>EV_000152</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>REV_000122</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>4</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>To uavhengige prototyp-forhåndsvurderinger er samstemte om god komfort: godt balansert fjæring som takler både lavfartshumper og ujevnt veidekke, samt god seteplass i begge rader. Basert på prototypkjøring, ikke ferdig produksjonsbil eller norsk-spesifikk testing. [Kriterium W002]</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>EV_000153</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>REV_000123</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>4</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Begge prototyp-forhåndsvurderinger fremhever god sikt (kort motorpanser, slanke A-stolper, stort bakvindu) og grei manøvrering i trange rom. Basert på prototypkjøring, ikke ferdig produksjonsbil. [Kriterium W003]</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>EV_000154</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>REV_000124</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Kjøreopplevelse</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>3</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Styringen beskrives som lett og bytilpasset av begge kilder, forutsigbar i normal kjøring - men What Car? presiserer selv at egenskaper på svingete veier forblir utestet. Score reflekterer en trygg, men ikke presisjonsorientert, kjørefølelse. Basert på prototypkjøring, ikke ferdig produksjonsbil. [Kriterium W004]</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>EV_000155</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>REV_000125</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>4</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>God kombinasjon av responsiv skjerm og fysiske snarveisknapper for klimaanlegg per prototyp-vurdering; navigasjonssystem bekreftet som standardutstyr i det norske markedet spesifikt. [Kriterium W005]</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>EV_000156</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>REV_000126</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>4</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Apple CarPlay bekreftet standard av en internasjonal kilde; fraværet fra den norske utstyrslisten er notert som en sannsynlig listeufullstendighet, ikke bekreftet fravær - lavere konfidens gitt denne kildeuenigheten. [Kriterium W007]</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>EV_000157</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>REV_000127</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>3</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Ryggekamera og parkeringssensorer foran/bak bekreftet standard i det norske markedet - god grunnutrustning, men uten 360-graders kamera slik enkelte konkurrenter tilbyr. [Kriterium W009]</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>EV_000158</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>REV_000128</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Opplevd kvalitet</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>3</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Overveiende positivt inntrykk av materialkvalitet for prisklassen (myke overflater øverst, hardere plast lavt nede), men usikkerhet rundt hvilken internasjonal materialpakke som faktisk tilsvarer den norske Selection-konfigurasjonen reduserer konfidensen. [Kriterium W010]</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>EV_000159</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>REV_000129</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Opplevd kvalitet</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>3</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>God justerbarhet for ratt og sete, samt fysiske betjeningselementer for hyppig brukte funksjoner - positivt førermiljø-inntrykk basert på prototypkjøring, ikke ferdig produksjonsbil. [Kriterium W012]</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>EV_000160</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>REV_000130</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Opplevd kvalitet</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>4</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Fysiske snarveisknapper for klimaanlegg fremhevet som en gjennomtenkt løsning som unngår unødig menynavigering - god betjeningskvalitet-vurdering fra prototyp-forhåndsvurdering. [Kriterium W013]</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>EV_000161</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>REV_000131</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>3</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Skoda/VW-konsernets merkevareomdømme er solid, men i motsetning til Elroq (som kunne støtte seg på den modne, flerårige MEB-plattformen) er MEB+ en helt ny plattform uten reell driftshistorikk - lavere konfidens enn Elroqs tilsvarende vurdering, per prinsippet om at manglende egen historikk gir lavere konfidens, ikke automatisk lavere score. [Kriterium W014]</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>EV_000162</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>REV_000132</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>4</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Samme solide, merkevaredekkende garanti- og serviceapparat som allerede dokumentert for Elroq - denne policyen er modelluavhengig, så høy konfidens til tross for at Epiq selv er helt ny. [Kriterium W015]</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>EV_000163</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>REV_000133</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Langtidseierskap</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>3</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Skodas generelle nordiske merkevareomdømme er godt, men MEB+-plattformen mangler den flerårige vintertest-historikken som støttet Elroqs tilsvarende vurdering - reflektert i lavere konfidens enn Elroqs W016-score. [Kriterium W016]</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>EV_000164</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>REV_000134</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Økonomi</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>3</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Solid utstyrsnivå til en pris under Elroq for en sammenlignbar (mindre) SUV - reell verdi i utstyr og pris, men score modereres av at dette er en ennå ikke levert modell uten sammenlignbar driftshistorikk. [Kriterium W017]</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>EV_000165</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>REV_000135</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Praktisk bruk</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>4</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Romslig bagasjerom for segmentet pluss frunk gir god fleksibilitet for voksne passasjerer og last - positivt for en husholdning uten barn hvor voksen-/lastfleksibilitet veier tyngre enn ISOFIX-hensyn. [Kriterium W018]</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>EV_000166</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>REV_000136</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Garasje</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>4</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Deterministisk beregnet fra offisiell lengdemargin (330mm), samme rubrikk som øvrige kjøretøy i sammenligningen. [Kriterium W019]</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>EV_000167</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>REV_000137</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Rekkevidde/lading</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>3</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Ladeegenskaper virker konkurransedyktige (133 kW DC oppgitt), men reell usikkerhet i det eksakte DC-tallet på tvers av kilder gir lavere konfidens enn ellers ved 8000 km/år-bruksmønsteret dette kriteriet vektlegges mot. [Kriterium W020]</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>EV_000168</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>1.9</t>
         </is>
       </c>
     </row>
@@ -39290,7 +42467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H152"/>
+  <dimension ref="A1:H169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -43412,6 +46589,450 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>EV_000152</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>What Car? (prototypkjøring) beskriver bilen som "hushed, with very little road noise" ved motorveifart. Electrifying.com (separat prototypkjøring i Porto) bemerker derimot at man "notice suspension and tyre noise", selv om helhetsinntrykket beskrives som "a refined and calm car". Reell kildeuenighet mellom to uavhengige forhåndsvurderinger av samme ikke-produksjonsklare prototyp.</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_SKODA_EPIQ_REVIEW,SRC_ELECTRIFYING_SKODA_EPIQ_REVIEW</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>EV_000153</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>What Car?: "suspension strikes a good balance between control and suppleness", håndterer lavfartshumper bedre enn konkurrenter, "body control in check over undulating roads" ved høyere fart. Electrifying.com: bilen "rides well even over very rough surfaces" på Portos dårlige veier. Begge kilder bekrefter god seteplass foran og bak.</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_SKODA_EPIQ_REVIEW,SRC_ELECTRIFYING_SKODA_EPIQ_REVIEW</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>EV_000154</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>What Car?: "short bonnet and slim windscreen pillars provide clear forward views", og "large back window means that you can see plenty behind you". Electrifying.com bekrefter "decent turning circle for those moments when you want to squeeze into a tight space".</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_SKODA_EPIQ_REVIEW,SRC_ELECTRIFYING_SKODA_EPIQ_REVIEW</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>EV_000155</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>What Car?: "light steering suggests it's been tuned to make effortlessly threading through town a priority" - men presiserer eksplisitt at "handling characteristics on twisty roads remain untested". Electrifying.com: styringen er "reasonably hefty and direct, yet light enough", kjørefølelsen "very grown-up" med "predictable pedal responses".</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_SKODA_EPIQ_REVIEW,SRC_ELECTRIFYING_SKODA_EPIQ_REVIEW</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>EV_000156</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>What Car?: 5,3-tommers digitalt display og 13-tommers berøringsskjerm er "clear and easy to read" og "reacts to your prods quickly"; fysiske snarveisknapper under skjermen forenkler klimaanlegg-betjening og unngår unødig menynavigering. Autoria.no (norsk prisliste) bekrefter "Navigasjonssystem" som standardutstyr på Epiq 55 Launch Edition.</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_SKODA_EPIQ_REVIEW,SRC_AUTORIA_SKODA_EPIQ_PRIS</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>EV_000157</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Electrifying.com bekrefter eksplisitt: "Standard 13-inch touchscreen with Apple CarPlay and Android Auto". Autoria.nos norske utstyrsliste for Launch Edition nevner derimot ikke Apple CarPlay til tross for en ellers omfattende liste - sannsynligvis en ufullstendig markedsføringsliste snarere enn reell fraværende funksjon, gitt at trådløs CarPlay/Android Auto er standard på tvers av hele Skoda/VW MEB-plattformen.</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>SRC_ELECTRIFYING_SKODA_EPIQ_REVIEW,SRC_AUTORIA_SKODA_EPIQ_PRIS</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>EV_000158</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Autoria.no (norsk prisliste for Epiq 55 Launch Edition) bekrefter "Parkeringssensorer foran og bak" og "Ryggekamera" som standardutstyr. Ingen 360-graders kamera er nevnt eller bekreftet tilgjengelig for denne konfigurasjonen.</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>SRC_AUTORIA_SKODA_EPIQ_PRIS</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>EV_000159</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>What Car?: kabinen har "soft touch materials all over the dashboard" med "scratchy plastics kept quite low down", vurdert som "impressive" for prisklassen. Electrifying.com beskriver ulike fargevalg/materialpakker (Loft med "part leatherette", Suite med "faux suede and leatherette") - navngivning som ikke er direkte bekreftet å tilsvare de norske Essence/Selection-nivåene.</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_SKODA_EPIQ_REVIEW,SRC_ELECTRIFYING_SKODA_EPIQ_REVIEW</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>EV_000160</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>What Car? bekrefter "plenty of steering wheel and seat adjustment" for å finne en komfortabel kjørestilling, kombinert med fysiske snarveisknapper som reduserer skjermavhengighet for hyppig brukte funksjoner.</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_SKODA_EPIQ_REVIEW</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>EV_000161</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>What Car? fremhever spesifikt at "physical shortcut buttons beneath the screen simplify climate control access, avoiding excessive menu diving" - en direkte kommentar til betjeningsdesign, ikke bare skjermkvalitet.</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>SRC_WHATCAR_SKODA_EPIQ_REVIEW</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>EV_000162</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Epiq bygges på MEB+, en ny plattform utviklet spesielt for kompakte elbiler, delt kun med den også ennå ikke lanserte VW ID.2. I motsetning til Elroqs MEB-plattform (delt med Enyaq/ID.3/ID.4/ID.5/Q4 e-tron, med flere års reell driftserfaring på tvers av merker - se W014-vurderingen for SKODA_ELROQ_SELECTION_60), har MEB+ ingen reell driftshistorikk å falle tilbake på ennå.</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>EV_000163</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Skoda-Norge (importert av Harald A. Møller AS) tilbyr samme garantivilkår på alle nye elbiler uavhengig av modell: 5 års/100 000 km generell nybilgaranti samt 8 års/160 000 km batterigaranti (minst 70% kapasitet) - samme merkevaredekkende policy allerede dokumentert for Elroq Selection 60, og et langt etablert, landsdekkende forhandlernett via Møller-apparatet.</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>EV_000164</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>MEB+-plattformen har ingen dokumentert flerårig nordisk vintererfaring ennå, i motsetning til Elroqs MEB-plattform som NAF/Motor har testet siden januar 2022 med gjennomgående sterke resultater. Skoda generelt har solid nordisk tilstedeværelse og erfaring, men den spesifikke MEB+-plattformen er uprøvd i nordisk klima.</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>EV_000165</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Epiq Selection 55 Launch Edition koster 359 900 kr og inkluderer adaptiv cruisekontroll, navigasjon, ryggekamera, parkeringssensorer foran/bak, oppvarmede seter/ratt og 18" felg som standard - 15 000 kr billigere enn Elroq Selection 60 (374 900 kr) for et mindre, men nyere og bedre grunnutstyrt kjøretøy. Prisen alene reflekterer ikke den ekstra usikkerheten som følger med en helt ny, ennå ikke levert modell.</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>EV_000166</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Sulland bekrefter 475 liter bagasjerom (ekspanderbart til 1345 liter med nedfelte seter) - stort for segmentet - samt en 25-liters frunk for ekstra oppbevaring (Skodas pressemateriale). Dimensjoner (4170x1800x1580mm) gir god kabinplass til tross for kompakte utvendige mål.</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ,SRC_SKODA_STORYBOARD_EPIQ_PRESSKIT</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>EV_000167</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Offisiell lengde 4170mm (Sulland) gir 330mm margin til 4500mm-grensen. Etter samme rubrikk som brukt for øvrige kjøretøy (&gt;=400mm=5, 250-399mm=4, 100-249mm=3, 1-99mm=2, over grensen=1): 330mm faller i 250-399mm-intervallet.</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>SRC_SULLAND_SKODA_EPIQ</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>EV_000168</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>SKODA_EPIQ_SELECTION_55_LAUNCH_EDITION</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>ArenaEV oppgir 11 kW AC og 133 kW DC-lading (10-80% på 24 minutter, per Sulland) for Epiq 55. Andre kilder oppgir avvikende DC-tall (105-125 kW) for samme variant - reell kildeuenighet, sannsynligvis fordi spesifikasjonene ikke er fullt stabilisert for denne ennå ikke leverte modellen.</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>SRC_ARENAEV_SKODA_EPIQ_CHARGING</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">

</xml_diff>